<commit_message>
Fix LowerLimit and InitialStorate, fix pMaxProd, adjust Hydro input file
Add todos for weighing cost in the objective function
</commit_message>
<xml_diff>
--- a/data/hydroExample/Power_HydroAssets.xlsx
+++ b/data/hydroExample/Power_HydroAssets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\hydroExample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3DD01D6-CD84-4DB3-BD96-20C2E74DAE2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B04642-23D8-4BAF-88E4-B5C363C48B89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34230" yWindow="-21705" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="136">
   <si>
     <t>Format:</t>
   </si>
@@ -150,12 +150,6 @@
     <t>ExisUnits</t>
   </si>
   <si>
-    <t>MaxProd</t>
-  </si>
-  <si>
-    <t>MinProd</t>
-  </si>
-  <si>
     <t>Qmax</t>
   </si>
   <si>
@@ -261,15 +255,6 @@
     <t>Number of existing units</t>
   </si>
   <si>
-    <t>Maximum active power output of the unit</t>
-  </si>
-  <si>
-    <t>Minimum active power output of the unit</t>
-  </si>
-  <si>
-    <t>Maximum consumption of the unit</t>
-  </si>
-  <si>
     <t>Efficiency of discharging the storage unit</t>
   </si>
   <si>
@@ -393,9 +378,6 @@
     <t>PowerFactorPump</t>
   </si>
   <si>
-    <t>MaxPump</t>
-  </si>
-  <si>
     <t>Maximum Pumping</t>
   </si>
   <si>
@@ -541,6 +523,18 @@
   </si>
   <si>
     <t>190 Mellach und Kuehlwasserturbine-KW</t>
+  </si>
+  <si>
+    <t>MaxProdWater</t>
+  </si>
+  <si>
+    <t>Maximum water intake of the unit</t>
+  </si>
+  <si>
+    <t>Maximum water consumption of the unit</t>
+  </si>
+  <si>
+    <t>MaxPumpWater</t>
   </si>
 </sst>
 </file>
@@ -556,7 +550,7 @@
     <numFmt numFmtId="168" formatCode="0.00000"/>
     <numFmt numFmtId="169" formatCode="0.0000000000"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -616,6 +610,18 @@
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
       <name val="Aptos"/>
       <family val="2"/>
     </font>
@@ -689,7 +695,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -757,6 +763,10 @@
     </xf>
     <xf numFmtId="2" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1064,32 +1074,32 @@
   <sheetPr>
     <tabColor rgb="FF008080"/>
   </sheetPr>
-  <dimension ref="A1:AE43"/>
+  <dimension ref="A1:AD43"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" customWidth="1"/>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
     <col min="3" max="3" width="29.85546875" customWidth="1"/>
-    <col min="4" max="9" width="15.7109375" customWidth="1"/>
-    <col min="10" max="12" width="21.7109375" customWidth="1"/>
-    <col min="13" max="16" width="15.7109375" customWidth="1"/>
-    <col min="17" max="17" width="20.7109375" customWidth="1"/>
-    <col min="18" max="18" width="20.42578125" customWidth="1"/>
-    <col min="19" max="19" width="20.5703125" customWidth="1"/>
-    <col min="20" max="21" width="15.7109375" customWidth="1"/>
-    <col min="22" max="23" width="20.7109375" customWidth="1"/>
-    <col min="24" max="24" width="22.7109375" customWidth="1"/>
-    <col min="25" max="25" width="15.7109375" customWidth="1"/>
-    <col min="26" max="27" width="20.140625" customWidth="1"/>
-    <col min="28" max="28" width="20.42578125" customWidth="1"/>
-    <col min="29" max="29" width="19.42578125" customWidth="1"/>
-    <col min="30" max="31" width="24.5703125" customWidth="1"/>
+    <col min="4" max="8" width="15.7109375" customWidth="1"/>
+    <col min="9" max="11" width="21.7109375" customWidth="1"/>
+    <col min="12" max="15" width="15.7109375" customWidth="1"/>
+    <col min="16" max="16" width="20.7109375" customWidth="1"/>
+    <col min="17" max="17" width="20.42578125" customWidth="1"/>
+    <col min="18" max="18" width="20.5703125" customWidth="1"/>
+    <col min="19" max="20" width="15.7109375" customWidth="1"/>
+    <col min="21" max="22" width="20.7109375" customWidth="1"/>
+    <col min="23" max="23" width="22.7109375" customWidth="1"/>
+    <col min="24" max="24" width="15.7109375" customWidth="1"/>
+    <col min="25" max="26" width="20.140625" customWidth="1"/>
+    <col min="27" max="27" width="20.42578125" customWidth="1"/>
+    <col min="28" max="28" width="19.42578125" customWidth="1"/>
+    <col min="29" max="30" width="24.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:30" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1119,17 +1129,16 @@
       <c r="AB1" s="1"/>
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
-      <c r="AE1" s="1"/>
-    </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
@@ -1149,464 +1158,449 @@
         <v>6</v>
       </c>
       <c r="G3" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="L3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="M3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="K3" s="5" t="s">
+      <c r="N3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="R3" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="L3" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="P3" s="5" t="s">
+      <c r="S3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="T3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="R3" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="T3" s="5" t="s">
+      <c r="U3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="U3" s="5" t="s">
+      <c r="V3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="V3" s="5" t="s">
+      <c r="W3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="W3" s="5" t="s">
+      <c r="X3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="X3" s="5" t="s">
+      <c r="Y3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="Y3" s="5" t="s">
+      <c r="Z3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="Z3" s="5" t="s">
+      <c r="AA3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="AA3" s="5" t="s">
+      <c r="AB3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="AB3" s="5" t="s">
+      <c r="AC3" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="AC3" s="5" t="s">
+      <c r="AD3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="AD3" s="5" t="s">
+    </row>
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="AE3" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>30</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="28" t="s">
+        <v>132</v>
+      </c>
+      <c r="H4" s="28" t="s">
+        <v>135</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="L4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="M4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="J4" s="6" t="s">
+      <c r="N4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="O4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q4" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="K4" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="N4" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="P4" s="6" t="s">
+      <c r="R4" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="S4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="T4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="U4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="V4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="W4" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="X4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y4" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="Q4" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="R4" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="S4" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="T4" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="U4" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="V4" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="W4" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="X4" s="6" t="s">
+      <c r="Z4" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="Y4" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="Z4" s="6" t="s">
+      <c r="AA4" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="AA4" s="6" t="s">
+      <c r="AB4" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="AB4" s="6" t="s">
+      <c r="AC4" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="AC4" s="6" t="s">
+      <c r="AD4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="AD4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="AE4" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:31" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:30" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="E5" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="G5" s="29" t="s">
+        <v>133</v>
+      </c>
+      <c r="H5" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="I5" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="J5" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="K5" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="L5" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="M5" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="N5" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="O5" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="P5" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="L5" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="M5" s="7" t="s">
+      <c r="Q5" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="N5" s="7" t="s">
+      <c r="R5" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="S5" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="T5" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="U5" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="Q5" s="7" t="s">
+      <c r="V5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="R5" s="7" t="s">
+      <c r="W5" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="S5" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="T5" s="7" t="s">
+      <c r="X5" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="U5" s="7" t="s">
+      <c r="Y5" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="V5" s="7" t="s">
+      <c r="Z5" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="W5" s="7" t="s">
+      <c r="AA5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AB5" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="AC5" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="X5" s="7" t="s">
+      <c r="AD5" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="Y5" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z5" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="AA5" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="AB5" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="AC5" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="AD5" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="AE5" s="7" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="6" spans="1:31" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:30" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="K6" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="L6" s="8"/>
+        <v>62</v>
+      </c>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8" t="s">
+        <v>62</v>
+      </c>
       <c r="M6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="N6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="O6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="P6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="Q6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="R6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="S6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="T6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="U6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="V6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="W6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="X6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="Y6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="Z6" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="AA6" s="8" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="AB6" s="8" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="AC6" s="8" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="AD6" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="AE6" s="8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="9"/>
       <c r="B7" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="K7" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="L7" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="N7" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="O7" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="P7" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="K7" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="L7" s="26" t="s">
-        <v>95</v>
-      </c>
-      <c r="M7" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="N7" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="O7" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="P7" s="9" t="s">
-        <v>73</v>
-      </c>
       <c r="Q7" s="9" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="R7" s="9" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="S7" s="9" t="s">
-        <v>96</v>
+        <v>70</v>
       </c>
       <c r="T7" s="9" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="U7" s="9" t="s">
         <v>72</v>
       </c>
       <c r="V7" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="W7" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="X7" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y7" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="Z7" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA7" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="AB7" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="AC7" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="AD7" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="W7" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="X7" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="Y7" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="Z7" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="AA7" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="AB7" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="AC7" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="AD7" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="AE7" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="20"/>
       <c r="C8" s="18" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F8" s="12">
         <v>1</v>
@@ -1617,75 +1611,72 @@
       <c r="H8" s="13">
         <v>0</v>
       </c>
-      <c r="I8" s="13">
-        <v>0</v>
-      </c>
-      <c r="J8" s="24">
+      <c r="I8" s="24">
         <v>1.3833147724009441E-3</v>
       </c>
+      <c r="J8" s="14">
+        <v>0</v>
+      </c>
       <c r="K8" s="14">
-        <v>0</v>
-      </c>
-      <c r="L8" s="14">
         <v>5000</v>
       </c>
+      <c r="L8" s="13"/>
       <c r="M8" s="13"/>
-      <c r="N8" s="13"/>
+      <c r="N8" s="14">
+        <v>0</v>
+      </c>
       <c r="O8" s="14">
-        <v>0</v>
-      </c>
-      <c r="P8" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q8" s="12">
-        <v>0</v>
+      <c r="P8" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="14">
+        <v>8.9915460206061365E-2</v>
       </c>
       <c r="R8" s="14">
-        <v>8.9915460206061365E-2</v>
-      </c>
-      <c r="S8" s="14">
+        <v>0</v>
+      </c>
+      <c r="S8" s="12">
         <v>0</v>
       </c>
       <c r="T8" s="12">
         <v>0</v>
       </c>
-      <c r="U8" s="12">
-        <v>0</v>
+      <c r="U8" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V8" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W8" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X8" s="13">
-        <f>L8/G8</f>
+      <c r="W8" s="13">
+        <f>K8/G8</f>
         <v>9.7813715953307394</v>
       </c>
-      <c r="Y8" s="15"/>
-      <c r="Z8" s="12">
+      <c r="X8" s="15"/>
+      <c r="Y8" s="12">
         <v>1960</v>
       </c>
-      <c r="AA8" s="12"/>
+      <c r="Z8" s="12"/>
+      <c r="AA8" s="16">
+        <v>4676666671</v>
+      </c>
       <c r="AB8" s="16">
-        <v>4676666671</v>
-      </c>
-      <c r="AC8" s="16">
         <v>1555000001</v>
       </c>
+      <c r="AC8" s="17"/>
       <c r="AD8" s="17"/>
-      <c r="AE8" s="17"/>
-    </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B9" s="20"/>
       <c r="C9" s="19" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F9" s="12">
         <v>1</v>
@@ -1696,69 +1687,66 @@
       <c r="H9" s="13">
         <v>0</v>
       </c>
-      <c r="I9" s="13">
-        <v>0</v>
-      </c>
-      <c r="J9" s="25">
+      <c r="I9" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J9" s="14">
+        <v>0</v>
+      </c>
       <c r="K9" s="14">
-        <v>0</v>
-      </c>
-      <c r="L9" s="14">
         <v>5000</v>
       </c>
+      <c r="N9" s="14">
+        <v>0</v>
+      </c>
       <c r="O9" s="14">
-        <v>0</v>
-      </c>
-      <c r="P9" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q9" s="12">
-        <v>0</v>
-      </c>
-      <c r="R9" s="25">
+      <c r="P9" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S9" s="27">
+      <c r="R9" s="27">
+        <v>0</v>
+      </c>
+      <c r="S9" s="12">
         <v>0</v>
       </c>
       <c r="T9" s="12">
         <v>0</v>
       </c>
-      <c r="U9" s="12">
-        <v>0</v>
+      <c r="U9" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V9" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W9" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X9" s="13">
-        <f t="shared" ref="X9:X43" si="0">L9/G9</f>
+      <c r="W9" s="13">
+        <f>K9/G9</f>
         <v>3.7159090909090908</v>
       </c>
-      <c r="Z9">
-        <v>0</v>
+      <c r="Y9">
+        <v>0</v>
+      </c>
+      <c r="AA9">
+        <v>4704999901</v>
       </c>
       <c r="AB9">
-        <v>4704999901</v>
-      </c>
-      <c r="AC9">
         <v>1519400001</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B10" s="20"/>
       <c r="C10" s="19" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F10" s="12">
         <v>1</v>
@@ -1769,69 +1757,66 @@
       <c r="H10" s="13">
         <v>0</v>
       </c>
-      <c r="I10" s="13">
-        <v>0</v>
-      </c>
-      <c r="J10" s="25">
+      <c r="I10" s="25">
         <v>1.7219053916301622E-4</v>
       </c>
+      <c r="J10" s="14">
+        <v>0</v>
+      </c>
       <c r="K10" s="14">
-        <v>0</v>
-      </c>
-      <c r="L10" s="14">
         <v>5000</v>
       </c>
+      <c r="N10" s="14">
+        <v>0</v>
+      </c>
       <c r="O10" s="14">
-        <v>0</v>
-      </c>
-      <c r="P10" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q10" s="12">
-        <v>0</v>
+      <c r="P10" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="25">
+        <v>1.1192385045596056E-2</v>
       </c>
       <c r="R10" s="25">
-        <v>1.1192385045596056E-2</v>
-      </c>
-      <c r="S10" s="27">
+        <v>0.32026898653096453</v>
+      </c>
+      <c r="S10" s="12">
         <v>0</v>
       </c>
       <c r="T10" s="12">
         <v>0</v>
       </c>
-      <c r="U10" s="12">
-        <v>0</v>
+      <c r="U10" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V10" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W10" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X10" s="13">
-        <f t="shared" si="0"/>
+      <c r="W10" s="13">
+        <f>K10/G10</f>
         <v>2.1639705882352942</v>
       </c>
-      <c r="Z10">
+      <c r="Y10">
         <v>1982</v>
       </c>
+      <c r="AA10">
+        <v>4710768617</v>
+      </c>
       <c r="AB10">
-        <v>4710768617</v>
-      </c>
-      <c r="AC10">
         <v>1406553496</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B11" s="20"/>
       <c r="C11" s="19" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F11" s="12">
         <v>1</v>
@@ -1842,69 +1827,66 @@
       <c r="H11" s="13">
         <v>0</v>
       </c>
-      <c r="I11" s="13">
-        <v>0</v>
-      </c>
-      <c r="J11" s="25">
+      <c r="I11" s="25">
         <v>1.3639768598388177E-4</v>
       </c>
+      <c r="J11" s="14">
+        <v>0</v>
+      </c>
       <c r="K11" s="14">
-        <v>0</v>
-      </c>
-      <c r="L11" s="14">
         <v>5000</v>
       </c>
+      <c r="N11" s="14">
+        <v>0</v>
+      </c>
       <c r="O11" s="14">
-        <v>0</v>
-      </c>
-      <c r="P11" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q11" s="12">
-        <v>0</v>
-      </c>
-      <c r="R11" s="25">
+      <c r="P11" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="25">
         <v>8.865849588952316E-3</v>
       </c>
-      <c r="S11" s="27">
+      <c r="R11" s="27">
+        <v>0</v>
+      </c>
+      <c r="S11" s="12">
         <v>0</v>
       </c>
       <c r="T11" s="12">
         <v>0</v>
       </c>
-      <c r="U11" s="12">
-        <v>0</v>
+      <c r="U11" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V11" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W11" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X11" s="13">
-        <f t="shared" si="0"/>
+      <c r="W11" s="13">
+        <f>K11/G11</f>
         <v>1.9160156250000002</v>
       </c>
-      <c r="Z11">
+      <c r="Y11">
         <v>1949</v>
       </c>
+      <c r="AA11">
+        <v>4741000001</v>
+      </c>
       <c r="AB11">
-        <v>4741000001</v>
-      </c>
-      <c r="AC11">
         <v>15214</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B12" s="20"/>
       <c r="C12" s="19" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F12" s="12">
         <v>1</v>
@@ -1915,69 +1897,66 @@
       <c r="H12" s="13">
         <v>0</v>
       </c>
-      <c r="I12" s="13">
-        <v>0</v>
-      </c>
-      <c r="J12" s="25">
+      <c r="I12" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J12" s="14">
+        <v>0</v>
+      </c>
       <c r="K12" s="14">
-        <v>0</v>
-      </c>
-      <c r="L12" s="14">
         <v>5000</v>
       </c>
+      <c r="N12" s="14">
+        <v>0</v>
+      </c>
       <c r="O12" s="14">
-        <v>0</v>
-      </c>
-      <c r="P12" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q12" s="12">
-        <v>0</v>
-      </c>
-      <c r="R12" s="25">
+      <c r="P12" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S12" s="27">
+      <c r="R12" s="27">
+        <v>0</v>
+      </c>
+      <c r="S12" s="12">
         <v>0</v>
       </c>
       <c r="T12" s="12">
         <v>0</v>
       </c>
-      <c r="U12" s="12">
-        <v>0</v>
+      <c r="U12" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V12" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W12" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X12" s="13">
-        <f t="shared" si="0"/>
+      <c r="W12" s="13">
+        <f>K12/G12</f>
         <v>6.1312499999999996</v>
       </c>
-      <c r="Z12">
+      <c r="Y12">
         <v>1994</v>
       </c>
+      <c r="AA12">
+        <v>4717426321</v>
+      </c>
       <c r="AB12">
-        <v>4717426321</v>
-      </c>
-      <c r="AC12">
         <v>1472277926</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B13" s="20"/>
       <c r="C13" s="19" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F13" s="12">
         <v>1</v>
@@ -1988,69 +1967,66 @@
       <c r="H13" s="13">
         <v>0</v>
       </c>
-      <c r="I13" s="13">
-        <v>0</v>
-      </c>
-      <c r="J13" s="25">
+      <c r="I13" s="25">
         <v>9.3643427926305622E-5</v>
       </c>
+      <c r="J13" s="14">
+        <v>0</v>
+      </c>
       <c r="K13" s="14">
-        <v>0</v>
-      </c>
-      <c r="L13" s="14">
         <v>5000</v>
       </c>
+      <c r="N13" s="14">
+        <v>0</v>
+      </c>
       <c r="O13" s="14">
-        <v>0</v>
-      </c>
-      <c r="P13" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q13" s="12">
-        <v>0</v>
-      </c>
-      <c r="R13" s="25">
+      <c r="P13" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="25">
         <v>6.0868228152098653E-3</v>
       </c>
-      <c r="S13" s="27">
+      <c r="R13" s="27">
+        <v>0</v>
+      </c>
+      <c r="S13" s="12">
         <v>0</v>
       </c>
       <c r="T13" s="12">
         <v>0</v>
       </c>
-      <c r="U13" s="12">
-        <v>0</v>
+      <c r="U13" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V13" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W13" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X13" s="13">
-        <f t="shared" si="0"/>
+      <c r="W13" s="13">
+        <f>K13/G13</f>
         <v>2.5546875</v>
       </c>
-      <c r="Z13">
+      <c r="Y13">
         <v>1998</v>
       </c>
+      <c r="AA13">
+        <v>4718651301</v>
+      </c>
       <c r="AB13">
-        <v>4718651301</v>
-      </c>
-      <c r="AC13">
         <v>1533601401</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B14" s="20"/>
       <c r="C14" s="19" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F14" s="12">
         <v>1</v>
@@ -2061,69 +2037,66 @@
       <c r="H14" s="13">
         <v>0</v>
       </c>
-      <c r="I14" s="13">
-        <v>0</v>
-      </c>
-      <c r="J14" s="25">
+      <c r="I14" s="25">
         <v>7.2708447849138697E-5</v>
       </c>
+      <c r="J14" s="14">
+        <v>0</v>
+      </c>
       <c r="K14" s="14">
-        <v>0</v>
-      </c>
-      <c r="L14" s="14">
         <v>5000</v>
       </c>
+      <c r="N14" s="14">
+        <v>0</v>
+      </c>
       <c r="O14" s="14">
-        <v>0</v>
-      </c>
-      <c r="P14" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q14" s="12">
-        <v>0</v>
-      </c>
-      <c r="R14" s="25">
+      <c r="P14" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="25">
         <v>4.7260491101940149E-3</v>
       </c>
-      <c r="S14" s="27">
+      <c r="R14" s="27">
+        <v>0</v>
+      </c>
+      <c r="S14" s="12">
         <v>0</v>
       </c>
       <c r="T14" s="12">
         <v>0</v>
       </c>
-      <c r="U14" s="12">
-        <v>0</v>
+      <c r="U14" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V14" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W14" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X14" s="13">
-        <f t="shared" si="0"/>
+      <c r="W14" s="13">
+        <f>K14/G14</f>
         <v>75.326785714285705</v>
       </c>
-      <c r="Z14">
+      <c r="Y14">
         <v>1974</v>
       </c>
+      <c r="AA14">
+        <v>46785118</v>
+      </c>
       <c r="AB14">
-        <v>46785118</v>
-      </c>
-      <c r="AC14">
         <v>1558555701</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B15" s="20"/>
       <c r="C15" s="19" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F15" s="12">
         <v>1</v>
@@ -2134,69 +2107,66 @@
       <c r="H15" s="13">
         <v>0</v>
       </c>
-      <c r="I15" s="13">
-        <v>0</v>
-      </c>
-      <c r="J15" s="25">
+      <c r="I15" s="25">
         <v>1.12898177984472E-4</v>
       </c>
+      <c r="J15" s="14">
+        <v>0</v>
+      </c>
       <c r="K15" s="14">
-        <v>0</v>
-      </c>
-      <c r="L15" s="14">
         <v>5000</v>
       </c>
+      <c r="N15" s="14">
+        <v>0</v>
+      </c>
       <c r="O15" s="14">
-        <v>0</v>
-      </c>
-      <c r="P15" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q15" s="12">
-        <v>0</v>
-      </c>
-      <c r="R15" s="25">
+      <c r="P15" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="25">
         <v>7.3383815689906798E-3</v>
       </c>
-      <c r="S15" s="27">
+      <c r="R15" s="27">
+        <v>0</v>
+      </c>
+      <c r="S15" s="12">
         <v>0</v>
       </c>
       <c r="T15" s="12">
         <v>0</v>
       </c>
-      <c r="U15" s="12">
-        <v>0</v>
+      <c r="U15" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V15" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W15" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X15" s="13">
-        <f t="shared" si="0"/>
+      <c r="W15" s="13">
+        <f>K15/G15</f>
         <v>72.284210526315803</v>
       </c>
-      <c r="Z15">
+      <c r="Y15">
         <v>2011</v>
       </c>
+      <c r="AA15">
+        <v>4699784101</v>
+      </c>
       <c r="AB15">
-        <v>4699784101</v>
-      </c>
-      <c r="AC15">
         <v>1546751901</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B16" s="20"/>
       <c r="C16" s="19" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F16" s="12">
         <v>1</v>
@@ -2207,69 +2177,66 @@
       <c r="H16" s="13">
         <v>0</v>
       </c>
-      <c r="I16" s="13">
-        <v>0</v>
-      </c>
-      <c r="J16" s="25">
+      <c r="I16" s="25">
         <v>1.9032505466392189E-5</v>
       </c>
+      <c r="J16" s="14">
+        <v>0</v>
+      </c>
       <c r="K16" s="14">
-        <v>0</v>
-      </c>
-      <c r="L16" s="14">
         <v>5000</v>
       </c>
+      <c r="N16" s="14">
+        <v>0</v>
+      </c>
       <c r="O16" s="14">
-        <v>0</v>
-      </c>
-      <c r="P16" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q16" s="12">
-        <v>0</v>
-      </c>
-      <c r="R16" s="25">
+      <c r="P16" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="25">
         <v>1.2371128553154923E-3</v>
       </c>
-      <c r="S16" s="27">
+      <c r="R16" s="27">
+        <v>0</v>
+      </c>
+      <c r="S16" s="12">
         <v>0</v>
       </c>
       <c r="T16" s="12">
         <v>0</v>
       </c>
-      <c r="U16" s="12">
-        <v>0</v>
+      <c r="U16" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V16" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W16" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X16" s="13">
-        <f t="shared" si="0"/>
+      <c r="W16" s="13">
+        <f>K16/G16</f>
         <v>82.333928571428558</v>
       </c>
-      <c r="Z16">
+      <c r="Y16">
         <v>1964</v>
       </c>
+      <c r="AA16">
+        <v>4682809068</v>
+      </c>
       <c r="AB16">
-        <v>4682809068</v>
-      </c>
-      <c r="AC16">
         <v>1556616553</v>
       </c>
     </row>
-    <row r="17" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B17" s="20"/>
       <c r="C17" s="19" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F17" s="12">
         <v>1</v>
@@ -2280,69 +2247,66 @@
       <c r="H17" s="13">
         <v>0</v>
       </c>
-      <c r="I17" s="13">
-        <v>0</v>
-      </c>
-      <c r="J17" s="25">
+      <c r="I17" s="25">
         <v>5.9495468904415532E-5</v>
       </c>
+      <c r="J17" s="14">
+        <v>0</v>
+      </c>
       <c r="K17" s="14">
-        <v>0</v>
-      </c>
-      <c r="L17" s="14">
         <v>5000</v>
       </c>
+      <c r="N17" s="14">
+        <v>0</v>
+      </c>
       <c r="O17" s="14">
-        <v>0</v>
-      </c>
-      <c r="P17" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q17" s="12">
-        <v>0</v>
-      </c>
-      <c r="R17" s="25">
+      <c r="P17" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="25">
         <v>3.8672054787870095E-3</v>
       </c>
-      <c r="S17" s="27">
+      <c r="R17" s="27">
+        <v>0</v>
+      </c>
+      <c r="S17" s="12">
         <v>0</v>
       </c>
       <c r="T17" s="12">
         <v>0</v>
       </c>
-      <c r="U17" s="12">
-        <v>0</v>
+      <c r="U17" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V17" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W17" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X17" s="13">
-        <f t="shared" si="0"/>
+      <c r="W17" s="13">
+        <f>K17/G17</f>
         <v>72.46022727272728</v>
       </c>
-      <c r="Z17">
+      <c r="Y17">
         <v>2024</v>
       </c>
+      <c r="AA17">
+        <v>4713909101</v>
+      </c>
       <c r="AB17">
-        <v>4713909101</v>
-      </c>
-      <c r="AC17">
         <v>1532804601</v>
       </c>
     </row>
-    <row r="18" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B18" s="20"/>
       <c r="C18" s="19" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F18" s="12">
         <v>1</v>
@@ -2353,69 +2317,66 @@
       <c r="H18" s="13">
         <v>0</v>
       </c>
-      <c r="I18" s="13">
-        <v>0</v>
-      </c>
-      <c r="J18" s="25">
+      <c r="I18" s="25">
         <v>1.0448815569668966E-4</v>
       </c>
+      <c r="J18" s="14">
+        <v>0</v>
+      </c>
       <c r="K18" s="14">
-        <v>0</v>
-      </c>
-      <c r="L18" s="14">
         <v>5000</v>
       </c>
+      <c r="N18" s="14">
+        <v>0</v>
+      </c>
       <c r="O18" s="14">
-        <v>0</v>
-      </c>
-      <c r="P18" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q18" s="12">
-        <v>0</v>
-      </c>
-      <c r="R18" s="25">
+      <c r="P18" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="25">
         <v>6.7917301202848283E-3</v>
       </c>
-      <c r="S18" s="27">
+      <c r="R18" s="27">
+        <v>0</v>
+      </c>
+      <c r="S18" s="12">
         <v>0</v>
       </c>
       <c r="T18" s="12">
         <v>0</v>
       </c>
-      <c r="U18" s="12">
-        <v>0</v>
+      <c r="U18" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V18" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W18" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X18" s="13">
-        <f t="shared" si="0"/>
+      <c r="W18" s="13">
+        <f>K18/G18</f>
         <v>74.341406250000006</v>
       </c>
-      <c r="Z18">
-        <v>0</v>
+      <c r="Y18">
+        <v>0</v>
+      </c>
+      <c r="AA18">
+        <v>4703986387</v>
       </c>
       <c r="AB18">
-        <v>4703986387</v>
-      </c>
-      <c r="AC18">
         <v>1544275136</v>
       </c>
     </row>
-    <row r="19" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B19" s="20"/>
       <c r="C19" s="19" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F19" s="12">
         <v>1</v>
@@ -2426,69 +2387,66 @@
       <c r="H19" s="13">
         <v>0</v>
       </c>
-      <c r="I19" s="13">
-        <v>0</v>
-      </c>
-      <c r="J19" s="25">
+      <c r="I19" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J19" s="14">
+        <v>0</v>
+      </c>
       <c r="K19" s="14">
-        <v>0</v>
-      </c>
-      <c r="L19" s="14">
         <v>5000</v>
       </c>
+      <c r="N19" s="14">
+        <v>0</v>
+      </c>
       <c r="O19" s="14">
-        <v>0</v>
-      </c>
-      <c r="P19" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q19" s="12">
-        <v>0</v>
-      </c>
-      <c r="R19" s="25">
+      <c r="P19" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S19" s="27">
+      <c r="R19" s="27">
+        <v>0</v>
+      </c>
+      <c r="S19" s="12">
         <v>0</v>
       </c>
       <c r="T19" s="12">
         <v>0</v>
       </c>
-      <c r="U19" s="12">
-        <v>0</v>
+      <c r="U19" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V19" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W19" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X19" s="13">
-        <f t="shared" si="0"/>
+      <c r="W19" s="13">
+        <f>K19/G19</f>
         <v>5.109375</v>
       </c>
-      <c r="Z19">
-        <v>0</v>
+      <c r="Y19">
+        <v>0</v>
+      </c>
+      <c r="AA19">
+        <v>4699409124</v>
       </c>
       <c r="AB19">
-        <v>4699409124</v>
-      </c>
-      <c r="AC19">
         <v>1508502495</v>
       </c>
     </row>
-    <row r="20" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B20" s="20"/>
       <c r="C20" s="19" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F20" s="12">
         <v>1</v>
@@ -2496,72 +2454,69 @@
       <c r="G20" s="25">
         <v>84.811416921508666</v>
       </c>
-      <c r="H20" s="13">
-        <v>0</v>
-      </c>
-      <c r="I20" s="23">
+      <c r="H20" s="23">
         <v>123.1396524</v>
       </c>
-      <c r="J20" s="25">
+      <c r="I20" s="25">
         <v>4.9272151773994549E-3</v>
       </c>
-      <c r="K20" s="22">
+      <c r="J20" s="22">
         <v>1.6999999999999999E-3</v>
       </c>
-      <c r="L20" s="22">
+      <c r="K20" s="14">
         <v>15000000</v>
       </c>
+      <c r="N20" s="14">
+        <v>0</v>
+      </c>
       <c r="O20" s="14">
-        <v>0</v>
-      </c>
-      <c r="P20" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q20" s="12">
+      <c r="P20" s="12">
         <v>1</v>
       </c>
-      <c r="R20" s="25">
+      <c r="Q20" s="25">
         <v>0.32026898653096453</v>
       </c>
-      <c r="S20" s="25">
-        <v>0.32026898653096453</v>
+      <c r="R20" s="27">
+        <v>0</v>
+      </c>
+      <c r="S20" s="12">
+        <v>0</v>
       </c>
       <c r="T20" s="12">
         <v>0</v>
       </c>
-      <c r="U20" s="12">
-        <v>0</v>
+      <c r="U20" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V20" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W20" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X20" s="13">
-        <f t="shared" si="0"/>
+      <c r="W20" s="13">
+        <f>K20/G20</f>
         <v>176862.98076923078</v>
       </c>
-      <c r="Z20">
-        <v>0</v>
+      <c r="Y20">
+        <v>0</v>
+      </c>
+      <c r="AA20">
+        <v>4710370743</v>
       </c>
       <c r="AB20">
-        <v>4710370743</v>
-      </c>
-      <c r="AC20">
         <v>1348112241</v>
       </c>
     </row>
-    <row r="21" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B21" s="20"/>
       <c r="C21" s="19" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F21" s="12">
         <v>1</v>
@@ -2572,69 +2527,66 @@
       <c r="H21" s="13">
         <v>0</v>
       </c>
-      <c r="I21" s="13">
-        <v>0</v>
-      </c>
-      <c r="J21" s="25">
+      <c r="I21" s="25">
         <v>1.0348150151375814E-4</v>
       </c>
+      <c r="J21" s="14">
+        <v>0</v>
+      </c>
       <c r="K21" s="14">
-        <v>0</v>
-      </c>
-      <c r="L21" s="14">
         <v>5000</v>
       </c>
+      <c r="N21" s="14">
+        <v>0</v>
+      </c>
       <c r="O21" s="14">
-        <v>0</v>
-      </c>
-      <c r="P21" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q21" s="12">
-        <v>0</v>
-      </c>
-      <c r="R21" s="25">
+      <c r="P21" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="25">
         <v>6.7262975983942794E-3</v>
       </c>
-      <c r="S21" s="27">
+      <c r="R21" s="27">
+        <v>0</v>
+      </c>
+      <c r="S21" s="12">
         <v>0</v>
       </c>
       <c r="T21" s="12">
         <v>0</v>
       </c>
-      <c r="U21" s="12">
-        <v>0</v>
+      <c r="U21" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V21" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W21" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X21" s="13">
-        <f t="shared" si="0"/>
+      <c r="W21" s="13">
+        <f>K21/G21</f>
         <v>72.284210526315803</v>
       </c>
-      <c r="Z21">
+      <c r="Y21">
         <v>2013</v>
       </c>
+      <c r="AA21">
+        <v>4694360461</v>
+      </c>
       <c r="AB21">
-        <v>4694360461</v>
-      </c>
-      <c r="AC21">
         <v>155040946</v>
       </c>
     </row>
-    <row r="22" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B22" s="20"/>
       <c r="C22" s="19" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F22" s="12">
         <v>1</v>
@@ -2645,69 +2597,66 @@
       <c r="H22" s="13">
         <v>0</v>
       </c>
-      <c r="I22" s="13">
-        <v>0</v>
-      </c>
-      <c r="J22" s="25">
+      <c r="I22" s="25">
         <v>1.4666336007454863E-4</v>
       </c>
+      <c r="J22" s="14">
+        <v>0</v>
+      </c>
       <c r="K22" s="14">
-        <v>0</v>
-      </c>
-      <c r="L22" s="14">
         <v>5000</v>
       </c>
+      <c r="N22" s="14">
+        <v>0</v>
+      </c>
       <c r="O22" s="14">
-        <v>0</v>
-      </c>
-      <c r="P22" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q22" s="12">
-        <v>0</v>
-      </c>
-      <c r="R22" s="25">
+      <c r="P22" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="25">
         <v>9.5331184048456606E-3</v>
       </c>
-      <c r="S22" s="27">
+      <c r="R22" s="27">
+        <v>0</v>
+      </c>
+      <c r="S22" s="12">
         <v>0</v>
       </c>
       <c r="T22" s="12">
         <v>0</v>
       </c>
-      <c r="U22" s="12">
-        <v>0</v>
+      <c r="U22" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V22" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W22" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X22" s="13">
-        <f t="shared" si="0"/>
+      <c r="W22" s="13">
+        <f>K22/G22</f>
         <v>58.587499999999999</v>
       </c>
-      <c r="Z22">
+      <c r="Y22">
         <v>2023</v>
       </c>
+      <c r="AA22">
+        <v>4729200001</v>
+      </c>
       <c r="AB22">
-        <v>4729200001</v>
-      </c>
-      <c r="AC22">
         <v>15323</v>
       </c>
     </row>
-    <row r="23" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B23" s="20"/>
       <c r="C23" s="19" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F23" s="12">
         <v>1</v>
@@ -2718,69 +2667,66 @@
       <c r="H23" s="13">
         <v>0</v>
       </c>
-      <c r="I23" s="13">
-        <v>0</v>
-      </c>
-      <c r="J23" s="25">
+      <c r="I23" s="25">
         <v>8.9709393743275537E-5</v>
       </c>
+      <c r="J23" s="14">
+        <v>0</v>
+      </c>
       <c r="K23" s="14">
-        <v>0</v>
-      </c>
-      <c r="L23" s="14">
         <v>5000</v>
       </c>
+      <c r="N23" s="14">
+        <v>0</v>
+      </c>
       <c r="O23" s="14">
-        <v>0</v>
-      </c>
-      <c r="P23" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q23" s="12">
-        <v>0</v>
-      </c>
-      <c r="R23" s="25">
+      <c r="P23" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="25">
         <v>5.8311105933129097E-3</v>
       </c>
-      <c r="S23" s="27">
+      <c r="R23" s="27">
+        <v>0</v>
+      </c>
+      <c r="S23" s="12">
         <v>0</v>
       </c>
       <c r="T23" s="12">
         <v>0</v>
       </c>
-      <c r="U23" s="12">
-        <v>0</v>
+      <c r="U23" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V23" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W23" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X23" s="13">
-        <f t="shared" si="0"/>
+      <c r="W23" s="13">
+        <f>K23/G23</f>
         <v>6.1919554455445542</v>
       </c>
-      <c r="Z23">
+      <c r="Y23">
         <v>1988</v>
       </c>
+      <c r="AA23">
+        <v>46857847</v>
+      </c>
       <c r="AB23">
-        <v>46857847</v>
-      </c>
-      <c r="AC23">
         <v>1553730001</v>
       </c>
     </row>
-    <row r="24" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B24" s="20"/>
       <c r="C24" s="19" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F24" s="12">
         <v>1</v>
@@ -2791,69 +2737,66 @@
       <c r="H24" s="13">
         <v>0</v>
       </c>
-      <c r="I24" s="13">
-        <v>0</v>
-      </c>
-      <c r="J24" s="25">
+      <c r="I24" s="25">
         <v>6.8370332515645875E-5</v>
       </c>
+      <c r="J24" s="14">
+        <v>0</v>
+      </c>
       <c r="K24" s="14">
-        <v>0</v>
-      </c>
-      <c r="L24" s="14">
         <v>5000</v>
       </c>
+      <c r="N24" s="14">
+        <v>0</v>
+      </c>
       <c r="O24" s="14">
-        <v>0</v>
-      </c>
-      <c r="P24" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q24" s="12">
-        <v>0</v>
-      </c>
-      <c r="R24" s="25">
+      <c r="P24" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="25">
         <v>4.444071613516982E-3</v>
       </c>
-      <c r="S24" s="27">
+      <c r="R24" s="27">
+        <v>0</v>
+      </c>
+      <c r="S24" s="12">
         <v>0</v>
       </c>
       <c r="T24" s="12">
         <v>0</v>
       </c>
-      <c r="U24" s="12">
-        <v>0</v>
+      <c r="U24" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V24" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W24" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X24" s="13">
-        <f t="shared" si="0"/>
+      <c r="W24" s="13">
+        <f>K24/G24</f>
         <v>9.81</v>
       </c>
-      <c r="Z24">
-        <v>0</v>
+      <c r="Y24">
+        <v>0</v>
+      </c>
+      <c r="AA24">
+        <v>4738847601</v>
       </c>
       <c r="AB24">
-        <v>4738847601</v>
-      </c>
-      <c r="AC24">
         <v>15095161</v>
       </c>
     </row>
-    <row r="25" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B25" s="20"/>
       <c r="C25" s="19" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F25" s="12">
         <v>1</v>
@@ -2864,69 +2807,66 @@
       <c r="H25" s="13">
         <v>0</v>
       </c>
-      <c r="I25" s="13">
-        <v>0</v>
-      </c>
-      <c r="J25" s="25">
+      <c r="I25" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J25" s="14">
+        <v>0</v>
+      </c>
       <c r="K25" s="14">
-        <v>0</v>
-      </c>
-      <c r="L25" s="14">
         <v>5000</v>
       </c>
+      <c r="N25" s="14">
+        <v>0</v>
+      </c>
       <c r="O25" s="14">
-        <v>0</v>
-      </c>
-      <c r="P25" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q25" s="12">
-        <v>0</v>
-      </c>
-      <c r="R25" s="25">
+      <c r="P25" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S25" s="27">
+      <c r="R25" s="27">
+        <v>0</v>
+      </c>
+      <c r="S25" s="12">
         <v>0</v>
       </c>
       <c r="T25" s="12">
         <v>0</v>
       </c>
-      <c r="U25" s="12">
-        <v>0</v>
+      <c r="U25" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V25" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W25" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X25" s="13">
-        <f t="shared" si="0"/>
+      <c r="W25" s="13">
+        <f>K25/G25</f>
         <v>7.5461538461538469</v>
       </c>
-      <c r="Z25">
-        <v>0</v>
+      <c r="Y25">
+        <v>0</v>
+      </c>
+      <c r="AA25">
+        <v>4674575769</v>
       </c>
       <c r="AB25">
-        <v>4674575769</v>
-      </c>
-      <c r="AC25">
         <v>1557182718</v>
       </c>
     </row>
-    <row r="26" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B26" s="20"/>
       <c r="C26" s="19" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F26" s="12">
         <v>1</v>
@@ -2937,69 +2877,66 @@
       <c r="H26" s="13">
         <v>0</v>
       </c>
-      <c r="I26" s="13">
-        <v>0</v>
-      </c>
-      <c r="J26" s="25">
+      <c r="I26" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J26" s="14">
+        <v>0</v>
+      </c>
       <c r="K26" s="14">
-        <v>0</v>
-      </c>
-      <c r="L26" s="14">
         <v>5000000</v>
       </c>
+      <c r="N26" s="14">
+        <v>0</v>
+      </c>
       <c r="O26" s="14">
-        <v>0</v>
-      </c>
-      <c r="P26" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q26" s="12">
+      <c r="P26" s="12">
         <v>1</v>
       </c>
-      <c r="R26" s="25">
+      <c r="Q26" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S26" s="27">
+      <c r="R26" s="27">
+        <v>0</v>
+      </c>
+      <c r="S26" s="12">
         <v>0</v>
       </c>
       <c r="T26" s="12">
         <v>0</v>
       </c>
-      <c r="U26" s="12">
-        <v>0</v>
+      <c r="U26" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V26" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W26" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X26" s="13">
-        <f t="shared" si="0"/>
+      <c r="W26" s="13">
+        <f>K26/G26</f>
         <v>8174.9999999999991</v>
       </c>
-      <c r="Z26">
-        <v>0</v>
+      <c r="Y26">
+        <v>0</v>
+      </c>
+      <c r="AA26">
+        <v>4697878577</v>
       </c>
       <c r="AB26">
-        <v>4697878577</v>
-      </c>
-      <c r="AC26">
         <v>1502319618</v>
       </c>
     </row>
-    <row r="27" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B27" s="20"/>
       <c r="C27" s="19" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F27" s="12">
         <v>1</v>
@@ -3010,69 +2947,66 @@
       <c r="H27" s="13">
         <v>0</v>
       </c>
-      <c r="I27" s="13">
-        <v>0</v>
-      </c>
-      <c r="J27" s="25">
+      <c r="I27" s="25">
         <v>9.8526263529088916E-5</v>
       </c>
+      <c r="J27" s="14">
+        <v>0</v>
+      </c>
       <c r="K27" s="14">
-        <v>0</v>
-      </c>
-      <c r="L27" s="14">
         <v>5000</v>
       </c>
+      <c r="N27" s="14">
+        <v>0</v>
+      </c>
       <c r="O27" s="14">
-        <v>0</v>
-      </c>
-      <c r="P27" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q27" s="12">
-        <v>0</v>
-      </c>
-      <c r="R27" s="25">
+      <c r="P27" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="25">
         <v>6.4042071293907796E-3</v>
       </c>
-      <c r="S27" s="27">
+      <c r="R27" s="27">
+        <v>0</v>
+      </c>
+      <c r="S27" s="12">
         <v>0</v>
       </c>
       <c r="T27" s="12">
         <v>0</v>
       </c>
-      <c r="U27" s="12">
-        <v>0</v>
+      <c r="U27" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V27" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W27" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X27" s="13">
-        <f t="shared" si="0"/>
+      <c r="W27" s="13">
+        <f>K27/G27</f>
         <v>8.4894230769230763</v>
       </c>
-      <c r="Z27">
+      <c r="Y27">
         <v>2009</v>
       </c>
+      <c r="AA27">
+        <v>4720926001</v>
+      </c>
       <c r="AB27">
-        <v>4720926001</v>
-      </c>
-      <c r="AC27">
         <v>15335656</v>
       </c>
     </row>
-    <row r="28" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B28" s="20"/>
       <c r="C28" s="19" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F28" s="12">
         <v>1</v>
@@ -3083,69 +3017,66 @@
       <c r="H28" s="13">
         <v>0</v>
       </c>
-      <c r="I28" s="13">
-        <v>0</v>
-      </c>
-      <c r="J28" s="25">
+      <c r="I28" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J28" s="14">
+        <v>0</v>
+      </c>
       <c r="K28" s="14">
-        <v>0</v>
-      </c>
-      <c r="L28" s="14">
         <v>5000</v>
       </c>
+      <c r="N28" s="14">
+        <v>0</v>
+      </c>
       <c r="O28" s="14">
-        <v>0</v>
-      </c>
-      <c r="P28" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q28" s="12">
-        <v>0</v>
-      </c>
-      <c r="R28" s="25">
+      <c r="P28" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S28" s="27">
+      <c r="R28" s="27">
+        <v>0</v>
+      </c>
+      <c r="S28" s="12">
         <v>0</v>
       </c>
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="12">
-        <v>0</v>
+      <c r="U28" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V28" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W28" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X28" s="13">
-        <f t="shared" si="0"/>
+      <c r="W28" s="13">
+        <f>K28/G28</f>
         <v>5.7034883720930241E-2</v>
       </c>
-      <c r="Z28">
+      <c r="Y28">
         <v>2013</v>
       </c>
+      <c r="AA28">
+        <v>4736520001</v>
+      </c>
       <c r="AB28">
-        <v>4736520001</v>
-      </c>
-      <c r="AC28">
         <v>1533440001</v>
       </c>
     </row>
-    <row r="29" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B29" s="20"/>
       <c r="C29" s="19" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F29" s="12">
         <v>1</v>
@@ -3156,69 +3087,66 @@
       <c r="H29" s="13">
         <v>0</v>
       </c>
-      <c r="I29" s="13">
-        <v>0</v>
-      </c>
-      <c r="J29" s="25">
+      <c r="I29" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J29" s="14">
+        <v>0</v>
+      </c>
       <c r="K29" s="14">
-        <v>0</v>
-      </c>
-      <c r="L29" s="14">
         <v>5000</v>
       </c>
+      <c r="N29" s="14">
+        <v>0</v>
+      </c>
       <c r="O29" s="14">
-        <v>0</v>
-      </c>
-      <c r="P29" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q29" s="12">
-        <v>0</v>
-      </c>
-      <c r="R29" s="25">
+      <c r="P29" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S29" s="27">
+      <c r="R29" s="27">
+        <v>0</v>
+      </c>
+      <c r="S29" s="12">
         <v>0</v>
       </c>
       <c r="T29" s="12">
         <v>0</v>
       </c>
-      <c r="U29" s="12">
-        <v>0</v>
+      <c r="U29" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V29" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W29" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X29" s="13">
-        <f t="shared" si="0"/>
+      <c r="W29" s="13">
+        <f>K29/G29</f>
         <v>61.312500000000007</v>
       </c>
-      <c r="Z29">
-        <v>0</v>
+      <c r="Y29">
+        <v>0</v>
+      </c>
+      <c r="AA29">
+        <v>4721774401</v>
       </c>
       <c r="AB29">
-        <v>4721774401</v>
-      </c>
-      <c r="AC29">
         <v>14599075</v>
       </c>
     </row>
-    <row r="30" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B30" s="20"/>
       <c r="C30" s="19" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F30" s="12">
         <v>1</v>
@@ -3229,69 +3157,66 @@
       <c r="H30" s="13">
         <v>0</v>
       </c>
-      <c r="I30" s="13">
-        <v>0</v>
-      </c>
-      <c r="J30" s="25">
+      <c r="I30" s="25">
         <v>7.8180055576928815E-5</v>
       </c>
+      <c r="J30" s="14">
+        <v>0</v>
+      </c>
       <c r="K30" s="14">
-        <v>0</v>
-      </c>
-      <c r="L30" s="14">
         <v>5000</v>
       </c>
+      <c r="N30" s="14">
+        <v>0</v>
+      </c>
       <c r="O30" s="14">
-        <v>0</v>
-      </c>
-      <c r="P30" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q30" s="12">
-        <v>0</v>
-      </c>
-      <c r="R30" s="25">
+      <c r="P30" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="25">
         <v>5.0817036125003724E-3</v>
       </c>
-      <c r="S30" s="27">
+      <c r="R30" s="27">
+        <v>0</v>
+      </c>
+      <c r="S30" s="12">
         <v>0</v>
       </c>
       <c r="T30" s="12">
         <v>0</v>
       </c>
-      <c r="U30" s="12">
-        <v>0</v>
+      <c r="U30" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V30" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W30" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X30" s="13">
-        <f t="shared" si="0"/>
+      <c r="W30" s="13">
+        <f>K30/G30</f>
         <v>7.8830357142857137</v>
       </c>
-      <c r="Z30">
-        <v>0</v>
+      <c r="Y30">
+        <v>0</v>
+      </c>
+      <c r="AA30">
+        <v>4725087014</v>
       </c>
       <c r="AB30">
-        <v>4725087014</v>
-      </c>
-      <c r="AC30">
         <v>1531009022</v>
       </c>
     </row>
-    <row r="31" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B31" s="20"/>
       <c r="C31" s="19" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F31" s="12">
         <v>1</v>
@@ -3302,69 +3227,66 @@
       <c r="H31" s="13">
         <v>0</v>
       </c>
-      <c r="I31" s="13">
-        <v>0</v>
-      </c>
-      <c r="J31" s="25">
+      <c r="I31" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J31" s="14">
+        <v>0</v>
+      </c>
       <c r="K31" s="14">
-        <v>0</v>
-      </c>
-      <c r="L31" s="14">
         <v>5000</v>
       </c>
+      <c r="N31" s="14">
+        <v>0</v>
+      </c>
       <c r="O31" s="14">
-        <v>0</v>
-      </c>
-      <c r="P31" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q31" s="12">
-        <v>0</v>
-      </c>
-      <c r="R31" s="25">
+      <c r="P31" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S31" s="27">
+      <c r="R31" s="27">
+        <v>0</v>
+      </c>
+      <c r="S31" s="12">
         <v>0</v>
       </c>
       <c r="T31" s="12">
         <v>0</v>
       </c>
-      <c r="U31" s="12">
-        <v>0</v>
+      <c r="U31" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V31" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W31" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X31" s="13">
-        <f t="shared" si="0"/>
+      <c r="W31" s="13">
+        <f>K31/G31</f>
         <v>122.62500000000001</v>
       </c>
-      <c r="Z31">
-        <v>0</v>
+      <c r="Y31">
+        <v>0</v>
+      </c>
+      <c r="AA31">
+        <v>4674433801</v>
       </c>
       <c r="AB31">
-        <v>4674433801</v>
-      </c>
-      <c r="AC31">
         <v>1557045501</v>
       </c>
     </row>
-    <row r="32" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B32" s="20"/>
       <c r="C32" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F32" s="12">
         <v>1</v>
@@ -3375,69 +3297,66 @@
       <c r="H32" s="13">
         <v>0</v>
       </c>
-      <c r="I32" s="13">
-        <v>0</v>
-      </c>
-      <c r="J32" s="25">
+      <c r="I32" s="25">
         <v>6.3496793032866511E-5</v>
       </c>
+      <c r="J32" s="14">
+        <v>0</v>
+      </c>
       <c r="K32" s="14">
-        <v>0</v>
-      </c>
-      <c r="L32" s="14">
         <v>5000</v>
       </c>
+      <c r="N32" s="14">
+        <v>0</v>
+      </c>
       <c r="O32" s="14">
-        <v>0</v>
-      </c>
-      <c r="P32" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q32" s="12">
-        <v>0</v>
-      </c>
-      <c r="R32" s="25">
+      <c r="P32" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="25">
         <v>4.1272915471363232E-3</v>
       </c>
-      <c r="S32" s="27">
+      <c r="R32" s="27">
+        <v>0</v>
+      </c>
+      <c r="S32" s="12">
         <v>0</v>
       </c>
       <c r="T32" s="12">
         <v>0</v>
       </c>
-      <c r="U32" s="12">
-        <v>0</v>
+      <c r="U32" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V32" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W32" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X32" s="13">
-        <f t="shared" si="0"/>
+      <c r="W32" s="13">
+        <f>K32/G32</f>
         <v>65.085576923076914</v>
       </c>
-      <c r="Z32">
+      <c r="Y32">
         <v>1982</v>
       </c>
+      <c r="AA32">
+        <v>4671685586</v>
+      </c>
       <c r="AB32">
-        <v>4671685586</v>
-      </c>
-      <c r="AC32">
         <v>1562152978</v>
       </c>
     </row>
-    <row r="33" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B33" s="20"/>
       <c r="C33" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F33" s="12">
         <v>1</v>
@@ -3448,69 +3367,66 @@
       <c r="H33" s="13">
         <v>0</v>
       </c>
-      <c r="I33" s="13">
-        <v>0</v>
-      </c>
-      <c r="J33" s="25">
+      <c r="I33" s="25">
         <v>1.6206168391813292E-4</v>
       </c>
+      <c r="J33" s="14">
+        <v>0</v>
+      </c>
       <c r="K33" s="14">
-        <v>0</v>
-      </c>
-      <c r="L33" s="14">
         <v>5000</v>
       </c>
+      <c r="N33" s="14">
+        <v>0</v>
+      </c>
       <c r="O33" s="14">
-        <v>0</v>
-      </c>
-      <c r="P33" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q33" s="12">
-        <v>0</v>
-      </c>
-      <c r="R33" s="25">
+      <c r="P33" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="25">
         <v>1.0534009454678639E-2</v>
       </c>
-      <c r="S33" s="27">
+      <c r="R33" s="27">
+        <v>0</v>
+      </c>
+      <c r="S33" s="12">
         <v>0</v>
       </c>
       <c r="T33" s="12">
         <v>0</v>
       </c>
-      <c r="U33" s="12">
-        <v>0</v>
+      <c r="U33" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V33" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W33" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X33" s="13">
-        <f t="shared" si="0"/>
+      <c r="W33" s="13">
+        <f>K33/G33</f>
         <v>173.71875</v>
       </c>
-      <c r="Z33">
+      <c r="Y33">
         <v>1985</v>
       </c>
+      <c r="AA33">
+        <v>4710441021</v>
+      </c>
       <c r="AB33">
-        <v>4710441021</v>
-      </c>
-      <c r="AC33">
         <v>1408673125</v>
       </c>
     </row>
-    <row r="34" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B34" s="20"/>
       <c r="C34" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F34" s="12">
         <v>1</v>
@@ -3521,69 +3437,66 @@
       <c r="H34" s="13">
         <v>0</v>
       </c>
-      <c r="I34" s="13">
-        <v>0</v>
-      </c>
-      <c r="J34" s="25">
+      <c r="I34" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J34" s="14">
+        <v>0</v>
+      </c>
       <c r="K34" s="14">
-        <v>0</v>
-      </c>
-      <c r="L34" s="14">
         <v>5000</v>
       </c>
+      <c r="N34" s="14">
+        <v>0</v>
+      </c>
       <c r="O34" s="14">
-        <v>0</v>
-      </c>
-      <c r="P34" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q34" s="12">
-        <v>0</v>
-      </c>
-      <c r="R34" s="25">
+      <c r="P34" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S34" s="27">
+      <c r="R34" s="27">
+        <v>0</v>
+      </c>
+      <c r="S34" s="12">
         <v>0</v>
       </c>
       <c r="T34" s="12">
         <v>0</v>
       </c>
-      <c r="U34" s="12">
-        <v>0</v>
+      <c r="U34" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V34" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W34" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X34" s="13">
-        <f t="shared" si="0"/>
+      <c r="W34" s="13">
+        <f>K34/G34</f>
         <v>7.6640625000000009</v>
       </c>
-      <c r="Z34">
-        <v>0</v>
+      <c r="Y34">
+        <v>0</v>
+      </c>
+      <c r="AA34">
+        <v>4698734792</v>
       </c>
       <c r="AB34">
-        <v>4698734792</v>
-      </c>
-      <c r="AC34">
         <v>150912762</v>
       </c>
     </row>
-    <row r="35" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B35" s="20"/>
       <c r="C35" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F35" s="12">
         <v>1</v>
@@ -3594,69 +3507,66 @@
       <c r="H35" s="13">
         <v>0</v>
       </c>
-      <c r="I35" s="13">
-        <v>0</v>
-      </c>
-      <c r="J35" s="25">
+      <c r="I35" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J35" s="14">
+        <v>0</v>
+      </c>
       <c r="K35" s="14">
-        <v>0</v>
-      </c>
-      <c r="L35" s="14">
         <v>5000</v>
       </c>
+      <c r="N35" s="14">
+        <v>0</v>
+      </c>
       <c r="O35" s="14">
-        <v>0</v>
-      </c>
-      <c r="P35" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q35" s="12">
-        <v>0</v>
-      </c>
-      <c r="R35" s="25">
+      <c r="P35" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S35" s="27">
+      <c r="R35" s="27">
+        <v>0</v>
+      </c>
+      <c r="S35" s="12">
         <v>0</v>
       </c>
       <c r="T35" s="12">
         <v>0</v>
       </c>
-      <c r="U35" s="12">
-        <v>0</v>
+      <c r="U35" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V35" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W35" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X35" s="13">
-        <f t="shared" si="0"/>
+      <c r="W35" s="13">
+        <f>K35/G35</f>
         <v>10.21875</v>
       </c>
-      <c r="Z35">
-        <v>0</v>
+      <c r="Y35">
+        <v>0</v>
+      </c>
+      <c r="AA35">
+        <v>4717522501</v>
       </c>
       <c r="AB35">
-        <v>4717522501</v>
-      </c>
-      <c r="AC35">
         <v>1532038501</v>
       </c>
     </row>
-    <row r="36" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B36" s="20"/>
       <c r="C36" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F36" s="12">
         <v>1</v>
@@ -3667,69 +3577,66 @@
       <c r="H36" s="13">
         <v>0</v>
       </c>
-      <c r="I36" s="13">
-        <v>0</v>
-      </c>
-      <c r="J36" s="25">
+      <c r="I36" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J36" s="14">
+        <v>0</v>
+      </c>
       <c r="K36" s="14">
-        <v>0</v>
-      </c>
-      <c r="L36" s="14">
         <v>5000</v>
       </c>
+      <c r="N36" s="14">
+        <v>0</v>
+      </c>
       <c r="O36" s="14">
-        <v>0</v>
-      </c>
-      <c r="P36" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q36" s="12">
-        <v>0</v>
-      </c>
-      <c r="R36" s="25">
+      <c r="P36" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S36" s="27">
+      <c r="R36" s="27">
+        <v>0</v>
+      </c>
+      <c r="S36" s="12">
         <v>0</v>
       </c>
       <c r="T36" s="12">
         <v>0</v>
       </c>
-      <c r="U36" s="12">
-        <v>0</v>
+      <c r="U36" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V36" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W36" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X36" s="13">
-        <f t="shared" si="0"/>
+      <c r="W36" s="13">
+        <f>K36/G36</f>
         <v>122.62500000000001</v>
       </c>
-      <c r="Z36">
-        <v>0</v>
+      <c r="Y36">
+        <v>0</v>
+      </c>
+      <c r="AA36">
+        <v>4702151301</v>
       </c>
       <c r="AB36">
-        <v>4702151301</v>
-      </c>
-      <c r="AC36">
         <v>1516653701</v>
       </c>
     </row>
-    <row r="37" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B37" s="20"/>
       <c r="C37" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F37" s="12">
         <v>1</v>
@@ -3740,69 +3647,66 @@
       <c r="H37" s="13">
         <v>0</v>
       </c>
-      <c r="I37" s="13">
-        <v>0</v>
-      </c>
-      <c r="J37" s="25">
+      <c r="I37" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J37" s="14">
+        <v>0</v>
+      </c>
       <c r="K37" s="14">
-        <v>0</v>
-      </c>
-      <c r="L37" s="14">
         <v>5000</v>
       </c>
+      <c r="N37" s="14">
+        <v>0</v>
+      </c>
       <c r="O37" s="14">
-        <v>0</v>
-      </c>
-      <c r="P37" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q37" s="12">
-        <v>0</v>
-      </c>
-      <c r="R37" s="25">
+      <c r="P37" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S37" s="27">
+      <c r="R37" s="27">
+        <v>0</v>
+      </c>
+      <c r="S37" s="12">
         <v>0</v>
       </c>
       <c r="T37" s="12">
         <v>0</v>
       </c>
-      <c r="U37" s="12">
-        <v>0</v>
+      <c r="U37" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V37" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W37" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X37" s="13">
-        <f t="shared" si="0"/>
+      <c r="W37" s="13">
+        <f>K37/G37</f>
         <v>122.62500000000001</v>
       </c>
-      <c r="Z37">
-        <v>0</v>
+      <c r="Y37">
+        <v>0</v>
+      </c>
+      <c r="AA37">
+        <v>4749543701</v>
       </c>
       <c r="AB37">
-        <v>4749543701</v>
-      </c>
-      <c r="AC37">
         <v>1499248</v>
       </c>
     </row>
-    <row r="38" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B38" s="20"/>
       <c r="C38" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F38" s="12">
         <v>1</v>
@@ -3813,69 +3717,66 @@
       <c r="H38" s="13">
         <v>0</v>
       </c>
-      <c r="I38" s="13">
-        <v>0</v>
-      </c>
-      <c r="J38" s="25">
+      <c r="I38" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J38" s="14">
+        <v>0</v>
+      </c>
       <c r="K38" s="14">
-        <v>0</v>
-      </c>
-      <c r="L38" s="14">
         <v>5000</v>
       </c>
+      <c r="N38" s="14">
+        <v>0</v>
+      </c>
       <c r="O38" s="14">
-        <v>0</v>
-      </c>
-      <c r="P38" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q38" s="12">
-        <v>0</v>
-      </c>
-      <c r="R38" s="25">
+      <c r="P38" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S38" s="27">
+      <c r="R38" s="27">
+        <v>0</v>
+      </c>
+      <c r="S38" s="12">
         <v>0</v>
       </c>
       <c r="T38" s="12">
         <v>0</v>
       </c>
-      <c r="U38" s="12">
-        <v>0</v>
+      <c r="U38" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V38" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W38" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X38" s="13">
-        <f t="shared" si="0"/>
+      <c r="W38" s="13">
+        <f>K38/G38</f>
         <v>7.9345588235294118</v>
       </c>
-      <c r="Z38">
+      <c r="Y38">
         <v>1982</v>
       </c>
+      <c r="AA38">
+        <v>4710900101</v>
+      </c>
       <c r="AB38">
-        <v>4710900101</v>
-      </c>
-      <c r="AC38">
         <v>1539200001</v>
       </c>
     </row>
-    <row r="39" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B39" s="20"/>
       <c r="C39" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F39" s="12">
         <v>1</v>
@@ -3886,69 +3787,66 @@
       <c r="H39" s="13">
         <v>0</v>
       </c>
-      <c r="I39" s="13">
-        <v>0</v>
-      </c>
-      <c r="J39" s="25">
+      <c r="I39" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J39" s="14">
+        <v>0</v>
+      </c>
       <c r="K39" s="14">
-        <v>0</v>
-      </c>
-      <c r="L39" s="14">
         <v>5000</v>
       </c>
+      <c r="N39" s="14">
+        <v>0</v>
+      </c>
       <c r="O39" s="14">
-        <v>0</v>
-      </c>
-      <c r="P39" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q39" s="12">
-        <v>0</v>
-      </c>
-      <c r="R39" s="25">
+      <c r="P39" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S39" s="27">
+      <c r="R39" s="27">
+        <v>0</v>
+      </c>
+      <c r="S39" s="12">
         <v>0</v>
       </c>
       <c r="T39" s="12">
         <v>0</v>
       </c>
-      <c r="U39" s="12">
-        <v>0</v>
+      <c r="U39" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V39" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W39" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X39" s="13">
-        <f t="shared" si="0"/>
+      <c r="W39" s="13">
+        <f>K39/G39</f>
         <v>122.62500000000001</v>
       </c>
-      <c r="Z39">
-        <v>0</v>
+      <c r="Y39">
+        <v>0</v>
+      </c>
+      <c r="AA39">
+        <v>4691254801</v>
       </c>
       <c r="AB39">
-        <v>4691254801</v>
-      </c>
-      <c r="AC39">
         <v>1548666401</v>
       </c>
     </row>
-    <row r="40" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B40" s="20"/>
       <c r="C40" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F40" s="12">
         <v>1</v>
@@ -3959,69 +3857,66 @@
       <c r="H40" s="13">
         <v>0</v>
       </c>
-      <c r="I40" s="13">
-        <v>0</v>
-      </c>
-      <c r="J40" s="25">
+      <c r="I40" s="25">
         <v>2.5224658889183604E-4</v>
       </c>
+      <c r="J40" s="14">
+        <v>0</v>
+      </c>
       <c r="K40" s="14">
-        <v>0</v>
-      </c>
-      <c r="L40" s="14">
         <v>5000</v>
       </c>
+      <c r="N40" s="14">
+        <v>0</v>
+      </c>
       <c r="O40" s="14">
-        <v>0</v>
-      </c>
-      <c r="P40" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q40" s="12">
-        <v>0</v>
-      </c>
-      <c r="R40" s="25">
+      <c r="P40" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="S40" s="27">
+      <c r="R40" s="27">
+        <v>0</v>
+      </c>
+      <c r="S40" s="12">
         <v>0</v>
       </c>
       <c r="T40" s="12">
         <v>0</v>
       </c>
-      <c r="U40" s="12">
-        <v>0</v>
+      <c r="U40" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V40" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W40" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X40" s="13">
-        <f t="shared" si="0"/>
+      <c r="W40" s="13">
+        <f>K40/G40</f>
         <v>2.2708333333333335</v>
       </c>
-      <c r="Z40">
+      <c r="Y40">
         <v>1988</v>
       </c>
+      <c r="AA40">
+        <v>4720008473</v>
+      </c>
       <c r="AB40">
-        <v>4720008473</v>
-      </c>
-      <c r="AC40">
         <v>1444253532</v>
       </c>
     </row>
-    <row r="41" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B41" s="20"/>
       <c r="C41" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F41" s="12">
         <v>1</v>
@@ -4032,69 +3927,66 @@
       <c r="H41" s="13">
         <v>0</v>
       </c>
-      <c r="I41" s="13">
-        <v>0</v>
-      </c>
-      <c r="J41" s="25">
+      <c r="I41" s="25">
         <v>1.010294719501774E-3</v>
       </c>
+      <c r="J41" s="14">
+        <v>0</v>
+      </c>
       <c r="K41" s="14">
-        <v>0</v>
-      </c>
-      <c r="L41" s="14">
         <v>5000</v>
       </c>
+      <c r="N41" s="14">
+        <v>0</v>
+      </c>
       <c r="O41" s="14">
-        <v>0</v>
-      </c>
-      <c r="P41" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q41" s="12">
-        <v>0</v>
-      </c>
-      <c r="R41" s="25">
+      <c r="P41" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="25">
         <v>6.5669156767615311E-2</v>
       </c>
-      <c r="S41" s="27">
+      <c r="R41" s="27">
+        <v>0</v>
+      </c>
+      <c r="S41" s="12">
         <v>0</v>
       </c>
       <c r="T41" s="12">
         <v>0</v>
       </c>
-      <c r="U41" s="12">
-        <v>0</v>
+      <c r="U41" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V41" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W41" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X41" s="13">
-        <f t="shared" si="0"/>
+      <c r="W41" s="13">
+        <f>K41/G41</f>
         <v>3113.4487500000005</v>
       </c>
-      <c r="Z41">
+      <c r="Y41">
         <v>1984</v>
       </c>
+      <c r="AA41">
+        <v>47164754</v>
+      </c>
       <c r="AB41">
-        <v>47164754</v>
-      </c>
-      <c r="AC41">
         <v>1347057096</v>
       </c>
     </row>
-    <row r="42" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B42" s="20"/>
       <c r="C42" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F42" s="12">
         <v>1</v>
@@ -4105,69 +3997,66 @@
       <c r="H42" s="13">
         <v>0</v>
       </c>
-      <c r="I42" s="13">
-        <v>0</v>
-      </c>
-      <c r="J42" s="25">
+      <c r="I42" s="25">
         <v>8.4414548638109697E-5</v>
       </c>
+      <c r="J42" s="14">
+        <v>0</v>
+      </c>
       <c r="K42" s="14">
-        <v>0</v>
-      </c>
-      <c r="L42" s="14">
         <v>5000</v>
       </c>
+      <c r="N42" s="14">
+        <v>0</v>
+      </c>
       <c r="O42" s="14">
-        <v>0</v>
-      </c>
-      <c r="P42" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q42" s="12">
-        <v>0</v>
-      </c>
-      <c r="R42" s="25">
+      <c r="P42" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="25">
         <v>5.48694566147713E-3</v>
       </c>
-      <c r="S42" s="27">
+      <c r="R42" s="27">
+        <v>0</v>
+      </c>
+      <c r="S42" s="12">
         <v>0</v>
       </c>
       <c r="T42" s="12">
         <v>0</v>
       </c>
-      <c r="U42" s="12">
-        <v>0</v>
+      <c r="U42" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V42" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W42" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X42" s="13">
-        <f t="shared" si="0"/>
+      <c r="W42" s="13">
+        <f>K42/G42</f>
         <v>1003.4812499999999</v>
       </c>
-      <c r="Z42">
+      <c r="Y42">
         <v>1925</v>
       </c>
+      <c r="AA42">
+        <v>4701838219</v>
+      </c>
       <c r="AB42">
-        <v>4701838219</v>
-      </c>
-      <c r="AC42">
         <v>1515986506</v>
       </c>
     </row>
-    <row r="43" spans="2:29" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B43" s="20"/>
       <c r="C43" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F43" s="12">
         <v>1</v>
@@ -4178,56 +4067,53 @@
       <c r="H43" s="13">
         <v>0</v>
       </c>
-      <c r="I43" s="13">
-        <v>0</v>
-      </c>
-      <c r="J43" s="25">
+      <c r="I43" s="25">
         <v>9.4294189287256525E-5</v>
       </c>
+      <c r="J43" s="14">
+        <v>0</v>
+      </c>
       <c r="K43" s="14">
-        <v>0</v>
-      </c>
-      <c r="L43" s="14">
         <v>5000</v>
       </c>
+      <c r="N43" s="14">
+        <v>0</v>
+      </c>
       <c r="O43" s="14">
-        <v>0</v>
-      </c>
-      <c r="P43" s="14">
         <v>0.5</v>
       </c>
-      <c r="Q43" s="12">
-        <v>0</v>
-      </c>
-      <c r="R43" s="25">
+      <c r="P43" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="25">
         <v>6.1291223036716736E-3</v>
       </c>
-      <c r="S43" s="27">
+      <c r="R43" s="27">
+        <v>0</v>
+      </c>
+      <c r="S43" s="12">
         <v>0</v>
       </c>
       <c r="T43" s="12">
         <v>0</v>
       </c>
-      <c r="U43" s="12">
-        <v>0</v>
+      <c r="U43" s="14">
+        <v>99999999999</v>
       </c>
       <c r="V43" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W43" s="14">
-        <v>99999999999</v>
-      </c>
-      <c r="X43" s="13">
-        <f t="shared" si="0"/>
+      <c r="W43" s="13">
+        <f>K43/G43</f>
         <v>52.656617647058823</v>
       </c>
-      <c r="Z43">
+      <c r="Y43">
         <v>1985</v>
       </c>
+      <c r="AA43">
+        <v>4691099901</v>
+      </c>
       <c r="AB43">
-        <v>4691099901</v>
-      </c>
-      <c r="AC43">
         <v>1548600001</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement writing of LEGO Power_Inflow file
</commit_message>
<xml_diff>
--- a/data/hydroExample/Power_HydroAssets.xlsx
+++ b/data/hydroExample/Power_HydroAssets.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\hydroExample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B04642-23D8-4BAF-88E4-B5C363C48B89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{741FC6AC-CBFF-46C4-90E9-8E50BB9CADD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34230" yWindow="-21705" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Scenario_2014" sheetId="1" r:id="rId1"/>
+    <sheet name="Scenario_2016" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1650,7 +1650,7 @@
         <v>99999999999</v>
       </c>
       <c r="W8" s="13">
-        <f>K8/G8</f>
+        <f t="shared" ref="W8:W43" si="0">K8/G8</f>
         <v>9.7813715953307394</v>
       </c>
       <c r="X8" s="15"/>
@@ -1724,7 +1724,7 @@
         <v>99999999999</v>
       </c>
       <c r="W9" s="13">
-        <f>K9/G9</f>
+        <f t="shared" si="0"/>
         <v>3.7159090909090908</v>
       </c>
       <c r="Y9">
@@ -1794,7 +1794,7 @@
         <v>99999999999</v>
       </c>
       <c r="W10" s="13">
-        <f>K10/G10</f>
+        <f t="shared" si="0"/>
         <v>2.1639705882352942</v>
       </c>
       <c r="Y10">
@@ -1864,7 +1864,7 @@
         <v>99999999999</v>
       </c>
       <c r="W11" s="13">
-        <f>K11/G11</f>
+        <f t="shared" si="0"/>
         <v>1.9160156250000002</v>
       </c>
       <c r="Y11">
@@ -1934,7 +1934,7 @@
         <v>99999999999</v>
       </c>
       <c r="W12" s="13">
-        <f>K12/G12</f>
+        <f t="shared" si="0"/>
         <v>6.1312499999999996</v>
       </c>
       <c r="Y12">
@@ -2004,7 +2004,7 @@
         <v>99999999999</v>
       </c>
       <c r="W13" s="13">
-        <f>K13/G13</f>
+        <f t="shared" si="0"/>
         <v>2.5546875</v>
       </c>
       <c r="Y13">
@@ -2074,7 +2074,7 @@
         <v>99999999999</v>
       </c>
       <c r="W14" s="13">
-        <f>K14/G14</f>
+        <f t="shared" si="0"/>
         <v>75.326785714285705</v>
       </c>
       <c r="Y14">
@@ -2144,7 +2144,7 @@
         <v>99999999999</v>
       </c>
       <c r="W15" s="13">
-        <f>K15/G15</f>
+        <f t="shared" si="0"/>
         <v>72.284210526315803</v>
       </c>
       <c r="Y15">
@@ -2214,7 +2214,7 @@
         <v>99999999999</v>
       </c>
       <c r="W16" s="13">
-        <f>K16/G16</f>
+        <f t="shared" si="0"/>
         <v>82.333928571428558</v>
       </c>
       <c r="Y16">
@@ -2284,7 +2284,7 @@
         <v>99999999999</v>
       </c>
       <c r="W17" s="13">
-        <f>K17/G17</f>
+        <f t="shared" si="0"/>
         <v>72.46022727272728</v>
       </c>
       <c r="Y17">
@@ -2354,7 +2354,7 @@
         <v>99999999999</v>
       </c>
       <c r="W18" s="13">
-        <f>K18/G18</f>
+        <f t="shared" si="0"/>
         <v>74.341406250000006</v>
       </c>
       <c r="Y18">
@@ -2424,7 +2424,7 @@
         <v>99999999999</v>
       </c>
       <c r="W19" s="13">
-        <f>K19/G19</f>
+        <f t="shared" si="0"/>
         <v>5.109375</v>
       </c>
       <c r="Y19">
@@ -2494,7 +2494,7 @@
         <v>99999999999</v>
       </c>
       <c r="W20" s="13">
-        <f>K20/G20</f>
+        <f t="shared" si="0"/>
         <v>176862.98076923078</v>
       </c>
       <c r="Y20">
@@ -2564,7 +2564,7 @@
         <v>99999999999</v>
       </c>
       <c r="W21" s="13">
-        <f>K21/G21</f>
+        <f t="shared" si="0"/>
         <v>72.284210526315803</v>
       </c>
       <c r="Y21">
@@ -2634,7 +2634,7 @@
         <v>99999999999</v>
       </c>
       <c r="W22" s="13">
-        <f>K22/G22</f>
+        <f t="shared" si="0"/>
         <v>58.587499999999999</v>
       </c>
       <c r="Y22">
@@ -2704,7 +2704,7 @@
         <v>99999999999</v>
       </c>
       <c r="W23" s="13">
-        <f>K23/G23</f>
+        <f t="shared" si="0"/>
         <v>6.1919554455445542</v>
       </c>
       <c r="Y23">
@@ -2774,7 +2774,7 @@
         <v>99999999999</v>
       </c>
       <c r="W24" s="13">
-        <f>K24/G24</f>
+        <f t="shared" si="0"/>
         <v>9.81</v>
       </c>
       <c r="Y24">
@@ -2844,7 +2844,7 @@
         <v>99999999999</v>
       </c>
       <c r="W25" s="13">
-        <f>K25/G25</f>
+        <f t="shared" si="0"/>
         <v>7.5461538461538469</v>
       </c>
       <c r="Y25">
@@ -2914,7 +2914,7 @@
         <v>99999999999</v>
       </c>
       <c r="W26" s="13">
-        <f>K26/G26</f>
+        <f t="shared" si="0"/>
         <v>8174.9999999999991</v>
       </c>
       <c r="Y26">
@@ -2984,7 +2984,7 @@
         <v>99999999999</v>
       </c>
       <c r="W27" s="13">
-        <f>K27/G27</f>
+        <f t="shared" si="0"/>
         <v>8.4894230769230763</v>
       </c>
       <c r="Y27">
@@ -3054,7 +3054,7 @@
         <v>99999999999</v>
       </c>
       <c r="W28" s="13">
-        <f>K28/G28</f>
+        <f t="shared" si="0"/>
         <v>5.7034883720930241E-2</v>
       </c>
       <c r="Y28">
@@ -3124,7 +3124,7 @@
         <v>99999999999</v>
       </c>
       <c r="W29" s="13">
-        <f>K29/G29</f>
+        <f t="shared" si="0"/>
         <v>61.312500000000007</v>
       </c>
       <c r="Y29">
@@ -3194,7 +3194,7 @@
         <v>99999999999</v>
       </c>
       <c r="W30" s="13">
-        <f>K30/G30</f>
+        <f t="shared" si="0"/>
         <v>7.8830357142857137</v>
       </c>
       <c r="Y30">
@@ -3264,7 +3264,7 @@
         <v>99999999999</v>
       </c>
       <c r="W31" s="13">
-        <f>K31/G31</f>
+        <f t="shared" si="0"/>
         <v>122.62500000000001</v>
       </c>
       <c r="Y31">
@@ -3334,7 +3334,7 @@
         <v>99999999999</v>
       </c>
       <c r="W32" s="13">
-        <f>K32/G32</f>
+        <f t="shared" si="0"/>
         <v>65.085576923076914</v>
       </c>
       <c r="Y32">
@@ -3404,7 +3404,7 @@
         <v>99999999999</v>
       </c>
       <c r="W33" s="13">
-        <f>K33/G33</f>
+        <f t="shared" si="0"/>
         <v>173.71875</v>
       </c>
       <c r="Y33">
@@ -3474,7 +3474,7 @@
         <v>99999999999</v>
       </c>
       <c r="W34" s="13">
-        <f>K34/G34</f>
+        <f t="shared" si="0"/>
         <v>7.6640625000000009</v>
       </c>
       <c r="Y34">
@@ -3544,7 +3544,7 @@
         <v>99999999999</v>
       </c>
       <c r="W35" s="13">
-        <f>K35/G35</f>
+        <f t="shared" si="0"/>
         <v>10.21875</v>
       </c>
       <c r="Y35">
@@ -3614,7 +3614,7 @@
         <v>99999999999</v>
       </c>
       <c r="W36" s="13">
-        <f>K36/G36</f>
+        <f t="shared" si="0"/>
         <v>122.62500000000001</v>
       </c>
       <c r="Y36">
@@ -3684,7 +3684,7 @@
         <v>99999999999</v>
       </c>
       <c r="W37" s="13">
-        <f>K37/G37</f>
+        <f t="shared" si="0"/>
         <v>122.62500000000001</v>
       </c>
       <c r="Y37">
@@ -3754,7 +3754,7 @@
         <v>99999999999</v>
       </c>
       <c r="W38" s="13">
-        <f>K38/G38</f>
+        <f t="shared" si="0"/>
         <v>7.9345588235294118</v>
       </c>
       <c r="Y38">
@@ -3824,7 +3824,7 @@
         <v>99999999999</v>
       </c>
       <c r="W39" s="13">
-        <f>K39/G39</f>
+        <f t="shared" si="0"/>
         <v>122.62500000000001</v>
       </c>
       <c r="Y39">
@@ -3894,7 +3894,7 @@
         <v>99999999999</v>
       </c>
       <c r="W40" s="13">
-        <f>K40/G40</f>
+        <f t="shared" si="0"/>
         <v>2.2708333333333335</v>
       </c>
       <c r="Y40">
@@ -3964,7 +3964,7 @@
         <v>99999999999</v>
       </c>
       <c r="W41" s="13">
-        <f>K41/G41</f>
+        <f t="shared" si="0"/>
         <v>3113.4487500000005</v>
       </c>
       <c r="Y41">
@@ -4034,7 +4034,7 @@
         <v>99999999999</v>
       </c>
       <c r="W42" s="13">
-        <f>K42/G42</f>
+        <f t="shared" si="0"/>
         <v>1003.4812499999999</v>
       </c>
       <c r="Y42">
@@ -4104,7 +4104,7 @@
         <v>99999999999</v>
       </c>
       <c r="W43" s="13">
-        <f>K43/G43</f>
+        <f t="shared" si="0"/>
         <v>52.656617647058823</v>
       </c>
       <c r="Y43">

</xml_diff>

<commit_message>
Update HydroAssets and Inflows_WaterAmount to fix data errors
</commit_message>
<xml_diff>
--- a/data/hydroExample/Power_HydroAssets.xlsx
+++ b/data/hydroExample/Power_HydroAssets.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\hydroExample\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth\Dropbox\Privat\Masterarbeit_2025\Old_calc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{741FC6AC-CBFF-46C4-90E9-8E50BB9CADD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAF0EB8E-050E-41A5-A4C2-B9211D80F72A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34230" yWindow="-21705" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Scenario_2016" sheetId="1" r:id="rId1"/>
+    <sheet name="Scenario_2014" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="138">
   <si>
     <t>Format:</t>
   </si>
@@ -150,6 +150,12 @@
     <t>ExisUnits</t>
   </si>
   <si>
+    <t>MaxProd</t>
+  </si>
+  <si>
+    <t>MinProd</t>
+  </si>
+  <si>
     <t>Qmax</t>
   </si>
   <si>
@@ -255,6 +261,15 @@
     <t>Number of existing units</t>
   </si>
   <si>
+    <t>Maximum active power output of the unit</t>
+  </si>
+  <si>
+    <t>Minimum active power output of the unit</t>
+  </si>
+  <si>
+    <t>Maximum consumption of the unit</t>
+  </si>
+  <si>
     <t>Efficiency of discharging the storage unit</t>
   </si>
   <si>
@@ -378,6 +393,9 @@
     <t>PowerFactorPump</t>
   </si>
   <si>
+    <t>MaxPump</t>
+  </si>
+  <si>
     <t>Maximum Pumping</t>
   </si>
   <si>
@@ -523,18 +541,6 @@
   </si>
   <si>
     <t>190 Mellach und Kuehlwasserturbine-KW</t>
-  </si>
-  <si>
-    <t>MaxProdWater</t>
-  </si>
-  <si>
-    <t>Maximum water intake of the unit</t>
-  </si>
-  <si>
-    <t>Maximum water consumption of the unit</t>
-  </si>
-  <si>
-    <t>MaxPumpWater</t>
   </si>
 </sst>
 </file>
@@ -550,7 +556,7 @@
     <numFmt numFmtId="168" formatCode="0.00000"/>
     <numFmt numFmtId="169" formatCode="0.0000000000"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -610,18 +616,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
       <name val="Aptos"/>
       <family val="2"/>
     </font>
@@ -695,7 +689,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -764,14 +758,10 @@
     <xf numFmtId="2" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Komma" xfId="1" builtinId="3"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1074,32 +1064,32 @@
   <sheetPr>
     <tabColor rgb="FF008080"/>
   </sheetPr>
-  <dimension ref="A1:AD43"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AE43"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" customWidth="1"/>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
     <col min="3" max="3" width="29.85546875" customWidth="1"/>
-    <col min="4" max="8" width="15.7109375" customWidth="1"/>
-    <col min="9" max="11" width="21.7109375" customWidth="1"/>
-    <col min="12" max="15" width="15.7109375" customWidth="1"/>
-    <col min="16" max="16" width="20.7109375" customWidth="1"/>
-    <col min="17" max="17" width="20.42578125" customWidth="1"/>
-    <col min="18" max="18" width="20.5703125" customWidth="1"/>
-    <col min="19" max="20" width="15.7109375" customWidth="1"/>
-    <col min="21" max="22" width="20.7109375" customWidth="1"/>
-    <col min="23" max="23" width="22.7109375" customWidth="1"/>
-    <col min="24" max="24" width="15.7109375" customWidth="1"/>
-    <col min="25" max="26" width="20.140625" customWidth="1"/>
-    <col min="27" max="27" width="20.42578125" customWidth="1"/>
-    <col min="28" max="28" width="19.42578125" customWidth="1"/>
-    <col min="29" max="30" width="24.5703125" customWidth="1"/>
+    <col min="4" max="9" width="15.7109375" customWidth="1"/>
+    <col min="10" max="12" width="21.7109375" customWidth="1"/>
+    <col min="13" max="16" width="15.7109375" customWidth="1"/>
+    <col min="17" max="17" width="20.7109375" customWidth="1"/>
+    <col min="18" max="18" width="20.42578125" customWidth="1"/>
+    <col min="19" max="19" width="20.5703125" customWidth="1"/>
+    <col min="20" max="21" width="15.7109375" customWidth="1"/>
+    <col min="22" max="23" width="20.7109375" customWidth="1"/>
+    <col min="24" max="24" width="22.7109375" customWidth="1"/>
+    <col min="25" max="25" width="15.7109375" customWidth="1"/>
+    <col min="26" max="27" width="20.140625" customWidth="1"/>
+    <col min="28" max="28" width="20.42578125" customWidth="1"/>
+    <col min="29" max="29" width="19.42578125" customWidth="1"/>
+    <col min="30" max="31" width="24.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:31" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1129,16 +1119,17 @@
       <c r="AB1" s="1"/>
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
@@ -1158,2962 +1149,3084 @@
         <v>6</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>132</v>
+        <v>7</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="K3" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="S3" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="L3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="P3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>12</v>
-      </c>
       <c r="T3" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Y3" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Z3" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="AA3" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="AB3" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AC3" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="AD3" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="AE3" s="5" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="28" t="s">
-        <v>132</v>
-      </c>
-      <c r="H4" s="28" t="s">
-        <v>135</v>
+      <c r="G4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>8</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>7</v>
+        <v>99</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="Q4" s="6" t="s">
-        <v>85</v>
+        <v>13</v>
       </c>
       <c r="R4" s="6" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="S4" s="6" t="s">
-        <v>12</v>
+        <v>92</v>
       </c>
       <c r="T4" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="U4" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="V4" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="W4" s="6" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="X4" s="6" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="Y4" s="6" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="Z4" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="AA4" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="AB4" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AC4" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="AD4" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="AE4" s="6" t="s">
+        <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:30" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G5" s="29" t="s">
-        <v>133</v>
-      </c>
-      <c r="H5" s="29" t="s">
-        <v>134</v>
+        <v>43</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>45</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>94</v>
+        <v>48</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="O5" s="7" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="Q5" s="7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="R5" s="7" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="S5" s="7" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="T5" s="7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="U5" s="7" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="V5" s="7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="W5" s="7" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="X5" s="7" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="Y5" s="7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="Z5" s="7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="AA5" s="7" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="AB5" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AC5" s="7" t="s">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="AD5" s="7" t="s">
-        <v>59</v>
+        <v>63</v>
+      </c>
+      <c r="AE5" s="7" t="s">
+        <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:30" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8" t="s">
-        <v>62</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="L6" s="8"/>
       <c r="M6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="N6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="O6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="P6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="Q6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="R6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="S6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="T6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="U6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="V6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="W6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="X6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="Y6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="Z6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="AA6" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="AB6" s="8" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="AC6" s="8" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="AD6" s="8" t="s">
-        <v>62</v>
+        <v>67</v>
+      </c>
+      <c r="AE6" s="8" t="s">
+        <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" s="9"/>
       <c r="B7" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="K7" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="L7" s="9" t="s">
-        <v>69</v>
+        <v>97</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="L7" s="26" t="s">
+        <v>95</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="N7" s="9" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="O7" s="9" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="P7" s="9" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="Q7" s="9" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="R7" s="9" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="S7" s="9" t="s">
-        <v>70</v>
+        <v>96</v>
       </c>
       <c r="T7" s="9" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="U7" s="9" t="s">
         <v>72</v>
       </c>
       <c r="V7" s="9" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="W7" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="X7" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="Y7" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="X7" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="Y7" s="9" t="s">
-        <v>74</v>
-      </c>
       <c r="Z7" s="9" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AA7" s="9" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="AB7" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="AC7" s="9" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AD7" s="9" t="s">
-        <v>77</v>
+        <v>81</v>
+      </c>
+      <c r="AE7" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="20"/>
       <c r="C8" s="18" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F8" s="12">
         <v>1</v>
       </c>
       <c r="G8" s="21">
-        <v>511.17575395937445</v>
+        <v>517142.78610676009</v>
       </c>
       <c r="H8" s="13">
         <v>0</v>
       </c>
-      <c r="I8" s="24">
-        <v>1.3833147724009441E-3</v>
-      </c>
-      <c r="J8" s="14">
-        <v>0</v>
+      <c r="I8" s="13">
+        <v>0</v>
+      </c>
+      <c r="J8" s="24">
+        <v>5.0276250000000002E-5</v>
       </c>
       <c r="K8" s="14">
+        <v>0</v>
+      </c>
+      <c r="L8" s="14">
         <v>5000</v>
       </c>
-      <c r="L8" s="13"/>
-      <c r="M8" s="13"/>
-      <c r="N8" s="14">
-        <v>0</v>
-      </c>
+      <c r="N8" s="13"/>
       <c r="O8" s="14">
+        <v>0</v>
+      </c>
+      <c r="P8" s="14">
         <v>0.5</v>
       </c>
-      <c r="P8" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="14">
+      <c r="Q8" s="12">
+        <v>0</v>
+      </c>
+      <c r="R8" s="14">
         <v>8.9915460206061365E-2</v>
       </c>
-      <c r="R8" s="14">
-        <v>0</v>
-      </c>
-      <c r="S8" s="12">
+      <c r="S8" s="14">
         <v>0</v>
       </c>
       <c r="T8" s="12">
         <v>0</v>
       </c>
-      <c r="U8" s="14">
-        <v>99999999999</v>
+      <c r="U8" s="12">
+        <v>0</v>
       </c>
       <c r="V8" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W8" s="13">
-        <f t="shared" ref="W8:W43" si="0">K8/G8</f>
-        <v>9.7813715953307394</v>
-      </c>
-      <c r="X8" s="15"/>
-      <c r="Y8" s="12">
+      <c r="W8" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X8" s="13">
+        <f>L8/G8</f>
+        <v>9.668509615384617E-3</v>
+      </c>
+      <c r="Y8" s="15"/>
+      <c r="Z8" s="12">
         <v>1960</v>
       </c>
-      <c r="Z8" s="12"/>
-      <c r="AA8" s="16">
+      <c r="AA8" s="12"/>
+      <c r="AB8" s="16">
         <v>4676666671</v>
       </c>
-      <c r="AB8" s="16">
+      <c r="AC8" s="16">
         <v>1555000001</v>
       </c>
-      <c r="AC8" s="17"/>
       <c r="AD8" s="17"/>
+      <c r="AE8" s="17"/>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B9" s="20"/>
       <c r="C9" s="19" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F9" s="12">
         <v>1</v>
       </c>
       <c r="G9" s="25">
-        <v>1345.565749235474</v>
+        <v>13455657.492354739</v>
       </c>
       <c r="H9" s="13">
         <v>0</v>
       </c>
-      <c r="I9" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J9" s="14">
-        <v>0</v>
+      <c r="I9" s="13">
+        <v>0</v>
+      </c>
+      <c r="J9" s="25">
+        <v>2.4524999999999998E-6</v>
       </c>
       <c r="K9" s="14">
+        <v>0</v>
+      </c>
+      <c r="L9" s="14">
         <v>5000</v>
       </c>
-      <c r="N9" s="14">
-        <v>0</v>
-      </c>
       <c r="O9" s="14">
+        <v>0</v>
+      </c>
+      <c r="P9" s="14">
         <v>0.5</v>
       </c>
-      <c r="P9" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="25">
+      <c r="Q9" s="12">
+        <v>0</v>
+      </c>
+      <c r="R9" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R9" s="27">
-        <v>0</v>
-      </c>
-      <c r="S9" s="12">
+      <c r="S9" s="27">
         <v>0</v>
       </c>
       <c r="T9" s="12">
         <v>0</v>
       </c>
-      <c r="U9" s="14">
-        <v>99999999999</v>
+      <c r="U9" s="12">
+        <v>0</v>
       </c>
       <c r="V9" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W9" s="13">
-        <f t="shared" si="0"/>
-        <v>3.7159090909090908</v>
-      </c>
-      <c r="Y9">
-        <v>0</v>
-      </c>
-      <c r="AA9">
+      <c r="W9" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X9" s="13">
+        <f t="shared" ref="X9:X43" si="0">L9/G9</f>
+        <v>3.7159090909090909E-4</v>
+      </c>
+      <c r="Z9">
+        <v>0</v>
+      </c>
+      <c r="AB9">
         <v>4704999901</v>
       </c>
-      <c r="AB9">
+      <c r="AC9">
         <v>1519400001</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B10" s="20"/>
       <c r="C10" s="19" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F10" s="12">
         <v>1</v>
       </c>
       <c r="G10" s="25">
-        <v>2310.567448182127</v>
+        <v>23105674.481821269</v>
       </c>
       <c r="H10" s="13">
         <v>0</v>
       </c>
-      <c r="I10" s="25">
-        <v>1.7219053916301622E-4</v>
-      </c>
-      <c r="J10" s="14">
-        <v>0</v>
+      <c r="I10" s="13">
+        <v>0</v>
+      </c>
+      <c r="J10" s="25">
+        <v>1.4715000000000002E-6</v>
       </c>
       <c r="K10" s="14">
+        <v>0</v>
+      </c>
+      <c r="L10" s="14">
         <v>5000</v>
       </c>
-      <c r="N10" s="14">
-        <v>0</v>
-      </c>
       <c r="O10" s="14">
+        <v>0</v>
+      </c>
+      <c r="P10" s="14">
         <v>0.5</v>
       </c>
-      <c r="P10" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="25">
+      <c r="Q10" s="12">
+        <v>0</v>
+      </c>
+      <c r="R10" s="25">
         <v>1.1192385045596056E-2</v>
       </c>
-      <c r="R10" s="25">
-        <v>0.32026898653096453</v>
-      </c>
-      <c r="S10" s="12">
+      <c r="S10" s="27">
         <v>0</v>
       </c>
       <c r="T10" s="12">
         <v>0</v>
       </c>
-      <c r="U10" s="14">
-        <v>99999999999</v>
+      <c r="U10" s="12">
+        <v>0</v>
       </c>
       <c r="V10" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W10" s="13">
+      <c r="W10" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X10" s="13">
         <f t="shared" si="0"/>
-        <v>2.1639705882352942</v>
-      </c>
-      <c r="Y10">
+        <v>2.1639705882352944E-4</v>
+      </c>
+      <c r="Z10">
         <v>1982</v>
       </c>
-      <c r="AA10">
+      <c r="AB10">
         <v>4710768617</v>
       </c>
-      <c r="AB10">
+      <c r="AC10">
         <v>1406553496</v>
       </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B11" s="20"/>
       <c r="C11" s="19" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F11" s="12">
         <v>1</v>
       </c>
       <c r="G11" s="25">
-        <v>2609.5820591233432</v>
+        <v>6523955.147808359</v>
       </c>
       <c r="H11" s="13">
         <v>0</v>
       </c>
-      <c r="I11" s="25">
-        <v>1.3639768598388177E-4</v>
-      </c>
-      <c r="J11" s="14">
-        <v>0</v>
+      <c r="I11" s="13">
+        <v>0</v>
+      </c>
+      <c r="J11" s="25">
+        <v>2.4524999999999998E-6</v>
       </c>
       <c r="K11" s="14">
+        <v>0</v>
+      </c>
+      <c r="L11" s="14">
         <v>5000</v>
       </c>
-      <c r="N11" s="14">
-        <v>0</v>
-      </c>
       <c r="O11" s="14">
+        <v>0</v>
+      </c>
+      <c r="P11" s="14">
         <v>0.5</v>
       </c>
-      <c r="P11" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="25">
+      <c r="Q11" s="12">
+        <v>0</v>
+      </c>
+      <c r="R11" s="25">
         <v>8.865849588952316E-3</v>
       </c>
-      <c r="R11" s="27">
-        <v>0</v>
-      </c>
-      <c r="S11" s="12">
+      <c r="S11" s="27">
         <v>0</v>
       </c>
       <c r="T11" s="12">
         <v>0</v>
       </c>
-      <c r="U11" s="14">
-        <v>99999999999</v>
+      <c r="U11" s="12">
+        <v>0</v>
       </c>
       <c r="V11" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W11" s="13">
+      <c r="W11" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X11" s="13">
         <f t="shared" si="0"/>
-        <v>1.9160156250000002</v>
-      </c>
-      <c r="Y11">
+        <v>7.6640624999999994E-4</v>
+      </c>
+      <c r="Z11">
         <v>1949</v>
       </c>
-      <c r="AA11">
+      <c r="AB11">
         <v>4741000001</v>
       </c>
-      <c r="AB11">
+      <c r="AC11">
         <v>15214</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B12" s="20"/>
       <c r="C12" s="19" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F12" s="12">
         <v>1</v>
       </c>
       <c r="G12" s="25">
-        <v>815.49439347604493</v>
+        <v>8154943.9347604485</v>
       </c>
       <c r="H12" s="13">
         <v>0</v>
       </c>
-      <c r="I12" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J12" s="14">
-        <v>0</v>
+      <c r="I12" s="13">
+        <v>0</v>
+      </c>
+      <c r="J12" s="25">
+        <v>2.6977499999999997E-6</v>
       </c>
       <c r="K12" s="14">
+        <v>0</v>
+      </c>
+      <c r="L12" s="14">
         <v>5000</v>
       </c>
-      <c r="N12" s="14">
-        <v>0</v>
-      </c>
       <c r="O12" s="14">
+        <v>0</v>
+      </c>
+      <c r="P12" s="14">
         <v>0.5</v>
       </c>
-      <c r="P12" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="25">
+      <c r="Q12" s="12">
+        <v>0</v>
+      </c>
+      <c r="R12" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R12" s="27">
-        <v>0</v>
-      </c>
-      <c r="S12" s="12">
+      <c r="S12" s="27">
         <v>0</v>
       </c>
       <c r="T12" s="12">
         <v>0</v>
       </c>
-      <c r="U12" s="14">
-        <v>99999999999</v>
+      <c r="U12" s="12">
+        <v>0</v>
       </c>
       <c r="V12" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W12" s="13">
+      <c r="W12" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X12" s="13">
         <f t="shared" si="0"/>
-        <v>6.1312499999999996</v>
-      </c>
-      <c r="Y12">
+        <v>6.1312499999999995E-4</v>
+      </c>
+      <c r="Z12">
         <v>1994</v>
       </c>
-      <c r="AA12">
+      <c r="AB12">
         <v>4717426321</v>
       </c>
-      <c r="AB12">
+      <c r="AC12">
         <v>1472277926</v>
       </c>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B13" s="20"/>
       <c r="C13" s="19" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F13" s="12">
         <v>1</v>
       </c>
       <c r="G13" s="25">
-        <v>1957.1865443425077</v>
+        <v>19571865.443425078</v>
       </c>
       <c r="H13" s="13">
         <v>0</v>
       </c>
-      <c r="I13" s="25">
-        <v>9.3643427926305622E-5</v>
-      </c>
-      <c r="J13" s="14">
-        <v>0</v>
+      <c r="I13" s="13">
+        <v>0</v>
+      </c>
+      <c r="J13" s="25">
+        <v>6.1312499999999995E-7</v>
       </c>
       <c r="K13" s="14">
+        <v>0</v>
+      </c>
+      <c r="L13" s="14">
         <v>5000</v>
       </c>
-      <c r="N13" s="14">
-        <v>0</v>
-      </c>
       <c r="O13" s="14">
+        <v>0</v>
+      </c>
+      <c r="P13" s="14">
         <v>0.5</v>
       </c>
-      <c r="P13" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="25">
+      <c r="Q13" s="12">
+        <v>0</v>
+      </c>
+      <c r="R13" s="25">
         <v>6.0868228152098653E-3</v>
       </c>
-      <c r="R13" s="27">
-        <v>0</v>
-      </c>
-      <c r="S13" s="12">
+      <c r="S13" s="27">
         <v>0</v>
       </c>
       <c r="T13" s="12">
         <v>0</v>
       </c>
-      <c r="U13" s="14">
-        <v>99999999999</v>
+      <c r="U13" s="12">
+        <v>0</v>
       </c>
       <c r="V13" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W13" s="13">
+      <c r="W13" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X13" s="13">
         <f t="shared" si="0"/>
-        <v>2.5546875</v>
-      </c>
-      <c r="Y13">
+        <v>2.5546875E-4</v>
+      </c>
+      <c r="Z13">
         <v>1998</v>
       </c>
-      <c r="AA13">
+      <c r="AB13">
         <v>4718651301</v>
       </c>
-      <c r="AB13">
+      <c r="AC13">
         <v>1533601401</v>
       </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B14" s="20"/>
       <c r="C14" s="19" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F14" s="12">
         <v>1</v>
       </c>
       <c r="G14" s="25">
-        <v>66.377450631771097</v>
+        <v>663774.50631771085</v>
       </c>
       <c r="H14" s="13">
         <v>0</v>
       </c>
-      <c r="I14" s="25">
-        <v>7.2708447849138697E-5</v>
-      </c>
-      <c r="J14" s="14">
-        <v>0</v>
+      <c r="I14" s="13">
+        <v>0</v>
+      </c>
+      <c r="J14" s="25">
+        <v>2.1091500000000003E-5</v>
       </c>
       <c r="K14" s="14">
+        <v>0</v>
+      </c>
+      <c r="L14" s="14">
         <v>5000</v>
       </c>
-      <c r="N14" s="14">
-        <v>0</v>
-      </c>
       <c r="O14" s="14">
+        <v>0</v>
+      </c>
+      <c r="P14" s="14">
         <v>0.5</v>
       </c>
-      <c r="P14" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="25">
+      <c r="Q14" s="12">
+        <v>0</v>
+      </c>
+      <c r="R14" s="25">
         <v>4.7260491101940149E-3</v>
       </c>
-      <c r="R14" s="27">
-        <v>0</v>
-      </c>
-      <c r="S14" s="12">
+      <c r="S14" s="27">
         <v>0</v>
       </c>
       <c r="T14" s="12">
         <v>0</v>
       </c>
-      <c r="U14" s="14">
-        <v>99999999999</v>
+      <c r="U14" s="12">
+        <v>0</v>
       </c>
       <c r="V14" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W14" s="13">
+      <c r="W14" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X14" s="13">
         <f t="shared" si="0"/>
-        <v>75.326785714285705</v>
-      </c>
-      <c r="Y14">
+        <v>7.5326785714285721E-3</v>
+      </c>
+      <c r="Z14">
         <v>1974</v>
       </c>
-      <c r="AA14">
+      <c r="AB14">
         <v>46785118</v>
       </c>
-      <c r="AB14">
+      <c r="AC14">
         <v>1558555701</v>
       </c>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B15" s="20"/>
       <c r="C15" s="19" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F15" s="12">
         <v>1</v>
       </c>
       <c r="G15" s="25">
-        <v>69.171399446628797</v>
+        <v>691713.99446628802</v>
       </c>
       <c r="H15" s="13">
         <v>0</v>
       </c>
-      <c r="I15" s="25">
-        <v>1.12898177984472E-4</v>
-      </c>
-      <c r="J15" s="14">
-        <v>0</v>
+      <c r="I15" s="13">
+        <v>0</v>
+      </c>
+      <c r="J15" s="25">
+        <v>2.7468000000000002E-5</v>
       </c>
       <c r="K15" s="14">
+        <v>0</v>
+      </c>
+      <c r="L15" s="14">
         <v>5000</v>
       </c>
-      <c r="N15" s="14">
-        <v>0</v>
-      </c>
       <c r="O15" s="14">
+        <v>0</v>
+      </c>
+      <c r="P15" s="14">
         <v>0.5</v>
       </c>
-      <c r="P15" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="25">
+      <c r="Q15" s="12">
+        <v>0</v>
+      </c>
+      <c r="R15" s="25">
         <v>7.3383815689906798E-3</v>
       </c>
-      <c r="R15" s="27">
-        <v>0</v>
-      </c>
-      <c r="S15" s="12">
+      <c r="S15" s="27">
         <v>0</v>
       </c>
       <c r="T15" s="12">
         <v>0</v>
       </c>
-      <c r="U15" s="14">
-        <v>99999999999</v>
+      <c r="U15" s="12">
+        <v>0</v>
       </c>
       <c r="V15" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W15" s="13">
+      <c r="W15" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X15" s="13">
         <f t="shared" si="0"/>
-        <v>72.284210526315803</v>
-      </c>
-      <c r="Y15">
+        <v>7.2284210526315793E-3</v>
+      </c>
+      <c r="Z15">
         <v>2011</v>
       </c>
-      <c r="AA15">
+      <c r="AB15">
         <v>4699784101</v>
       </c>
-      <c r="AB15">
+      <c r="AC15">
         <v>1546751901</v>
       </c>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B16" s="20"/>
       <c r="C16" s="19" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F16" s="12">
         <v>1</v>
       </c>
       <c r="G16" s="25">
-        <v>60.728305897152282</v>
+        <v>607283.05897152273</v>
       </c>
       <c r="H16" s="13">
         <v>0</v>
       </c>
-      <c r="I16" s="25">
-        <v>1.9032505466392189E-5</v>
-      </c>
-      <c r="J16" s="14">
-        <v>0</v>
+      <c r="I16" s="13">
+        <v>0</v>
+      </c>
+      <c r="J16" s="25">
+        <v>2.3053500000000002E-5</v>
       </c>
       <c r="K16" s="14">
+        <v>0</v>
+      </c>
+      <c r="L16" s="14">
         <v>5000</v>
       </c>
-      <c r="N16" s="14">
-        <v>0</v>
-      </c>
       <c r="O16" s="14">
+        <v>0</v>
+      </c>
+      <c r="P16" s="14">
         <v>0.5</v>
       </c>
-      <c r="P16" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="25">
+      <c r="Q16" s="12">
+        <v>0</v>
+      </c>
+      <c r="R16" s="25">
         <v>1.2371128553154923E-3</v>
       </c>
-      <c r="R16" s="27">
-        <v>0</v>
-      </c>
-      <c r="S16" s="12">
+      <c r="S16" s="27">
         <v>0</v>
       </c>
       <c r="T16" s="12">
         <v>0</v>
       </c>
-      <c r="U16" s="14">
-        <v>99999999999</v>
+      <c r="U16" s="12">
+        <v>0</v>
       </c>
       <c r="V16" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W16" s="13">
+      <c r="W16" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X16" s="13">
         <f t="shared" si="0"/>
-        <v>82.333928571428558</v>
-      </c>
-      <c r="Y16">
+        <v>8.2333928571428575E-3</v>
+      </c>
+      <c r="Z16">
         <v>1964</v>
       </c>
-      <c r="AA16">
+      <c r="AB16">
         <v>4682809068</v>
       </c>
-      <c r="AB16">
+      <c r="AC16">
         <v>1556616553</v>
       </c>
     </row>
-    <row r="17" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B17" s="20"/>
       <c r="C17" s="19" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F17" s="12">
         <v>1</v>
       </c>
       <c r="G17" s="25">
-        <v>69.003371755665327</v>
+        <v>690033.71755665331</v>
       </c>
       <c r="H17" s="13">
         <v>0</v>
       </c>
-      <c r="I17" s="25">
-        <v>5.9495468904415532E-5</v>
-      </c>
-      <c r="J17" s="14">
-        <v>0</v>
+      <c r="I17" s="13">
+        <v>0</v>
+      </c>
+      <c r="J17" s="25">
+        <v>1.5941249999999999E-5</v>
       </c>
       <c r="K17" s="14">
+        <v>0</v>
+      </c>
+      <c r="L17" s="14">
         <v>5000</v>
       </c>
-      <c r="N17" s="14">
-        <v>0</v>
-      </c>
       <c r="O17" s="14">
+        <v>0</v>
+      </c>
+      <c r="P17" s="14">
         <v>0.5</v>
       </c>
-      <c r="P17" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="25">
+      <c r="Q17" s="12">
+        <v>0</v>
+      </c>
+      <c r="R17" s="25">
         <v>3.8672054787870095E-3</v>
       </c>
-      <c r="R17" s="27">
-        <v>0</v>
-      </c>
-      <c r="S17" s="12">
+      <c r="S17" s="27">
         <v>0</v>
       </c>
       <c r="T17" s="12">
         <v>0</v>
       </c>
-      <c r="U17" s="14">
-        <v>99999999999</v>
+      <c r="U17" s="12">
+        <v>0</v>
       </c>
       <c r="V17" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W17" s="13">
+      <c r="W17" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X17" s="13">
         <f t="shared" si="0"/>
-        <v>72.46022727272728</v>
-      </c>
-      <c r="Y17">
+        <v>7.2460227272727277E-3</v>
+      </c>
+      <c r="Z17">
         <v>2024</v>
       </c>
-      <c r="AA17">
+      <c r="AB17">
         <v>4713909101</v>
       </c>
-      <c r="AB17">
+      <c r="AC17">
         <v>1532804601</v>
       </c>
     </row>
-    <row r="18" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B18" s="20"/>
       <c r="C18" s="19" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F18" s="12">
         <v>1</v>
       </c>
       <c r="G18" s="25">
-        <v>67.257269565034619</v>
+        <v>744033.54456319555</v>
       </c>
       <c r="H18" s="13">
         <v>0</v>
       </c>
-      <c r="I18" s="25">
-        <v>1.0448815569668966E-4</v>
-      </c>
-      <c r="J18" s="14">
-        <v>0</v>
+      <c r="I18" s="13">
+        <v>0</v>
+      </c>
+      <c r="J18" s="25">
+        <v>2.3789249999999999E-5</v>
       </c>
       <c r="K18" s="14">
+        <v>0</v>
+      </c>
+      <c r="L18" s="14">
         <v>5000</v>
       </c>
-      <c r="N18" s="14">
-        <v>0</v>
-      </c>
       <c r="O18" s="14">
+        <v>0</v>
+      </c>
+      <c r="P18" s="14">
         <v>0.5</v>
       </c>
-      <c r="P18" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="25">
+      <c r="Q18" s="12">
+        <v>0</v>
+      </c>
+      <c r="R18" s="25">
         <v>6.7917301202848283E-3</v>
       </c>
-      <c r="R18" s="27">
-        <v>0</v>
-      </c>
-      <c r="S18" s="12">
+      <c r="S18" s="27">
         <v>0</v>
       </c>
       <c r="T18" s="12">
         <v>0</v>
       </c>
-      <c r="U18" s="14">
-        <v>99999999999</v>
+      <c r="U18" s="12">
+        <v>0</v>
       </c>
       <c r="V18" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W18" s="13">
+      <c r="W18" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X18" s="13">
         <f t="shared" si="0"/>
-        <v>74.341406250000006</v>
-      </c>
-      <c r="Y18">
-        <v>0</v>
-      </c>
-      <c r="AA18">
+        <v>6.7201271186440679E-3</v>
+      </c>
+      <c r="Z18">
+        <v>0</v>
+      </c>
+      <c r="AB18">
         <v>4703986387</v>
       </c>
-      <c r="AB18">
+      <c r="AC18">
         <v>1544275136</v>
       </c>
     </row>
-    <row r="19" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B19" s="20"/>
       <c r="C19" s="19" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F19" s="12">
         <v>1</v>
       </c>
       <c r="G19" s="25">
-        <v>978.59327217125383</v>
+        <v>2446483.1804281347</v>
       </c>
       <c r="H19" s="13">
         <v>0</v>
       </c>
-      <c r="I19" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J19" s="14">
-        <v>0</v>
+      <c r="I19" s="13">
+        <v>0</v>
+      </c>
+      <c r="J19" s="25">
+        <v>2.4524999999999998E-6</v>
       </c>
       <c r="K19" s="14">
+        <v>0</v>
+      </c>
+      <c r="L19" s="14">
         <v>5000</v>
       </c>
-      <c r="N19" s="14">
-        <v>0</v>
-      </c>
       <c r="O19" s="14">
+        <v>0</v>
+      </c>
+      <c r="P19" s="14">
         <v>0.5</v>
       </c>
-      <c r="P19" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="25">
+      <c r="Q19" s="12">
+        <v>0</v>
+      </c>
+      <c r="R19" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R19" s="27">
-        <v>0</v>
-      </c>
-      <c r="S19" s="12">
+      <c r="S19" s="27">
         <v>0</v>
       </c>
       <c r="T19" s="12">
         <v>0</v>
       </c>
-      <c r="U19" s="14">
-        <v>99999999999</v>
+      <c r="U19" s="12">
+        <v>0</v>
       </c>
       <c r="V19" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W19" s="13">
+      <c r="W19" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X19" s="13">
         <f t="shared" si="0"/>
-        <v>5.109375</v>
-      </c>
-      <c r="Y19">
-        <v>0</v>
-      </c>
-      <c r="AA19">
+        <v>2.04375E-3</v>
+      </c>
+      <c r="Z19">
+        <v>0</v>
+      </c>
+      <c r="AB19">
         <v>4699409124</v>
       </c>
-      <c r="AB19">
+      <c r="AC19">
         <v>1508502495</v>
       </c>
     </row>
-    <row r="20" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B20" s="20"/>
       <c r="C20" s="19" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F20" s="12">
         <v>1</v>
       </c>
       <c r="G20" s="25">
-        <v>84.811416921508666</v>
-      </c>
-      <c r="H20" s="23">
+        <v>848114.16921508661</v>
+      </c>
+      <c r="H20" s="13">
+        <v>0</v>
+      </c>
+      <c r="I20" s="23">
         <v>123.1396524</v>
       </c>
-      <c r="I20" s="25">
-        <v>4.9272151773994549E-3</v>
-      </c>
-      <c r="J20" s="22">
+      <c r="J20" s="25">
+        <v>1.2262500000000001E-4</v>
+      </c>
+      <c r="K20" s="22">
         <v>1.6999999999999999E-3</v>
       </c>
-      <c r="K20" s="14">
+      <c r="L20" s="22">
         <v>15000000</v>
       </c>
-      <c r="N20" s="14">
-        <v>0</v>
-      </c>
       <c r="O20" s="14">
+        <v>0</v>
+      </c>
+      <c r="P20" s="14">
         <v>0.5</v>
       </c>
-      <c r="P20" s="12">
+      <c r="Q20" s="12">
         <v>1</v>
       </c>
-      <c r="Q20" s="25">
+      <c r="R20" s="25">
         <v>0.32026898653096453</v>
       </c>
-      <c r="R20" s="27">
-        <v>0</v>
-      </c>
-      <c r="S20" s="12">
-        <v>0</v>
+      <c r="S20" s="25">
+        <v>0.32026898653096453</v>
       </c>
       <c r="T20" s="12">
         <v>0</v>
       </c>
-      <c r="U20" s="14">
-        <v>99999999999</v>
+      <c r="U20" s="12">
+        <v>0</v>
       </c>
       <c r="V20" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W20" s="13">
+      <c r="W20" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X20" s="13">
         <f t="shared" si="0"/>
-        <v>176862.98076923078</v>
-      </c>
-      <c r="Y20">
-        <v>0</v>
-      </c>
-      <c r="AA20">
+        <v>17.686298076923077</v>
+      </c>
+      <c r="Z20">
+        <v>0</v>
+      </c>
+      <c r="AB20">
         <v>4710370743</v>
       </c>
-      <c r="AB20">
+      <c r="AC20">
         <v>1348112241</v>
       </c>
     </row>
-    <row r="21" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B21" s="20"/>
       <c r="C21" s="19" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F21" s="12">
         <v>1</v>
       </c>
       <c r="G21" s="25">
-        <v>69.171399446628797</v>
+        <v>691713.99446628802</v>
       </c>
       <c r="H21" s="13">
         <v>0</v>
       </c>
-      <c r="I21" s="25">
-        <v>1.0348150151375814E-4</v>
-      </c>
-      <c r="J21" s="14">
-        <v>0</v>
+      <c r="I21" s="13">
+        <v>0</v>
+      </c>
+      <c r="J21" s="25">
+        <v>2.7468000000000002E-5</v>
       </c>
       <c r="K21" s="14">
+        <v>0</v>
+      </c>
+      <c r="L21" s="14">
         <v>5000</v>
       </c>
-      <c r="N21" s="14">
-        <v>0</v>
-      </c>
       <c r="O21" s="14">
+        <v>0</v>
+      </c>
+      <c r="P21" s="14">
         <v>0.5</v>
       </c>
-      <c r="P21" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="25">
+      <c r="Q21" s="12">
+        <v>0</v>
+      </c>
+      <c r="R21" s="25">
         <v>6.7262975983942794E-3</v>
       </c>
-      <c r="R21" s="27">
-        <v>0</v>
-      </c>
-      <c r="S21" s="12">
+      <c r="S21" s="27">
         <v>0</v>
       </c>
       <c r="T21" s="12">
         <v>0</v>
       </c>
-      <c r="U21" s="14">
-        <v>99999999999</v>
+      <c r="U21" s="12">
+        <v>0</v>
       </c>
       <c r="V21" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W21" s="13">
+      <c r="W21" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X21" s="13">
         <f t="shared" si="0"/>
-        <v>72.284210526315803</v>
-      </c>
-      <c r="Y21">
+        <v>7.2284210526315793E-3</v>
+      </c>
+      <c r="Z21">
         <v>2013</v>
       </c>
-      <c r="AA21">
+      <c r="AB21">
         <v>4694360461</v>
       </c>
-      <c r="AB21">
+      <c r="AC21">
         <v>155040946</v>
       </c>
     </row>
-    <row r="22" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B22" s="20"/>
       <c r="C22" s="19" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F22" s="12">
         <v>1</v>
       </c>
       <c r="G22" s="25">
-        <v>85.342436526562835</v>
+        <v>853424.36526562821</v>
       </c>
       <c r="H22" s="13">
         <v>0</v>
       </c>
-      <c r="I22" s="25">
-        <v>1.4666336007454863E-4</v>
-      </c>
-      <c r="J22" s="14">
-        <v>0</v>
+      <c r="I22" s="13">
+        <v>0</v>
+      </c>
+      <c r="J22" s="25">
+        <v>2.1091500000000003E-5</v>
       </c>
       <c r="K22" s="14">
+        <v>0</v>
+      </c>
+      <c r="L22" s="14">
         <v>5000</v>
       </c>
-      <c r="N22" s="14">
-        <v>0</v>
-      </c>
       <c r="O22" s="14">
+        <v>0</v>
+      </c>
+      <c r="P22" s="14">
         <v>0.5</v>
       </c>
-      <c r="P22" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="25">
+      <c r="Q22" s="12">
+        <v>0</v>
+      </c>
+      <c r="R22" s="25">
         <v>9.5331184048456606E-3</v>
       </c>
-      <c r="R22" s="27">
-        <v>0</v>
-      </c>
-      <c r="S22" s="12">
+      <c r="S22" s="27">
         <v>0</v>
       </c>
       <c r="T22" s="12">
         <v>0</v>
       </c>
-      <c r="U22" s="14">
-        <v>99999999999</v>
+      <c r="U22" s="12">
+        <v>0</v>
       </c>
       <c r="V22" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W22" s="13">
+      <c r="W22" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X22" s="13">
         <f t="shared" si="0"/>
-        <v>58.587499999999999</v>
-      </c>
-      <c r="Y22">
+        <v>5.8587500000000011E-3</v>
+      </c>
+      <c r="Z22">
         <v>2023</v>
       </c>
-      <c r="AA22">
+      <c r="AB22">
         <v>4729200001</v>
       </c>
-      <c r="AB22">
+      <c r="AC22">
         <v>15323</v>
       </c>
     </row>
-    <row r="23" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B23" s="20"/>
       <c r="C23" s="19" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F23" s="12">
         <v>1</v>
       </c>
       <c r="G23" s="25">
-        <v>807.49935040275034</v>
+        <v>399752.15366472787</v>
       </c>
       <c r="H23" s="13">
         <v>0</v>
       </c>
-      <c r="I23" s="25">
-        <v>8.9709393743275537E-5</v>
-      </c>
-      <c r="J23" s="14">
-        <v>0</v>
+      <c r="I23" s="13">
+        <v>0</v>
+      </c>
+      <c r="J23" s="25">
+        <v>2.5015500000000001E-5</v>
       </c>
       <c r="K23" s="14">
+        <v>0</v>
+      </c>
+      <c r="L23" s="14">
         <v>5000</v>
       </c>
-      <c r="N23" s="14">
-        <v>0</v>
-      </c>
       <c r="O23" s="14">
+        <v>0</v>
+      </c>
+      <c r="P23" s="14">
         <v>0.5</v>
       </c>
-      <c r="P23" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="25">
+      <c r="Q23" s="12">
+        <v>0</v>
+      </c>
+      <c r="R23" s="25">
         <v>5.8311105933129097E-3</v>
       </c>
-      <c r="R23" s="27">
-        <v>0</v>
-      </c>
-      <c r="S23" s="12">
+      <c r="S23" s="27">
         <v>0</v>
       </c>
       <c r="T23" s="12">
         <v>0</v>
       </c>
-      <c r="U23" s="14">
-        <v>99999999999</v>
+      <c r="U23" s="12">
+        <v>0</v>
       </c>
       <c r="V23" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W23" s="13">
+      <c r="W23" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X23" s="13">
         <f t="shared" si="0"/>
-        <v>6.1919554455445542</v>
-      </c>
-      <c r="Y23">
+        <v>1.250775E-2</v>
+      </c>
+      <c r="Z23">
         <v>1988</v>
       </c>
-      <c r="AA23">
+      <c r="AB23">
         <v>46857847</v>
       </c>
-      <c r="AB23">
+      <c r="AC23">
         <v>1553730001</v>
       </c>
     </row>
-    <row r="24" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B24" s="20"/>
       <c r="C24" s="19" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F24" s="12">
         <v>1</v>
       </c>
       <c r="G24" s="25">
-        <v>509.68399592252803</v>
+        <v>5096839.9592252802</v>
       </c>
       <c r="H24" s="13">
         <v>0</v>
       </c>
-      <c r="I24" s="25">
-        <v>6.8370332515645875E-5</v>
-      </c>
-      <c r="J24" s="14">
-        <v>0</v>
+      <c r="I24" s="13">
+        <v>0</v>
+      </c>
+      <c r="J24" s="25">
+        <v>1.962E-6</v>
       </c>
       <c r="K24" s="14">
+        <v>0</v>
+      </c>
+      <c r="L24" s="14">
         <v>5000</v>
       </c>
-      <c r="N24" s="14">
-        <v>0</v>
-      </c>
       <c r="O24" s="14">
+        <v>0</v>
+      </c>
+      <c r="P24" s="14">
         <v>0.5</v>
       </c>
-      <c r="P24" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="25">
+      <c r="Q24" s="12">
+        <v>0</v>
+      </c>
+      <c r="R24" s="25">
         <v>4.444071613516982E-3</v>
       </c>
-      <c r="R24" s="27">
-        <v>0</v>
-      </c>
-      <c r="S24" s="12">
+      <c r="S24" s="27">
         <v>0</v>
       </c>
       <c r="T24" s="12">
         <v>0</v>
       </c>
-      <c r="U24" s="14">
-        <v>99999999999</v>
+      <c r="U24" s="12">
+        <v>0</v>
       </c>
       <c r="V24" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W24" s="13">
+      <c r="W24" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X24" s="13">
         <f t="shared" si="0"/>
-        <v>9.81</v>
-      </c>
-      <c r="Y24">
-        <v>0</v>
-      </c>
-      <c r="AA24">
+        <v>9.810000000000001E-4</v>
+      </c>
+      <c r="Z24">
+        <v>0</v>
+      </c>
+      <c r="AB24">
         <v>4738847601</v>
       </c>
-      <c r="AB24">
+      <c r="AC24">
         <v>15095161</v>
       </c>
     </row>
-    <row r="25" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B25" s="20"/>
       <c r="C25" s="19" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F25" s="12">
         <v>1</v>
       </c>
       <c r="G25" s="25">
-        <v>662.5891946992864</v>
+        <v>6625891.9469928648</v>
       </c>
       <c r="H25" s="13">
         <v>0</v>
       </c>
-      <c r="I25" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J25" s="14">
-        <v>0</v>
+      <c r="I25" s="13">
+        <v>0</v>
+      </c>
+      <c r="J25" s="25">
+        <v>1.962E-6</v>
       </c>
       <c r="K25" s="14">
+        <v>0</v>
+      </c>
+      <c r="L25" s="14">
         <v>5000</v>
       </c>
-      <c r="N25" s="14">
-        <v>0</v>
-      </c>
       <c r="O25" s="14">
+        <v>0</v>
+      </c>
+      <c r="P25" s="14">
         <v>0.5</v>
       </c>
-      <c r="P25" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="25">
+      <c r="Q25" s="12">
+        <v>0</v>
+      </c>
+      <c r="R25" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R25" s="27">
-        <v>0</v>
-      </c>
-      <c r="S25" s="12">
+      <c r="S25" s="27">
         <v>0</v>
       </c>
       <c r="T25" s="12">
         <v>0</v>
       </c>
-      <c r="U25" s="14">
-        <v>99999999999</v>
+      <c r="U25" s="12">
+        <v>0</v>
       </c>
       <c r="V25" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W25" s="13">
+      <c r="W25" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X25" s="13">
         <f t="shared" si="0"/>
-        <v>7.5461538461538469</v>
-      </c>
-      <c r="Y25">
-        <v>0</v>
-      </c>
-      <c r="AA25">
+        <v>7.5461538461538461E-4</v>
+      </c>
+      <c r="Z25">
+        <v>0</v>
+      </c>
+      <c r="AB25">
         <v>4674575769</v>
       </c>
-      <c r="AB25">
+      <c r="AC25">
         <v>1557182718</v>
       </c>
     </row>
-    <row r="26" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B26" s="20"/>
       <c r="C26" s="19" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F26" s="12">
         <v>1</v>
       </c>
       <c r="G26" s="25">
-        <v>611.6207951070337</v>
+        <v>6116207.9510703366</v>
       </c>
       <c r="H26" s="13">
         <v>0</v>
       </c>
-      <c r="I26" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J26" s="14">
-        <v>0</v>
+      <c r="I26" s="13">
+        <v>0</v>
+      </c>
+      <c r="J26" s="25">
+        <v>2.4524999999999998E-6</v>
       </c>
       <c r="K26" s="14">
+        <v>0</v>
+      </c>
+      <c r="L26" s="14">
         <v>5000000</v>
       </c>
-      <c r="N26" s="14">
-        <v>0</v>
-      </c>
       <c r="O26" s="14">
+        <v>0</v>
+      </c>
+      <c r="P26" s="14">
         <v>0.5</v>
       </c>
-      <c r="P26" s="12">
+      <c r="Q26" s="12">
         <v>1</v>
       </c>
-      <c r="Q26" s="25">
+      <c r="R26" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R26" s="27">
-        <v>0</v>
-      </c>
-      <c r="S26" s="12">
+      <c r="S26" s="27">
         <v>0</v>
       </c>
       <c r="T26" s="12">
         <v>0</v>
       </c>
-      <c r="U26" s="14">
-        <v>99999999999</v>
+      <c r="U26" s="12">
+        <v>0</v>
       </c>
       <c r="V26" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W26" s="13">
+      <c r="W26" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X26" s="13">
         <f t="shared" si="0"/>
-        <v>8174.9999999999991</v>
-      </c>
-      <c r="Y26">
-        <v>0</v>
-      </c>
-      <c r="AA26">
+        <v>0.8175</v>
+      </c>
+      <c r="Z26">
+        <v>0</v>
+      </c>
+      <c r="AB26">
         <v>4697878577</v>
       </c>
-      <c r="AB26">
+      <c r="AC26">
         <v>1502319618</v>
       </c>
     </row>
-    <row r="27" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B27" s="20"/>
       <c r="C27" s="19" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F27" s="12">
         <v>1</v>
       </c>
       <c r="G27" s="25">
-        <v>588.96817306603248</v>
+        <v>5889681.730660324</v>
       </c>
       <c r="H27" s="13">
         <v>0</v>
       </c>
-      <c r="I27" s="25">
-        <v>9.8526263529088916E-5</v>
-      </c>
-      <c r="J27" s="14">
-        <v>0</v>
+      <c r="I27" s="13">
+        <v>0</v>
+      </c>
+      <c r="J27" s="25">
+        <v>2.2072499999999999E-6</v>
       </c>
       <c r="K27" s="14">
+        <v>0</v>
+      </c>
+      <c r="L27" s="14">
         <v>5000</v>
       </c>
-      <c r="N27" s="14">
-        <v>0</v>
-      </c>
       <c r="O27" s="14">
+        <v>0</v>
+      </c>
+      <c r="P27" s="14">
         <v>0.5</v>
       </c>
-      <c r="P27" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="25">
+      <c r="Q27" s="12">
+        <v>0</v>
+      </c>
+      <c r="R27" s="25">
         <v>6.4042071293907796E-3</v>
       </c>
-      <c r="R27" s="27">
-        <v>0</v>
-      </c>
-      <c r="S27" s="12">
+      <c r="S27" s="27">
         <v>0</v>
       </c>
       <c r="T27" s="12">
         <v>0</v>
       </c>
-      <c r="U27" s="14">
-        <v>99999999999</v>
+      <c r="U27" s="12">
+        <v>0</v>
       </c>
       <c r="V27" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W27" s="13">
+      <c r="W27" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X27" s="13">
         <f t="shared" si="0"/>
-        <v>8.4894230769230763</v>
-      </c>
-      <c r="Y27">
+        <v>8.4894230769230771E-4</v>
+      </c>
+      <c r="Z27">
         <v>2009</v>
       </c>
-      <c r="AA27">
+      <c r="AB27">
         <v>4720926001</v>
       </c>
-      <c r="AB27">
+      <c r="AC27">
         <v>15335656</v>
       </c>
     </row>
-    <row r="28" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B28" s="20"/>
       <c r="C28" s="19" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F28" s="12">
         <v>1</v>
       </c>
       <c r="G28" s="25">
-        <v>87665.647298674812</v>
+        <v>9637661.0138078034</v>
       </c>
       <c r="H28" s="13">
         <v>0</v>
       </c>
-      <c r="I28" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J28" s="14">
-        <v>0</v>
+      <c r="I28" s="13">
+        <v>0</v>
+      </c>
+      <c r="J28" s="25">
+        <v>2.6977499999999997E-6</v>
       </c>
       <c r="K28" s="14">
+        <v>0</v>
+      </c>
+      <c r="L28" s="14">
         <v>5000</v>
       </c>
-      <c r="N28" s="14">
-        <v>0</v>
-      </c>
       <c r="O28" s="14">
+        <v>0</v>
+      </c>
+      <c r="P28" s="14">
         <v>0.5</v>
       </c>
-      <c r="P28" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="25">
+      <c r="Q28" s="12">
+        <v>0</v>
+      </c>
+      <c r="R28" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R28" s="27">
-        <v>0</v>
-      </c>
-      <c r="S28" s="12">
+      <c r="S28" s="27">
         <v>0</v>
       </c>
       <c r="T28" s="12">
         <v>0</v>
       </c>
-      <c r="U28" s="14">
-        <v>99999999999</v>
+      <c r="U28" s="12">
+        <v>0</v>
       </c>
       <c r="V28" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W28" s="13">
+      <c r="W28" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X28" s="13">
         <f t="shared" si="0"/>
-        <v>5.7034883720930241E-2</v>
-      </c>
-      <c r="Y28">
+        <v>5.1879807692307685E-4</v>
+      </c>
+      <c r="Z28">
         <v>2013</v>
       </c>
-      <c r="AA28">
+      <c r="AB28">
         <v>4736520001</v>
       </c>
-      <c r="AB28">
+      <c r="AC28">
         <v>1533440001</v>
       </c>
     </row>
-    <row r="29" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B29" s="20"/>
       <c r="C29" s="19" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F29" s="12">
         <v>1</v>
       </c>
       <c r="G29" s="25">
-        <v>81.549439347604476</v>
+        <v>815494.39347604488</v>
       </c>
       <c r="H29" s="13">
         <v>0</v>
       </c>
-      <c r="I29" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J29" s="14">
-        <v>0</v>
+      <c r="I29" s="13">
+        <v>0</v>
+      </c>
+      <c r="J29" s="25">
+        <v>2.4524999999999998E-6</v>
       </c>
       <c r="K29" s="14">
+        <v>0</v>
+      </c>
+      <c r="L29" s="14">
         <v>5000</v>
       </c>
-      <c r="N29" s="14">
-        <v>0</v>
-      </c>
       <c r="O29" s="14">
+        <v>0</v>
+      </c>
+      <c r="P29" s="14">
         <v>0.5</v>
       </c>
-      <c r="P29" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="25">
+      <c r="Q29" s="12">
+        <v>0</v>
+      </c>
+      <c r="R29" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R29" s="27">
-        <v>0</v>
-      </c>
-      <c r="S29" s="12">
+      <c r="S29" s="27">
         <v>0</v>
       </c>
       <c r="T29" s="12">
         <v>0</v>
       </c>
-      <c r="U29" s="14">
-        <v>99999999999</v>
+      <c r="U29" s="12">
+        <v>0</v>
       </c>
       <c r="V29" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W29" s="13">
+      <c r="W29" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X29" s="13">
         <f t="shared" si="0"/>
-        <v>61.312500000000007</v>
-      </c>
-      <c r="Y29">
-        <v>0</v>
-      </c>
-      <c r="AA29">
+        <v>6.1312499999999995E-3</v>
+      </c>
+      <c r="Z29">
+        <v>0</v>
+      </c>
+      <c r="AB29">
         <v>4721774401</v>
       </c>
-      <c r="AB29">
+      <c r="AC29">
         <v>14599075</v>
       </c>
     </row>
-    <row r="30" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B30" s="20"/>
       <c r="C30" s="19" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F30" s="12">
         <v>1</v>
       </c>
       <c r="G30" s="25">
-        <v>634.27341714803492</v>
+        <v>6342734.1714803493</v>
       </c>
       <c r="H30" s="13">
         <v>0</v>
       </c>
-      <c r="I30" s="25">
-        <v>7.8180055576928815E-5</v>
-      </c>
-      <c r="J30" s="14">
-        <v>0</v>
+      <c r="I30" s="13">
+        <v>0</v>
+      </c>
+      <c r="J30" s="25">
+        <v>2.2072499999999999E-6</v>
       </c>
       <c r="K30" s="14">
+        <v>0</v>
+      </c>
+      <c r="L30" s="14">
         <v>5000</v>
       </c>
-      <c r="N30" s="14">
-        <v>0</v>
-      </c>
       <c r="O30" s="14">
+        <v>0</v>
+      </c>
+      <c r="P30" s="14">
         <v>0.5</v>
       </c>
-      <c r="P30" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="25">
+      <c r="Q30" s="12">
+        <v>0</v>
+      </c>
+      <c r="R30" s="25">
         <v>5.0817036125003724E-3</v>
       </c>
-      <c r="R30" s="27">
-        <v>0</v>
-      </c>
-      <c r="S30" s="12">
+      <c r="S30" s="27">
         <v>0</v>
       </c>
       <c r="T30" s="12">
         <v>0</v>
       </c>
-      <c r="U30" s="14">
-        <v>99999999999</v>
+      <c r="U30" s="12">
+        <v>0</v>
       </c>
       <c r="V30" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W30" s="13">
+      <c r="W30" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X30" s="13">
         <f t="shared" si="0"/>
-        <v>7.8830357142857137</v>
-      </c>
-      <c r="Y30">
-        <v>0</v>
-      </c>
-      <c r="AA30">
+        <v>7.8830357142857142E-4</v>
+      </c>
+      <c r="Z30">
+        <v>0</v>
+      </c>
+      <c r="AB30">
         <v>4725087014</v>
       </c>
-      <c r="AB30">
+      <c r="AC30">
         <v>1531009022</v>
       </c>
     </row>
-    <row r="31" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B31" s="20"/>
       <c r="C31" s="19" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F31" s="12">
         <v>1</v>
       </c>
       <c r="G31" s="25">
-        <v>40.774719673802238</v>
+        <v>407747.19673802244</v>
       </c>
       <c r="H31" s="13">
         <v>0</v>
       </c>
-      <c r="I31" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J31" s="14">
-        <v>0</v>
+      <c r="I31" s="13">
+        <v>0</v>
+      </c>
+      <c r="J31" s="25">
+        <v>2.4524999999999998E-6</v>
       </c>
       <c r="K31" s="14">
+        <v>0</v>
+      </c>
+      <c r="L31" s="14">
         <v>5000</v>
       </c>
-      <c r="N31" s="14">
-        <v>0</v>
-      </c>
       <c r="O31" s="14">
+        <v>0</v>
+      </c>
+      <c r="P31" s="14">
         <v>0.5</v>
       </c>
-      <c r="P31" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q31" s="25">
+      <c r="Q31" s="12">
+        <v>0</v>
+      </c>
+      <c r="R31" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R31" s="27">
-        <v>0</v>
-      </c>
-      <c r="S31" s="12">
+      <c r="S31" s="27">
         <v>0</v>
       </c>
       <c r="T31" s="12">
         <v>0</v>
       </c>
-      <c r="U31" s="14">
-        <v>99999999999</v>
+      <c r="U31" s="12">
+        <v>0</v>
       </c>
       <c r="V31" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W31" s="13">
+      <c r="W31" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X31" s="13">
         <f t="shared" si="0"/>
-        <v>122.62500000000001</v>
-      </c>
-      <c r="Y31">
-        <v>0</v>
-      </c>
-      <c r="AA31">
+        <v>1.2262499999999999E-2</v>
+      </c>
+      <c r="Z31">
+        <v>0</v>
+      </c>
+      <c r="AB31">
         <v>4674433801</v>
       </c>
-      <c r="AB31">
+      <c r="AC31">
         <v>1557045501</v>
       </c>
     </row>
-    <row r="32" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B32" s="20"/>
       <c r="C32" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F32" s="12">
         <v>1</v>
       </c>
       <c r="G32" s="25">
-        <v>76.821935617308583</v>
+        <v>768219.35617308575</v>
       </c>
       <c r="H32" s="13">
         <v>0</v>
       </c>
-      <c r="I32" s="25">
-        <v>6.3496793032866511E-5</v>
-      </c>
-      <c r="J32" s="14">
-        <v>0</v>
+      <c r="I32" s="13">
+        <v>0</v>
+      </c>
+      <c r="J32" s="25">
+        <v>1.6922249999999999E-5</v>
       </c>
       <c r="K32" s="14">
+        <v>0</v>
+      </c>
+      <c r="L32" s="14">
         <v>5000</v>
       </c>
-      <c r="N32" s="14">
-        <v>0</v>
-      </c>
       <c r="O32" s="14">
+        <v>0</v>
+      </c>
+      <c r="P32" s="14">
         <v>0.5</v>
       </c>
-      <c r="P32" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q32" s="25">
+      <c r="Q32" s="12">
+        <v>0</v>
+      </c>
+      <c r="R32" s="25">
         <v>4.1272915471363232E-3</v>
       </c>
-      <c r="R32" s="27">
-        <v>0</v>
-      </c>
-      <c r="S32" s="12">
+      <c r="S32" s="27">
         <v>0</v>
       </c>
       <c r="T32" s="12">
         <v>0</v>
       </c>
-      <c r="U32" s="14">
-        <v>99999999999</v>
+      <c r="U32" s="12">
+        <v>0</v>
       </c>
       <c r="V32" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W32" s="13">
+      <c r="W32" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X32" s="13">
         <f t="shared" si="0"/>
-        <v>65.085576923076914</v>
-      </c>
-      <c r="Y32">
+        <v>6.508557692307692E-3</v>
+      </c>
+      <c r="Z32">
         <v>1982</v>
       </c>
-      <c r="AA32">
+      <c r="AB32">
         <v>4671685586</v>
       </c>
-      <c r="AB32">
+      <c r="AC32">
         <v>1562152978</v>
       </c>
     </row>
-    <row r="33" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B33" s="20"/>
       <c r="C33" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F33" s="12">
         <v>1</v>
       </c>
       <c r="G33" s="25">
-        <v>28.782155063860408</v>
+        <v>287821.55063860409</v>
       </c>
       <c r="H33" s="13">
         <v>0</v>
       </c>
-      <c r="I33" s="25">
-        <v>1.6206168391813292E-4</v>
-      </c>
-      <c r="J33" s="14">
-        <v>0</v>
+      <c r="I33" s="13">
+        <v>0</v>
+      </c>
+      <c r="J33" s="25">
+        <v>2.0846250000000001E-5</v>
       </c>
       <c r="K33" s="14">
+        <v>0</v>
+      </c>
+      <c r="L33" s="14">
         <v>5000</v>
       </c>
-      <c r="N33" s="14">
-        <v>0</v>
-      </c>
       <c r="O33" s="14">
+        <v>0</v>
+      </c>
+      <c r="P33" s="14">
         <v>0.5</v>
       </c>
-      <c r="P33" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q33" s="25">
+      <c r="Q33" s="12">
+        <v>0</v>
+      </c>
+      <c r="R33" s="25">
         <v>1.0534009454678639E-2</v>
       </c>
-      <c r="R33" s="27">
-        <v>0</v>
-      </c>
-      <c r="S33" s="12">
+      <c r="S33" s="27">
         <v>0</v>
       </c>
       <c r="T33" s="12">
         <v>0</v>
       </c>
-      <c r="U33" s="14">
-        <v>99999999999</v>
+      <c r="U33" s="12">
+        <v>0</v>
       </c>
       <c r="V33" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W33" s="13">
+      <c r="W33" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X33" s="13">
         <f t="shared" si="0"/>
-        <v>173.71875</v>
-      </c>
-      <c r="Y33">
+        <v>1.7371874999999998E-2</v>
+      </c>
+      <c r="Z33">
         <v>1985</v>
       </c>
-      <c r="AA33">
+      <c r="AB33">
         <v>4710441021</v>
       </c>
-      <c r="AB33">
+      <c r="AC33">
         <v>1408673125</v>
       </c>
     </row>
-    <row r="34" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B34" s="20"/>
       <c r="C34" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F34" s="12">
         <v>1</v>
       </c>
       <c r="G34" s="25">
-        <v>652.39551478083581</v>
+        <v>6523955.147808359</v>
       </c>
       <c r="H34" s="13">
         <v>0</v>
       </c>
-      <c r="I34" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J34" s="14">
-        <v>0</v>
+      <c r="I34" s="13">
+        <v>0</v>
+      </c>
+      <c r="J34" s="25">
+        <v>2.4524999999999998E-6</v>
       </c>
       <c r="K34" s="14">
+        <v>0</v>
+      </c>
+      <c r="L34" s="14">
         <v>5000</v>
       </c>
-      <c r="N34" s="14">
-        <v>0</v>
-      </c>
       <c r="O34" s="14">
+        <v>0</v>
+      </c>
+      <c r="P34" s="14">
         <v>0.5</v>
       </c>
-      <c r="P34" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="25">
+      <c r="Q34" s="12">
+        <v>0</v>
+      </c>
+      <c r="R34" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R34" s="27">
-        <v>0</v>
-      </c>
-      <c r="S34" s="12">
+      <c r="S34" s="27">
         <v>0</v>
       </c>
       <c r="T34" s="12">
         <v>0</v>
       </c>
-      <c r="U34" s="14">
-        <v>99999999999</v>
+      <c r="U34" s="12">
+        <v>0</v>
       </c>
       <c r="V34" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W34" s="13">
+      <c r="W34" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X34" s="13">
         <f t="shared" si="0"/>
-        <v>7.6640625000000009</v>
-      </c>
-      <c r="Y34">
-        <v>0</v>
-      </c>
-      <c r="AA34">
+        <v>7.6640624999999994E-4</v>
+      </c>
+      <c r="Z34">
+        <v>0</v>
+      </c>
+      <c r="AB34">
         <v>4698734792</v>
       </c>
-      <c r="AB34">
+      <c r="AC34">
         <v>150912762</v>
       </c>
     </row>
-    <row r="35" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B35" s="20"/>
       <c r="C35" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F35" s="12">
         <v>1</v>
       </c>
       <c r="G35" s="25">
-        <v>489.29663608562691</v>
+        <v>4892966.3608562695</v>
       </c>
       <c r="H35" s="13">
         <v>0</v>
       </c>
-      <c r="I35" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J35" s="14">
-        <v>0</v>
+      <c r="I35" s="13">
+        <v>0</v>
+      </c>
+      <c r="J35" s="25">
+        <v>2.4524999999999998E-6</v>
       </c>
       <c r="K35" s="14">
+        <v>0</v>
+      </c>
+      <c r="L35" s="14">
         <v>5000</v>
       </c>
-      <c r="N35" s="14">
-        <v>0</v>
-      </c>
       <c r="O35" s="14">
+        <v>0</v>
+      </c>
+      <c r="P35" s="14">
         <v>0.5</v>
       </c>
-      <c r="P35" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q35" s="25">
+      <c r="Q35" s="12">
+        <v>0</v>
+      </c>
+      <c r="R35" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R35" s="27">
-        <v>0</v>
-      </c>
-      <c r="S35" s="12">
+      <c r="S35" s="27">
         <v>0</v>
       </c>
       <c r="T35" s="12">
         <v>0</v>
       </c>
-      <c r="U35" s="14">
-        <v>99999999999</v>
+      <c r="U35" s="12">
+        <v>0</v>
       </c>
       <c r="V35" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W35" s="13">
+      <c r="W35" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X35" s="13">
         <f t="shared" si="0"/>
-        <v>10.21875</v>
-      </c>
-      <c r="Y35">
-        <v>0</v>
-      </c>
-      <c r="AA35">
+        <v>1.021875E-3</v>
+      </c>
+      <c r="Z35">
+        <v>0</v>
+      </c>
+      <c r="AB35">
         <v>4717522501</v>
       </c>
-      <c r="AB35">
+      <c r="AC35">
         <v>1532038501</v>
       </c>
     </row>
-    <row r="36" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B36" s="20"/>
       <c r="C36" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F36" s="12">
         <v>1</v>
       </c>
       <c r="G36" s="25">
-        <v>40.774719673802238</v>
+        <v>407747.19673802244</v>
       </c>
       <c r="H36" s="13">
         <v>0</v>
       </c>
-      <c r="I36" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J36" s="14">
-        <v>0</v>
+      <c r="I36" s="13">
+        <v>0</v>
+      </c>
+      <c r="J36" s="25">
+        <v>2.4524999999999998E-6</v>
       </c>
       <c r="K36" s="14">
+        <v>0</v>
+      </c>
+      <c r="L36" s="14">
         <v>5000</v>
       </c>
-      <c r="N36" s="14">
-        <v>0</v>
-      </c>
       <c r="O36" s="14">
+        <v>0</v>
+      </c>
+      <c r="P36" s="14">
         <v>0.5</v>
       </c>
-      <c r="P36" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q36" s="25">
+      <c r="Q36" s="12">
+        <v>0</v>
+      </c>
+      <c r="R36" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R36" s="27">
-        <v>0</v>
-      </c>
-      <c r="S36" s="12">
+      <c r="S36" s="27">
         <v>0</v>
       </c>
       <c r="T36" s="12">
         <v>0</v>
       </c>
-      <c r="U36" s="14">
-        <v>99999999999</v>
+      <c r="U36" s="12">
+        <v>0</v>
       </c>
       <c r="V36" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W36" s="13">
+      <c r="W36" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X36" s="13">
         <f t="shared" si="0"/>
-        <v>122.62500000000001</v>
-      </c>
-      <c r="Y36">
-        <v>0</v>
-      </c>
-      <c r="AA36">
+        <v>1.2262499999999999E-2</v>
+      </c>
+      <c r="Z36">
+        <v>0</v>
+      </c>
+      <c r="AB36">
         <v>4702151301</v>
       </c>
-      <c r="AB36">
+      <c r="AC36">
         <v>1516653701</v>
       </c>
     </row>
-    <row r="37" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B37" s="20"/>
       <c r="C37" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F37" s="12">
         <v>1</v>
       </c>
       <c r="G37" s="25">
-        <v>40.774719673802238</v>
+        <v>407747.19673802244</v>
       </c>
       <c r="H37" s="13">
         <v>0</v>
       </c>
-      <c r="I37" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J37" s="14">
-        <v>0</v>
+      <c r="I37" s="13">
+        <v>0</v>
+      </c>
+      <c r="J37" s="25">
+        <v>2.4524999999999998E-6</v>
       </c>
       <c r="K37" s="14">
+        <v>0</v>
+      </c>
+      <c r="L37" s="14">
         <v>5000</v>
       </c>
-      <c r="N37" s="14">
-        <v>0</v>
-      </c>
       <c r="O37" s="14">
+        <v>0</v>
+      </c>
+      <c r="P37" s="14">
         <v>0.5</v>
       </c>
-      <c r="P37" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q37" s="25">
+      <c r="Q37" s="12">
+        <v>0</v>
+      </c>
+      <c r="R37" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R37" s="27">
-        <v>0</v>
-      </c>
-      <c r="S37" s="12">
+      <c r="S37" s="27">
         <v>0</v>
       </c>
       <c r="T37" s="12">
         <v>0</v>
       </c>
-      <c r="U37" s="14">
-        <v>99999999999</v>
+      <c r="U37" s="12">
+        <v>0</v>
       </c>
       <c r="V37" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W37" s="13">
+      <c r="W37" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X37" s="13">
         <f t="shared" si="0"/>
-        <v>122.62500000000001</v>
-      </c>
-      <c r="Y37">
-        <v>0</v>
-      </c>
-      <c r="AA37">
+        <v>1.2262499999999999E-2</v>
+      </c>
+      <c r="Z37">
+        <v>0</v>
+      </c>
+      <c r="AB37">
         <v>4749543701</v>
       </c>
-      <c r="AB37">
+      <c r="AC37">
         <v>1499248</v>
       </c>
     </row>
-    <row r="38" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B38" s="20"/>
       <c r="C38" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F38" s="12">
         <v>1</v>
       </c>
       <c r="G38" s="25">
-        <v>630.1547585951256</v>
+        <v>6301547.5859512556</v>
       </c>
       <c r="H38" s="13">
         <v>0</v>
       </c>
-      <c r="I38" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J38" s="14">
-        <v>0</v>
+      <c r="I38" s="13">
+        <v>0</v>
+      </c>
+      <c r="J38" s="25">
+        <v>2.6977499999999997E-6</v>
       </c>
       <c r="K38" s="14">
+        <v>0</v>
+      </c>
+      <c r="L38" s="14">
         <v>5000</v>
       </c>
-      <c r="N38" s="14">
-        <v>0</v>
-      </c>
       <c r="O38" s="14">
+        <v>0</v>
+      </c>
+      <c r="P38" s="14">
         <v>0.5</v>
       </c>
-      <c r="P38" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q38" s="25">
+      <c r="Q38" s="12">
+        <v>0</v>
+      </c>
+      <c r="R38" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R38" s="27">
-        <v>0</v>
-      </c>
-      <c r="S38" s="12">
+      <c r="S38" s="27">
         <v>0</v>
       </c>
       <c r="T38" s="12">
         <v>0</v>
       </c>
-      <c r="U38" s="14">
-        <v>99999999999</v>
+      <c r="U38" s="12">
+        <v>0</v>
       </c>
       <c r="V38" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W38" s="13">
+      <c r="W38" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X38" s="13">
         <f t="shared" si="0"/>
-        <v>7.9345588235294118</v>
-      </c>
-      <c r="Y38">
+        <v>7.9345588235294113E-4</v>
+      </c>
+      <c r="Z38">
         <v>1982</v>
       </c>
-      <c r="AA38">
+      <c r="AB38">
         <v>4710900101</v>
       </c>
-      <c r="AB38">
+      <c r="AC38">
         <v>1539200001</v>
       </c>
     </row>
-    <row r="39" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B39" s="20"/>
       <c r="C39" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F39" s="12">
         <v>1</v>
       </c>
       <c r="G39" s="25">
-        <v>40.774719673802238</v>
+        <v>407747.19673802244</v>
       </c>
       <c r="H39" s="13">
         <v>0</v>
       </c>
-      <c r="I39" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J39" s="14">
-        <v>0</v>
+      <c r="I39" s="13">
+        <v>0</v>
+      </c>
+      <c r="J39" s="25">
+        <v>2.4524999999999998E-6</v>
       </c>
       <c r="K39" s="14">
+        <v>0</v>
+      </c>
+      <c r="L39" s="14">
         <v>5000</v>
       </c>
-      <c r="N39" s="14">
-        <v>0</v>
-      </c>
       <c r="O39" s="14">
+        <v>0</v>
+      </c>
+      <c r="P39" s="14">
         <v>0.5</v>
       </c>
-      <c r="P39" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q39" s="25">
+      <c r="Q39" s="12">
+        <v>0</v>
+      </c>
+      <c r="R39" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R39" s="27">
-        <v>0</v>
-      </c>
-      <c r="S39" s="12">
+      <c r="S39" s="27">
         <v>0</v>
       </c>
       <c r="T39" s="12">
         <v>0</v>
       </c>
-      <c r="U39" s="14">
-        <v>99999999999</v>
+      <c r="U39" s="12">
+        <v>0</v>
       </c>
       <c r="V39" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W39" s="13">
+      <c r="W39" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X39" s="13">
         <f t="shared" si="0"/>
-        <v>122.62500000000001</v>
-      </c>
-      <c r="Y39">
-        <v>0</v>
-      </c>
-      <c r="AA39">
+        <v>1.2262499999999999E-2</v>
+      </c>
+      <c r="Z39">
+        <v>0</v>
+      </c>
+      <c r="AB39">
         <v>4691254801</v>
       </c>
-      <c r="AB39">
+      <c r="AC39">
         <v>1548666401</v>
       </c>
     </row>
-    <row r="40" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B40" s="20"/>
       <c r="C40" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F40" s="12">
         <v>1</v>
       </c>
       <c r="G40" s="25">
-        <v>2201.8348623853208</v>
+        <v>1997961.26401631</v>
       </c>
       <c r="H40" s="13">
         <v>0</v>
       </c>
-      <c r="I40" s="25">
-        <v>2.5224658889183604E-4</v>
-      </c>
-      <c r="J40" s="14">
-        <v>0</v>
+      <c r="I40" s="13">
+        <v>0</v>
+      </c>
+      <c r="J40" s="25">
+        <v>2.4524999999999998E-6</v>
       </c>
       <c r="K40" s="14">
+        <v>0</v>
+      </c>
+      <c r="L40" s="14">
         <v>5000</v>
       </c>
-      <c r="N40" s="14">
-        <v>0</v>
-      </c>
       <c r="O40" s="14">
+        <v>0</v>
+      </c>
+      <c r="P40" s="14">
         <v>0.5</v>
       </c>
-      <c r="P40" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q40" s="25">
+      <c r="Q40" s="12">
+        <v>0</v>
+      </c>
+      <c r="R40" s="25">
         <v>1.2856572927425324E-2</v>
       </c>
-      <c r="R40" s="27">
-        <v>0</v>
-      </c>
-      <c r="S40" s="12">
+      <c r="S40" s="27">
         <v>0</v>
       </c>
       <c r="T40" s="12">
         <v>0</v>
       </c>
-      <c r="U40" s="14">
-        <v>99999999999</v>
+      <c r="U40" s="12">
+        <v>0</v>
       </c>
       <c r="V40" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W40" s="13">
+      <c r="W40" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X40" s="13">
         <f t="shared" si="0"/>
-        <v>2.2708333333333335</v>
-      </c>
-      <c r="Y40">
+        <v>2.502551020408163E-3</v>
+      </c>
+      <c r="Z40">
         <v>1988</v>
       </c>
-      <c r="AA40">
+      <c r="AB40">
         <v>4720008473</v>
       </c>
-      <c r="AB40">
+      <c r="AC40">
         <v>1444253532</v>
       </c>
     </row>
-    <row r="41" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B41" s="20"/>
       <c r="C41" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F41" s="12">
         <v>1</v>
       </c>
       <c r="G41" s="25">
-        <v>1.6059361825050114</v>
+        <v>16059.361825050113</v>
       </c>
       <c r="H41" s="13">
         <v>0</v>
       </c>
-      <c r="I41" s="25">
-        <v>1.010294719501774E-3</v>
-      </c>
-      <c r="J41" s="14">
-        <v>0</v>
+      <c r="I41" s="13">
+        <v>0</v>
+      </c>
+      <c r="J41" s="25">
+        <v>6.2268974999999999E-4</v>
       </c>
       <c r="K41" s="14">
+        <v>0</v>
+      </c>
+      <c r="L41" s="14">
         <v>5000</v>
       </c>
-      <c r="N41" s="14">
-        <v>0</v>
-      </c>
       <c r="O41" s="14">
+        <v>0</v>
+      </c>
+      <c r="P41" s="14">
         <v>0.5</v>
       </c>
-      <c r="P41" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q41" s="25">
+      <c r="Q41" s="12">
+        <v>0</v>
+      </c>
+      <c r="R41" s="25">
         <v>6.5669156767615311E-2</v>
       </c>
-      <c r="R41" s="27">
-        <v>0</v>
-      </c>
-      <c r="S41" s="12">
+      <c r="S41" s="27">
         <v>0</v>
       </c>
       <c r="T41" s="12">
         <v>0</v>
       </c>
-      <c r="U41" s="14">
-        <v>99999999999</v>
+      <c r="U41" s="12">
+        <v>0</v>
       </c>
       <c r="V41" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W41" s="13">
+      <c r="W41" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X41" s="13">
         <f t="shared" si="0"/>
-        <v>3113.4487500000005</v>
-      </c>
-      <c r="Y41">
+        <v>0.31134487500000002</v>
+      </c>
+      <c r="Z41">
         <v>1984</v>
       </c>
-      <c r="AA41">
+      <c r="AB41">
         <v>47164754</v>
       </c>
-      <c r="AB41">
+      <c r="AC41">
         <v>1347057096</v>
       </c>
     </row>
-    <row r="42" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B42" s="20"/>
       <c r="C42" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F42" s="12">
         <v>1</v>
       </c>
       <c r="G42" s="25">
-        <v>4.9826541352915168</v>
+        <v>49826.54135291517</v>
       </c>
       <c r="H42" s="13">
         <v>0</v>
       </c>
-      <c r="I42" s="25">
-        <v>8.4414548638109697E-5</v>
-      </c>
-      <c r="J42" s="14">
-        <v>0</v>
+      <c r="I42" s="13">
+        <v>0</v>
+      </c>
+      <c r="J42" s="25">
+        <v>6.0208875000000001E-4</v>
       </c>
       <c r="K42" s="14">
+        <v>0</v>
+      </c>
+      <c r="L42" s="14">
         <v>5000</v>
       </c>
-      <c r="N42" s="14">
-        <v>0</v>
-      </c>
       <c r="O42" s="14">
+        <v>0</v>
+      </c>
+      <c r="P42" s="14">
         <v>0.5</v>
       </c>
-      <c r="P42" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q42" s="25">
+      <c r="Q42" s="12">
+        <v>0</v>
+      </c>
+      <c r="R42" s="25">
         <v>5.48694566147713E-3</v>
       </c>
-      <c r="R42" s="27">
-        <v>0</v>
-      </c>
-      <c r="S42" s="12">
+      <c r="S42" s="27">
         <v>0</v>
       </c>
       <c r="T42" s="12">
         <v>0</v>
       </c>
-      <c r="U42" s="14">
-        <v>99999999999</v>
+      <c r="U42" s="12">
+        <v>0</v>
       </c>
       <c r="V42" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W42" s="13">
+      <c r="W42" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X42" s="13">
         <f t="shared" si="0"/>
-        <v>1003.4812499999999</v>
-      </c>
-      <c r="Y42">
+        <v>0.10034812499999998</v>
+      </c>
+      <c r="Z42">
         <v>1925</v>
       </c>
-      <c r="AA42">
+      <c r="AB42">
         <v>4701838219</v>
       </c>
-      <c r="AB42">
+      <c r="AC42">
         <v>1515986506</v>
       </c>
     </row>
-    <row r="43" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B43" s="20"/>
       <c r="C43" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F43" s="12">
         <v>1</v>
       </c>
       <c r="G43" s="25">
-        <v>94.954826637621665</v>
+        <v>949548.26637621643</v>
       </c>
       <c r="H43" s="13">
         <v>0</v>
       </c>
-      <c r="I43" s="25">
-        <v>9.4294189287256525E-5</v>
-      </c>
-      <c r="J43" s="14">
-        <v>0</v>
+      <c r="I43" s="13">
+        <v>0</v>
+      </c>
+      <c r="J43" s="25">
+        <v>1.7903250000000002E-5</v>
       </c>
       <c r="K43" s="14">
+        <v>0</v>
+      </c>
+      <c r="L43" s="14">
         <v>5000</v>
       </c>
-      <c r="N43" s="14">
-        <v>0</v>
-      </c>
       <c r="O43" s="14">
+        <v>0</v>
+      </c>
+      <c r="P43" s="14">
         <v>0.5</v>
       </c>
-      <c r="P43" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q43" s="25">
+      <c r="Q43" s="12">
+        <v>0</v>
+      </c>
+      <c r="R43" s="25">
         <v>6.1291223036716736E-3</v>
       </c>
-      <c r="R43" s="27">
-        <v>0</v>
-      </c>
-      <c r="S43" s="12">
+      <c r="S43" s="27">
         <v>0</v>
       </c>
       <c r="T43" s="12">
         <v>0</v>
       </c>
-      <c r="U43" s="14">
-        <v>99999999999</v>
+      <c r="U43" s="12">
+        <v>0</v>
       </c>
       <c r="V43" s="14">
         <v>99999999999</v>
       </c>
-      <c r="W43" s="13">
+      <c r="W43" s="14">
+        <v>99999999999</v>
+      </c>
+      <c r="X43" s="13">
         <f t="shared" si="0"/>
-        <v>52.656617647058823</v>
-      </c>
-      <c r="Y43">
+        <v>5.2656617647058833E-3</v>
+      </c>
+      <c r="Z43">
         <v>1985</v>
       </c>
-      <c r="AA43">
+      <c r="AB43">
         <v>4691099901</v>
       </c>
-      <c r="AB43">
+      <c r="AC43">
         <v>1548600001</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update HydroAssets & Network, add example Storage & VRES
</commit_message>
<xml_diff>
--- a/data/hydroExample/Power_HydroAssets.xlsx
+++ b/data/hydroExample/Power_HydroAssets.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth\Dropbox\Privat\Masterarbeit_2025\Old_calc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\hydroExample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAF0EB8E-050E-41A5-A4C2-B9211D80F72A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{634B25AA-2B10-40E5-9D7C-994AF12F11DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="53445" yWindow="-21585" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Scenario_2014" sheetId="1" r:id="rId1"/>
+    <sheet name="Scenario_2015" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="140">
   <si>
     <t>Format:</t>
   </si>
@@ -393,9 +393,6 @@
     <t>PowerFactorPump</t>
   </si>
   <si>
-    <t>MaxPump</t>
-  </si>
-  <si>
     <t>Maximum Pumping</t>
   </si>
   <si>
@@ -541,6 +538,15 @@
   </si>
   <si>
     <t>190 Mellach und Kuehlwasserturbine-KW</t>
+  </si>
+  <si>
+    <t>MaxProdWater</t>
+  </si>
+  <si>
+    <t>MinProdWater</t>
+  </si>
+  <si>
+    <t>MaxPumpWater</t>
   </si>
 </sst>
 </file>
@@ -568,26 +574,31 @@
       <b/>
       <sz val="11"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
       <color rgb="FFFFFFFF"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -760,8 +771,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Komma" xfId="1" builtinId="3"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1065,12 +1076,14 @@
     <tabColor rgb="FF008080"/>
   </sheetPr>
   <dimension ref="A1:AE43"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" customWidth="1"/>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
     <col min="3" max="3" width="29.85546875" customWidth="1"/>
-    <col min="4" max="9" width="15.7109375" customWidth="1"/>
+    <col min="4" max="6" width="15.7109375" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" customWidth="1"/>
+    <col min="8" max="9" width="15.7109375" customWidth="1"/>
     <col min="10" max="12" width="21.7109375" customWidth="1"/>
     <col min="13" max="16" width="15.7109375" customWidth="1"/>
     <col min="17" max="17" width="20.7109375" customWidth="1"/>
@@ -1089,7 +1102,7 @@
     <row r="1" spans="1:31" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1126,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
@@ -1155,7 +1168,7 @@
         <v>8</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>84</v>
@@ -1164,7 +1177,7 @@
         <v>86</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M3" s="5" t="s">
         <v>9</v>
@@ -1182,10 +1195,10 @@
         <v>13</v>
       </c>
       <c r="R3" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="S3" s="5" t="s">
         <v>91</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>92</v>
       </c>
       <c r="T3" s="5" t="s">
         <v>14</v>
@@ -1244,13 +1257,13 @@
         <v>6</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>7</v>
+        <v>137</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>8</v>
+        <v>138</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>88</v>
+        <v>139</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>85</v>
@@ -1259,7 +1272,7 @@
         <v>87</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M4" s="6" t="s">
         <v>9</v>
@@ -1277,10 +1290,10 @@
         <v>13</v>
       </c>
       <c r="R4" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="S4" s="6" t="s">
         <v>91</v>
-      </c>
-      <c r="S4" s="6" t="s">
-        <v>92</v>
       </c>
       <c r="T4" s="6" t="s">
         <v>14</v>
@@ -1352,7 +1365,7 @@
         <v>48</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M5" s="7" t="s">
         <v>49</v>
@@ -1521,22 +1534,22 @@
         <v>72</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L7" s="26" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M7" s="9" t="s">
         <v>74</v>
@@ -1554,10 +1567,10 @@
         <v>75</v>
       </c>
       <c r="R7" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S7" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="T7" s="9" t="s">
         <v>75</v>
@@ -1600,13 +1613,13 @@
       <c r="A8" s="10"/>
       <c r="B8" s="20"/>
       <c r="C8" s="18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F8" s="12">
         <v>1</v>
@@ -1678,13 +1691,13 @@
     <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B9" s="20"/>
       <c r="C9" s="19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F9" s="12">
         <v>1</v>
@@ -1751,13 +1764,13 @@
     <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B10" s="20"/>
       <c r="C10" s="19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F10" s="12">
         <v>1</v>
@@ -1824,13 +1837,13 @@
     <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B11" s="20"/>
       <c r="C11" s="19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F11" s="12">
         <v>1</v>
@@ -1897,13 +1910,13 @@
     <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B12" s="20"/>
       <c r="C12" s="19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F12" s="12">
         <v>1</v>
@@ -1970,13 +1983,13 @@
     <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B13" s="20"/>
       <c r="C13" s="19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F13" s="12">
         <v>1</v>
@@ -2043,13 +2056,13 @@
     <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B14" s="20"/>
       <c r="C14" s="19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F14" s="12">
         <v>1</v>
@@ -2116,13 +2129,13 @@
     <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B15" s="20"/>
       <c r="C15" s="19" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F15" s="12">
         <v>1</v>
@@ -2189,13 +2202,13 @@
     <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="B16" s="20"/>
       <c r="C16" s="19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F16" s="12">
         <v>1</v>
@@ -2262,13 +2275,13 @@
     <row r="17" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B17" s="20"/>
       <c r="C17" s="19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F17" s="12">
         <v>1</v>
@@ -2335,13 +2348,13 @@
     <row r="18" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B18" s="20"/>
       <c r="C18" s="19" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D18" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F18" s="12">
         <v>1</v>
@@ -2408,13 +2421,13 @@
     <row r="19" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B19" s="20"/>
       <c r="C19" s="19" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F19" s="12">
         <v>1</v>
@@ -2481,13 +2494,13 @@
     <row r="20" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B20" s="20"/>
       <c r="C20" s="19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D20" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F20" s="12">
         <v>1</v>
@@ -2554,13 +2567,13 @@
     <row r="21" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B21" s="20"/>
       <c r="C21" s="19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F21" s="12">
         <v>1</v>
@@ -2627,13 +2640,13 @@
     <row r="22" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B22" s="20"/>
       <c r="C22" s="19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D22" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F22" s="12">
         <v>1</v>
@@ -2700,13 +2713,13 @@
     <row r="23" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B23" s="20"/>
       <c r="C23" s="19" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F23" s="12">
         <v>1</v>
@@ -2773,13 +2786,13 @@
     <row r="24" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B24" s="20"/>
       <c r="C24" s="19" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F24" s="12">
         <v>1</v>
@@ -2846,13 +2859,13 @@
     <row r="25" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B25" s="20"/>
       <c r="C25" s="19" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D25" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F25" s="12">
         <v>1</v>
@@ -2919,13 +2932,13 @@
     <row r="26" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B26" s="20"/>
       <c r="C26" s="19" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F26" s="12">
         <v>1</v>
@@ -2992,13 +3005,13 @@
     <row r="27" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B27" s="20"/>
       <c r="C27" s="19" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F27" s="12">
         <v>1</v>
@@ -3065,13 +3078,13 @@
     <row r="28" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B28" s="20"/>
       <c r="C28" s="19" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F28" s="12">
         <v>1</v>
@@ -3138,13 +3151,13 @@
     <row r="29" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B29" s="20"/>
       <c r="C29" s="19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F29" s="12">
         <v>1</v>
@@ -3211,13 +3224,13 @@
     <row r="30" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B30" s="20"/>
       <c r="C30" s="19" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F30" s="12">
         <v>1</v>
@@ -3284,13 +3297,13 @@
     <row r="31" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B31" s="20"/>
       <c r="C31" s="19" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F31" s="12">
         <v>1</v>
@@ -3357,13 +3370,13 @@
     <row r="32" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B32" s="20"/>
       <c r="C32" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D32" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F32" s="12">
         <v>1</v>
@@ -3430,13 +3443,13 @@
     <row r="33" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B33" s="20"/>
       <c r="C33" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D33" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F33" s="12">
         <v>1</v>
@@ -3503,13 +3516,13 @@
     <row r="34" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B34" s="20"/>
       <c r="C34" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F34" s="12">
         <v>1</v>
@@ -3576,13 +3589,13 @@
     <row r="35" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B35" s="20"/>
       <c r="C35" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F35" s="12">
         <v>1</v>
@@ -3649,13 +3662,13 @@
     <row r="36" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B36" s="20"/>
       <c r="C36" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D36" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F36" s="12">
         <v>1</v>
@@ -3722,13 +3735,13 @@
     <row r="37" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B37" s="20"/>
       <c r="C37" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D37" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F37" s="12">
         <v>1</v>
@@ -3795,13 +3808,13 @@
     <row r="38" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B38" s="20"/>
       <c r="C38" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D38" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F38" s="12">
         <v>1</v>
@@ -3868,13 +3881,13 @@
     <row r="39" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B39" s="20"/>
       <c r="C39" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D39" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F39" s="12">
         <v>1</v>
@@ -3941,13 +3954,13 @@
     <row r="40" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B40" s="20"/>
       <c r="C40" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D40" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F40" s="12">
         <v>1</v>
@@ -4014,13 +4027,13 @@
     <row r="41" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B41" s="20"/>
       <c r="C41" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D41" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F41" s="12">
         <v>1</v>
@@ -4087,13 +4100,13 @@
     <row r="42" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B42" s="20"/>
       <c r="C42" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D42" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F42" s="12">
         <v>1</v>
@@ -4160,13 +4173,13 @@
     <row r="43" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B43" s="20"/>
       <c r="C43" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D43" s="11" t="s">
         <v>83</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F43" s="12">
         <v>1</v>

</xml_diff>

<commit_message>
Update hydro_example with additional files
</commit_message>
<xml_diff>
--- a/data/hydroExample/Power_HydroAssets.xlsx
+++ b/data/hydroExample/Power_HydroAssets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\hydroExample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9030A1EF-A120-43AC-8B64-B4D4D6CB149A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61F17E12-2723-458F-A215-44D9954CF8F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34230" yWindow="-21705" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario_2016" sheetId="1" r:id="rId1"/>
@@ -1805,8 +1805,8 @@
       <c r="R10" s="25">
         <v>1.1192385045596056E-2</v>
       </c>
-      <c r="S10" s="27">
-        <v>0</v>
+      <c r="S10" s="25">
+        <v>1.1192385045596056E-2</v>
       </c>
       <c r="T10" s="12">
         <v>0</v>
@@ -2535,8 +2535,8 @@
       <c r="R20" s="25">
         <v>0.32026898653096453</v>
       </c>
-      <c r="S20" s="25">
-        <v>0.32026898653096453</v>
+      <c r="S20" s="27">
+        <v>0</v>
       </c>
       <c r="T20" s="12">
         <v>0</v>

</xml_diff>

<commit_message>
Add storage level constraint
Setting storage level at the last k equal to the storage of the first k
</commit_message>
<xml_diff>
--- a/data/hydroExample/Power_HydroAssets.xlsx
+++ b/data/hydroExample/Power_HydroAssets.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\hydroExample\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth\Git\LEGO-Pyomo\data\hydroExample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67E1F8A9-FFA3-4A30-8416-4FB65BB104E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D245B9AC-96A0-44A8-889F-6A4B203A8264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34230" yWindow="-21705" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario_2016" sheetId="1" r:id="rId1"/>
@@ -750,7 +750,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1054,30 +1054,30 @@
     <tabColor rgb="FF008080"/>
   </sheetPr>
   <dimension ref="A1:AE43"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.5703125" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" customWidth="1"/>
-    <col min="3" max="3" width="29.85546875" customWidth="1"/>
-    <col min="4" max="6" width="15.7109375" customWidth="1"/>
-    <col min="7" max="7" width="17.42578125" customWidth="1"/>
-    <col min="8" max="9" width="15.7109375" customWidth="1"/>
-    <col min="10" max="12" width="21.7109375" customWidth="1"/>
-    <col min="13" max="16" width="15.7109375" customWidth="1"/>
-    <col min="17" max="17" width="20.7109375" customWidth="1"/>
-    <col min="18" max="18" width="20.42578125" customWidth="1"/>
-    <col min="19" max="19" width="20.5703125" customWidth="1"/>
-    <col min="20" max="21" width="15.7109375" customWidth="1"/>
-    <col min="22" max="23" width="20.7109375" customWidth="1"/>
-    <col min="24" max="24" width="22.7109375" customWidth="1"/>
-    <col min="25" max="25" width="15.7109375" customWidth="1"/>
-    <col min="26" max="27" width="20.140625" customWidth="1"/>
-    <col min="28" max="28" width="20.42578125" customWidth="1"/>
-    <col min="29" max="29" width="19.42578125" customWidth="1"/>
-    <col min="30" max="31" width="24.5703125" customWidth="1"/>
+    <col min="1" max="1" width="5.54296875" customWidth="1"/>
+    <col min="2" max="2" width="19.7265625" customWidth="1"/>
+    <col min="3" max="3" width="29.81640625" customWidth="1"/>
+    <col min="4" max="6" width="15.7265625" customWidth="1"/>
+    <col min="7" max="7" width="17.453125" customWidth="1"/>
+    <col min="8" max="9" width="15.7265625" customWidth="1"/>
+    <col min="10" max="12" width="21.7265625" customWidth="1"/>
+    <col min="13" max="16" width="15.7265625" customWidth="1"/>
+    <col min="17" max="17" width="20.7265625" customWidth="1"/>
+    <col min="18" max="18" width="20.453125" customWidth="1"/>
+    <col min="19" max="19" width="20.54296875" customWidth="1"/>
+    <col min="20" max="21" width="15.7265625" customWidth="1"/>
+    <col min="22" max="23" width="20.7265625" customWidth="1"/>
+    <col min="24" max="24" width="22.7265625" customWidth="1"/>
+    <col min="25" max="25" width="15.7265625" customWidth="1"/>
+    <col min="26" max="27" width="20.1796875" customWidth="1"/>
+    <col min="28" max="28" width="20.453125" customWidth="1"/>
+    <col min="29" max="29" width="19.453125" customWidth="1"/>
+    <col min="30" max="31" width="24.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:31" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>96</v>
@@ -1112,7 +1112,7 @@
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1120,7 +1120,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
@@ -1215,7 +1215,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
         <v>26</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:31" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7"/>
       <c r="B5" s="7" t="s">
         <v>39</v>
@@ -1403,7 +1403,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:31" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8"/>
       <c r="B6" s="8" t="s">
         <v>63</v>
@@ -1494,7 +1494,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A7" s="9"/>
       <c r="B7" s="9" t="s">
         <v>66</v>
@@ -1587,7 +1587,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A8" s="10"/>
       <c r="B8" s="19"/>
       <c r="C8" s="18" t="s">
@@ -1603,7 +1603,7 @@
         <v>1</v>
       </c>
       <c r="G8" s="22">
-        <v>517142.78610676009</v>
+        <v>18795.432911392403</v>
       </c>
       <c r="H8" s="13">
         <v>0</v>
@@ -1612,13 +1612,13 @@
         <v>0</v>
       </c>
       <c r="J8" s="22">
-        <v>5.0276250000000002E-5</v>
+        <v>1.3833147724009441E-3</v>
       </c>
       <c r="K8" s="14">
         <v>0</v>
       </c>
       <c r="L8" s="14">
-        <v>5000</v>
+        <v>225545.19493670884</v>
       </c>
       <c r="M8" s="13"/>
       <c r="N8" s="13"/>
@@ -1632,7 +1632,7 @@
         <v>0</v>
       </c>
       <c r="R8" s="22">
-        <v>4.4957730103030681E-3</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S8" s="24">
         <v>0</v>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="X8" s="13">
         <f>L8/G8</f>
-        <v>9.668509615384617E-3</v>
+        <v>12</v>
       </c>
       <c r="Y8" s="15"/>
       <c r="Z8" s="12">
@@ -1671,7 +1671,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A9" s="10"/>
       <c r="B9" s="19"/>
       <c r="C9" s="18" t="s">
@@ -1687,7 +1687,7 @@
         <v>1</v>
       </c>
       <c r="G9" s="22">
-        <v>13455657.492354739</v>
+        <v>76314.213344048214</v>
       </c>
       <c r="H9" s="13">
         <v>0</v>
@@ -1696,13 +1696,13 @@
         <v>0</v>
       </c>
       <c r="J9" s="22">
-        <v>2.4524999999999998E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K9" s="14">
         <v>0</v>
       </c>
       <c r="L9" s="14">
-        <v>5000</v>
+        <v>915770.56012857857</v>
       </c>
       <c r="M9" s="13"/>
       <c r="N9" s="13"/>
@@ -1716,7 +1716,7 @@
         <v>0</v>
       </c>
       <c r="R9" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S9" s="24">
         <v>0</v>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="X9" s="13">
         <f t="shared" ref="X9:X43" si="0">L9/G9</f>
-        <v>3.7159090909090909E-4</v>
+        <v>12</v>
       </c>
       <c r="Y9" s="15"/>
       <c r="Z9" s="12"/>
@@ -1753,7 +1753,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A10" s="10"/>
       <c r="B10" s="19"/>
       <c r="C10" s="18" t="s">
@@ -1769,7 +1769,7 @@
         <v>1</v>
       </c>
       <c r="G10" s="22">
-        <v>23105674.481821269</v>
+        <v>197455.68000000002</v>
       </c>
       <c r="H10" s="13">
         <v>0</v>
@@ -1778,13 +1778,13 @@
         <v>123.1396524</v>
       </c>
       <c r="J10" s="22">
-        <v>1.4715000000000002E-6</v>
+        <v>1.7219053916301622E-4</v>
       </c>
       <c r="K10" s="20">
         <v>1.6999999999999999E-3</v>
       </c>
       <c r="L10" s="14">
-        <v>5000</v>
+        <v>2369468.16</v>
       </c>
       <c r="M10" s="13"/>
       <c r="N10" s="13"/>
@@ -1798,10 +1798,10 @@
         <v>0</v>
       </c>
       <c r="R10" s="22">
-        <v>5.5961925227980276E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S10" s="22">
-        <v>1.1192385045596056E-2</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="T10" s="12">
         <v>0</v>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="X10" s="13">
         <f t="shared" si="0"/>
-        <v>2.1639705882352944E-4</v>
+        <v>12</v>
       </c>
       <c r="Y10" s="15"/>
       <c r="Z10" s="12">
@@ -1837,7 +1837,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A11" s="10"/>
       <c r="B11" s="19"/>
       <c r="C11" s="18" t="s">
@@ -1853,7 +1853,7 @@
         <v>1</v>
       </c>
       <c r="G11" s="22">
-        <v>6523955.147808359</v>
+        <v>117304.04284051221</v>
       </c>
       <c r="H11" s="13">
         <v>0</v>
@@ -1862,13 +1862,13 @@
         <v>0</v>
       </c>
       <c r="J11" s="22">
-        <v>2.4524999999999998E-6</v>
+        <v>1.3639768598388177E-4</v>
       </c>
       <c r="K11" s="14">
         <v>0</v>
       </c>
       <c r="L11" s="14">
-        <v>5000</v>
+        <v>1407648.5140861464</v>
       </c>
       <c r="M11" s="13"/>
       <c r="N11" s="13"/>
@@ -1882,7 +1882,7 @@
         <v>0</v>
       </c>
       <c r="R11" s="22">
-        <v>4.432924794476158E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S11" s="24">
         <v>0</v>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="X11" s="13">
         <f t="shared" si="0"/>
-        <v>7.6640624999999994E-4</v>
+        <v>11.999999999999998</v>
       </c>
       <c r="Y11" s="15"/>
       <c r="Z11" s="12">
@@ -1921,7 +1921,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A12" s="10"/>
       <c r="B12" s="19"/>
       <c r="C12" s="18" t="s">
@@ -1937,7 +1937,7 @@
         <v>1</v>
       </c>
       <c r="G12" s="22">
-        <v>8154943.9347604485</v>
+        <v>50876.142229365476</v>
       </c>
       <c r="H12" s="13">
         <v>0</v>
@@ -1946,13 +1946,13 @@
         <v>0</v>
       </c>
       <c r="J12" s="22">
-        <v>2.6977499999999997E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K12" s="14">
         <v>0</v>
       </c>
       <c r="L12" s="14">
-        <v>5000</v>
+        <v>610513.70675238571</v>
       </c>
       <c r="M12" s="13"/>
       <c r="N12" s="13"/>
@@ -1966,7 +1966,7 @@
         <v>0</v>
       </c>
       <c r="R12" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S12" s="24">
         <v>0</v>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="X12" s="13">
         <f t="shared" si="0"/>
-        <v>6.1312499999999995E-4</v>
+        <v>12</v>
       </c>
       <c r="Y12" s="15"/>
       <c r="Z12" s="12">
@@ -2005,7 +2005,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A13" s="10"/>
       <c r="B13" s="19"/>
       <c r="C13" s="18" t="s">
@@ -2021,7 +2021,7 @@
         <v>1</v>
       </c>
       <c r="G13" s="22">
-        <v>19571865.443425078</v>
+        <v>128145.67200000001</v>
       </c>
       <c r="H13" s="13">
         <v>0</v>
@@ -2030,13 +2030,13 @@
         <v>0</v>
       </c>
       <c r="J13" s="22">
-        <v>6.1312499999999995E-7</v>
+        <v>9.3643427926305622E-5</v>
       </c>
       <c r="K13" s="14">
         <v>0</v>
       </c>
       <c r="L13" s="14">
-        <v>5000</v>
+        <v>1537748.064</v>
       </c>
       <c r="M13" s="13"/>
       <c r="N13" s="13"/>
@@ -2050,7 +2050,7 @@
         <v>0</v>
       </c>
       <c r="R13" s="22">
-        <v>3.0434114076049329E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S13" s="24">
         <v>0</v>
@@ -2069,7 +2069,7 @@
       </c>
       <c r="X13" s="13">
         <f t="shared" si="0"/>
-        <v>2.5546875E-4</v>
+        <v>12</v>
       </c>
       <c r="Y13" s="15"/>
       <c r="Z13" s="12">
@@ -2089,7 +2089,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A14" s="10"/>
       <c r="B14" s="19"/>
       <c r="C14" s="18" t="s">
@@ -2105,7 +2105,7 @@
         <v>1</v>
       </c>
       <c r="G14" s="22">
-        <v>663774.50631771085</v>
+        <v>192549.84</v>
       </c>
       <c r="H14" s="13">
         <v>0</v>
@@ -2114,13 +2114,13 @@
         <v>0</v>
       </c>
       <c r="J14" s="22">
-        <v>2.1091500000000003E-5</v>
+        <v>7.2708447849138697E-5</v>
       </c>
       <c r="K14" s="14">
         <v>0</v>
       </c>
       <c r="L14" s="14">
-        <v>5000</v>
+        <v>2310598.08</v>
       </c>
       <c r="M14" s="13"/>
       <c r="N14" s="13"/>
@@ -2134,7 +2134,7 @@
         <v>0</v>
       </c>
       <c r="R14" s="22">
-        <v>2.3630245550970073E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S14" s="24">
         <v>0</v>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="X14" s="13">
         <f t="shared" si="0"/>
-        <v>7.5326785714285721E-3</v>
+        <v>12</v>
       </c>
       <c r="Y14" s="15"/>
       <c r="Z14" s="12">
@@ -2173,7 +2173,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A15" s="10"/>
       <c r="B15" s="19"/>
       <c r="C15" s="18" t="s">
@@ -2189,7 +2189,7 @@
         <v>1</v>
       </c>
       <c r="G15" s="22">
-        <v>691713.99446628802</v>
+        <v>168293.23855530474</v>
       </c>
       <c r="H15" s="13">
         <v>0</v>
@@ -2198,13 +2198,13 @@
         <v>0</v>
       </c>
       <c r="J15" s="22">
-        <v>2.7468000000000002E-5</v>
+        <v>1.12898177984472E-4</v>
       </c>
       <c r="K15" s="14">
         <v>0</v>
       </c>
       <c r="L15" s="14">
-        <v>5000</v>
+        <v>2019518.8626636569</v>
       </c>
       <c r="M15" s="13"/>
       <c r="N15" s="13"/>
@@ -2218,7 +2218,7 @@
         <v>0</v>
       </c>
       <c r="R15" s="22">
-        <v>3.6691907844953398E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S15" s="24">
         <v>0</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="X15" s="13">
         <f t="shared" si="0"/>
-        <v>7.2284210526315793E-3</v>
+        <v>12</v>
       </c>
       <c r="Y15" s="15"/>
       <c r="Z15" s="12">
@@ -2257,7 +2257,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A16" s="10"/>
       <c r="B16" s="19"/>
       <c r="C16" s="18" t="s">
@@ -2273,7 +2273,7 @@
         <v>1</v>
       </c>
       <c r="G16" s="22">
-        <v>607283.05897152273</v>
+        <v>735583.65842696629</v>
       </c>
       <c r="H16" s="13">
         <v>0</v>
@@ -2282,13 +2282,13 @@
         <v>0</v>
       </c>
       <c r="J16" s="22">
-        <v>2.3053500000000002E-5</v>
+        <v>1.9032505466392189E-5</v>
       </c>
       <c r="K16" s="14">
         <v>0</v>
       </c>
       <c r="L16" s="14">
-        <v>5000</v>
+        <v>8827003.9011235945</v>
       </c>
       <c r="M16" s="13"/>
       <c r="N16" s="13"/>
@@ -2302,7 +2302,7 @@
         <v>0</v>
       </c>
       <c r="R16" s="22">
-        <v>6.1855642765774616E-5</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S16" s="24">
         <v>0</v>
@@ -2321,7 +2321,7 @@
       </c>
       <c r="X16" s="13">
         <f t="shared" si="0"/>
-        <v>8.2333928571428575E-3</v>
+        <v>11.999999999999998</v>
       </c>
       <c r="Y16" s="15"/>
       <c r="Z16" s="12">
@@ -2341,7 +2341,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A17" s="10"/>
       <c r="B17" s="19"/>
       <c r="C17" s="18" t="s">
@@ -2357,7 +2357,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="22">
-        <v>690033.71755665331</v>
+        <v>184888.02933333334</v>
       </c>
       <c r="H17" s="13">
         <v>0</v>
@@ -2366,13 +2366,13 @@
         <v>0</v>
       </c>
       <c r="J17" s="22">
-        <v>1.5941249999999999E-5</v>
+        <v>5.9495468904415532E-5</v>
       </c>
       <c r="K17" s="14">
         <v>0</v>
       </c>
       <c r="L17" s="14">
-        <v>5000</v>
+        <v>2218656.352</v>
       </c>
       <c r="M17" s="13"/>
       <c r="N17" s="13"/>
@@ -2386,7 +2386,7 @@
         <v>0</v>
       </c>
       <c r="R17" s="22">
-        <v>1.9336027393935048E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S17" s="24">
         <v>0</v>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="X17" s="13">
         <f t="shared" si="0"/>
-        <v>7.2460227272727277E-3</v>
+        <v>12</v>
       </c>
       <c r="Y17" s="15"/>
       <c r="Z17" s="12">
@@ -2425,7 +2425,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A18" s="10"/>
       <c r="B18" s="19"/>
       <c r="C18" s="18" t="s">
@@ -2441,7 +2441,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="22">
-        <v>744033.54456319555</v>
+        <v>169397.1903512195</v>
       </c>
       <c r="H18" s="13">
         <v>0</v>
@@ -2450,13 +2450,13 @@
         <v>0</v>
       </c>
       <c r="J18" s="22">
-        <v>2.3789249999999999E-5</v>
+        <v>1.0448815569668966E-4</v>
       </c>
       <c r="K18" s="14">
         <v>0</v>
       </c>
       <c r="L18" s="14">
-        <v>5000</v>
+        <v>2032766.284214634</v>
       </c>
       <c r="M18" s="13"/>
       <c r="N18" s="13"/>
@@ -2470,7 +2470,7 @@
         <v>0</v>
       </c>
       <c r="R18" s="22">
-        <v>3.3958650601424142E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S18" s="24">
         <v>0</v>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="X18" s="13">
         <f t="shared" si="0"/>
-        <v>6.7201271186440679E-3</v>
+        <v>12</v>
       </c>
       <c r="Y18" s="15"/>
       <c r="Z18" s="12"/>
@@ -2507,7 +2507,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A19" s="10"/>
       <c r="B19" s="19"/>
       <c r="C19" s="18" t="s">
@@ -2523,7 +2523,7 @@
         <v>1</v>
       </c>
       <c r="G19" s="22">
-        <v>2446483.1804281347</v>
+        <v>13875.311517099675</v>
       </c>
       <c r="H19" s="13">
         <v>0</v>
@@ -2532,13 +2532,13 @@
         <v>0</v>
       </c>
       <c r="J19" s="22">
-        <v>2.4524999999999998E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K19" s="14">
         <v>0</v>
       </c>
       <c r="L19" s="14">
-        <v>5000</v>
+        <v>166503.7382051961</v>
       </c>
       <c r="M19" s="13"/>
       <c r="N19" s="13"/>
@@ -2552,7 +2552,7 @@
         <v>0</v>
       </c>
       <c r="R19" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S19" s="24">
         <v>0</v>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="X19" s="13">
         <f t="shared" si="0"/>
-        <v>2.04375E-3</v>
+        <v>12</v>
       </c>
       <c r="Y19" s="15"/>
       <c r="Z19" s="12"/>
@@ -2589,7 +2589,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A20" s="10"/>
       <c r="B20" s="19"/>
       <c r="C20" s="18" t="s">
@@ -2605,7 +2605,7 @@
         <v>1</v>
       </c>
       <c r="G20" s="22">
-        <v>848114.16921508661</v>
+        <v>21107.257600000001</v>
       </c>
       <c r="H20" s="13">
         <v>0</v>
@@ -2614,7 +2614,7 @@
         <v>0</v>
       </c>
       <c r="J20" s="22">
-        <v>1.2262500000000001E-4</v>
+        <v>4.9272151773994549E-3</v>
       </c>
       <c r="K20" s="14">
         <v>0</v>
@@ -2634,7 +2634,7 @@
         <v>1</v>
       </c>
       <c r="R20" s="22">
-        <v>1.6013449326548225E-2</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S20" s="24">
         <v>0</v>
@@ -2653,7 +2653,7 @@
       </c>
       <c r="X20" s="13">
         <f t="shared" si="0"/>
-        <v>17.686298076923077</v>
+        <v>710.65603520184447</v>
       </c>
       <c r="Y20" s="15"/>
       <c r="Z20" s="12"/>
@@ -2671,7 +2671,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A21" s="10"/>
       <c r="B21" s="19"/>
       <c r="C21" s="18" t="s">
@@ -2687,7 +2687,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="22">
-        <v>691713.99446628802</v>
+        <v>183607.69530845954</v>
       </c>
       <c r="H21" s="13">
         <v>0</v>
@@ -2696,13 +2696,13 @@
         <v>0</v>
       </c>
       <c r="J21" s="22">
-        <v>2.7468000000000002E-5</v>
+        <v>1.0348150151375814E-4</v>
       </c>
       <c r="K21" s="14">
         <v>0</v>
       </c>
       <c r="L21" s="14">
-        <v>5000</v>
+        <v>2203292.3437015144</v>
       </c>
       <c r="M21" s="13"/>
       <c r="N21" s="13"/>
@@ -2716,7 +2716,7 @@
         <v>0</v>
       </c>
       <c r="R21" s="22">
-        <v>3.3631487991971396E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S21" s="24">
         <v>0</v>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="X21" s="13">
         <f t="shared" si="0"/>
-        <v>7.2284210526315793E-3</v>
+        <v>12</v>
       </c>
       <c r="Y21" s="15"/>
       <c r="Z21" s="12">
@@ -2755,7 +2755,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A22" s="10"/>
       <c r="B22" s="19"/>
       <c r="C22" s="18" t="s">
@@ -2771,7 +2771,7 @@
         <v>1</v>
       </c>
       <c r="G22" s="22">
-        <v>853424.36526562821</v>
+        <v>122730.03966942149</v>
       </c>
       <c r="H22" s="13">
         <v>0</v>
@@ -2780,13 +2780,13 @@
         <v>0</v>
       </c>
       <c r="J22" s="22">
-        <v>2.1091500000000003E-5</v>
+        <v>1.4666336007454863E-4</v>
       </c>
       <c r="K22" s="14">
         <v>0</v>
       </c>
       <c r="L22" s="14">
-        <v>5000</v>
+        <v>1472760.4760330578</v>
       </c>
       <c r="M22" s="13"/>
       <c r="N22" s="13"/>
@@ -2800,7 +2800,7 @@
         <v>0</v>
       </c>
       <c r="R22" s="22">
-        <v>4.7665592024228302E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S22" s="24">
         <v>0</v>
@@ -2819,7 +2819,7 @@
       </c>
       <c r="X22" s="13">
         <f t="shared" si="0"/>
-        <v>5.8587500000000011E-3</v>
+        <v>12</v>
       </c>
       <c r="Y22" s="15"/>
       <c r="Z22" s="12">
@@ -2839,7 +2839,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A23" s="10"/>
       <c r="B23" s="19"/>
       <c r="C23" s="18" t="s">
@@ -2855,7 +2855,7 @@
         <v>1</v>
       </c>
       <c r="G23" s="22">
-        <v>399752.15366472787</v>
+        <v>111471.04648390942</v>
       </c>
       <c r="H23" s="13">
         <v>0</v>
@@ -2864,13 +2864,13 @@
         <v>0</v>
       </c>
       <c r="J23" s="22">
-        <v>2.5015500000000001E-5</v>
+        <v>8.9709393743275537E-5</v>
       </c>
       <c r="K23" s="14">
         <v>0</v>
       </c>
       <c r="L23" s="14">
-        <v>5000</v>
+        <v>1337652.557806913</v>
       </c>
       <c r="M23" s="13"/>
       <c r="N23" s="13"/>
@@ -2884,7 +2884,7 @@
         <v>0</v>
       </c>
       <c r="R23" s="22">
-        <v>2.9155552966564547E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S23" s="24">
         <v>0</v>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="X23" s="13">
         <f t="shared" si="0"/>
-        <v>1.250775E-2</v>
+        <v>12</v>
       </c>
       <c r="Y23" s="15"/>
       <c r="Z23" s="12">
@@ -2923,7 +2923,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A24" s="10"/>
       <c r="B24" s="19"/>
       <c r="C24" s="18" t="s">
@@ -2939,7 +2939,7 @@
         <v>1</v>
       </c>
       <c r="G24" s="22">
-        <v>5096839.9592252802</v>
+        <v>146262.2694969576</v>
       </c>
       <c r="H24" s="13">
         <v>0</v>
@@ -2948,13 +2948,13 @@
         <v>0</v>
       </c>
       <c r="J24" s="22">
-        <v>1.962E-6</v>
+        <v>6.8370332515645875E-5</v>
       </c>
       <c r="K24" s="14">
         <v>0</v>
       </c>
       <c r="L24" s="14">
-        <v>5000</v>
+        <v>1755147.2339634912</v>
       </c>
       <c r="M24" s="13"/>
       <c r="N24" s="13"/>
@@ -2968,7 +2968,7 @@
         <v>0</v>
       </c>
       <c r="R24" s="22">
-        <v>2.2220358067584909E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S24" s="24">
         <v>0</v>
@@ -2987,7 +2987,7 @@
       </c>
       <c r="X24" s="13">
         <f t="shared" si="0"/>
-        <v>9.810000000000001E-4</v>
+        <v>12</v>
       </c>
       <c r="Y24" s="15"/>
       <c r="Z24" s="12"/>
@@ -3005,7 +3005,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A25" s="10"/>
       <c r="B25" s="19"/>
       <c r="C25" s="18" t="s">
@@ -3021,7 +3021,7 @@
         <v>1</v>
       </c>
       <c r="G25" s="22">
-        <v>6625891.9469928648</v>
+        <v>30063.174953715963</v>
       </c>
       <c r="H25" s="13">
         <v>0</v>
@@ -3030,13 +3030,13 @@
         <v>0</v>
       </c>
       <c r="J25" s="22">
-        <v>1.962E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K25" s="14">
         <v>0</v>
       </c>
       <c r="L25" s="14">
-        <v>5000</v>
+        <v>360758.09944459156</v>
       </c>
       <c r="M25" s="13"/>
       <c r="N25" s="13"/>
@@ -3050,7 +3050,7 @@
         <v>0</v>
       </c>
       <c r="R25" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S25" s="24">
         <v>0</v>
@@ -3069,7 +3069,7 @@
       </c>
       <c r="X25" s="13">
         <f t="shared" si="0"/>
-        <v>7.5461538461538461E-4</v>
+        <v>12</v>
       </c>
       <c r="Y25" s="15"/>
       <c r="Z25" s="12"/>
@@ -3087,7 +3087,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A26" s="10"/>
       <c r="B26" s="19"/>
       <c r="C26" s="18" t="s">
@@ -3103,7 +3103,7 @@
         <v>1</v>
       </c>
       <c r="G26" s="22">
-        <v>6116207.9510703366</v>
+        <v>34688.278792749188</v>
       </c>
       <c r="H26" s="13">
         <v>0</v>
@@ -3112,13 +3112,13 @@
         <v>0</v>
       </c>
       <c r="J26" s="22">
-        <v>2.4524999999999998E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K26" s="14">
         <v>0</v>
       </c>
       <c r="L26" s="14">
-        <v>5000000</v>
+        <v>416259.34551299026</v>
       </c>
       <c r="M26" s="13"/>
       <c r="N26" s="13"/>
@@ -3132,7 +3132,7 @@
         <v>1</v>
       </c>
       <c r="R26" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S26" s="24">
         <v>0</v>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="X26" s="13">
         <f t="shared" si="0"/>
-        <v>0.8175</v>
+        <v>12</v>
       </c>
       <c r="Y26" s="15"/>
       <c r="Z26" s="12"/>
@@ -3169,7 +3169,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A27" s="10"/>
       <c r="B27" s="19"/>
       <c r="C27" s="18" t="s">
@@ -3185,7 +3185,7 @@
         <v>1</v>
       </c>
       <c r="G27" s="22">
-        <v>5889681.730660324</v>
+        <v>131944.51443052923</v>
       </c>
       <c r="H27" s="13">
         <v>0</v>
@@ -3194,13 +3194,13 @@
         <v>0</v>
       </c>
       <c r="J27" s="22">
-        <v>2.2072499999999999E-6</v>
+        <v>9.8526263529088916E-5</v>
       </c>
       <c r="K27" s="14">
         <v>0</v>
       </c>
       <c r="L27" s="14">
-        <v>5000</v>
+        <v>1583334.1731663509</v>
       </c>
       <c r="M27" s="13"/>
       <c r="N27" s="13"/>
@@ -3214,7 +3214,7 @@
         <v>0</v>
       </c>
       <c r="R27" s="22">
-        <v>3.2021035646953897E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S27" s="24">
         <v>0</v>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="X27" s="13">
         <f t="shared" si="0"/>
-        <v>8.4894230769230771E-4</v>
+        <v>12</v>
       </c>
       <c r="Y27" s="15"/>
       <c r="Z27" s="12">
@@ -3253,7 +3253,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A28" s="10"/>
       <c r="B28" s="19"/>
       <c r="C28" s="18" t="s">
@@ -3269,7 +3269,7 @@
         <v>1</v>
       </c>
       <c r="G28" s="22">
-        <v>9637661.0138078034</v>
+        <v>60126.349907431926</v>
       </c>
       <c r="H28" s="13">
         <v>0</v>
@@ -3278,13 +3278,13 @@
         <v>0</v>
       </c>
       <c r="J28" s="22">
-        <v>2.6977499999999997E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K28" s="14">
         <v>0</v>
       </c>
       <c r="L28" s="14">
-        <v>5000</v>
+        <v>721516.19888918311</v>
       </c>
       <c r="M28" s="13"/>
       <c r="N28" s="13"/>
@@ -3298,7 +3298,7 @@
         <v>0</v>
       </c>
       <c r="R28" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S28" s="24">
         <v>0</v>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="X28" s="13">
         <f t="shared" si="0"/>
-        <v>5.1879807692307685E-4</v>
+        <v>12</v>
       </c>
       <c r="Y28" s="15"/>
       <c r="Z28" s="12">
@@ -3337,7 +3337,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A29" s="10"/>
       <c r="B29" s="19"/>
       <c r="C29" s="18" t="s">
@@ -3353,7 +3353,7 @@
         <v>1</v>
       </c>
       <c r="G29" s="22">
-        <v>815494.39347604488</v>
+        <v>4625.1038390332251</v>
       </c>
       <c r="H29" s="13">
         <v>0</v>
@@ -3362,13 +3362,13 @@
         <v>0</v>
       </c>
       <c r="J29" s="22">
-        <v>2.4524999999999998E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K29" s="14">
         <v>0</v>
       </c>
       <c r="L29" s="14">
-        <v>5000</v>
+        <v>55501.246068398701</v>
       </c>
       <c r="M29" s="13"/>
       <c r="N29" s="13"/>
@@ -3382,7 +3382,7 @@
         <v>0</v>
       </c>
       <c r="R29" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S29" s="24">
         <v>0</v>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="X29" s="13">
         <f t="shared" si="0"/>
-        <v>6.1312499999999995E-3</v>
+        <v>12</v>
       </c>
       <c r="Y29" s="15"/>
       <c r="Z29" s="12"/>
@@ -3419,7 +3419,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A30" s="10"/>
       <c r="B30" s="19"/>
       <c r="C30" s="18" t="s">
@@ -3435,7 +3435,7 @@
         <v>1</v>
       </c>
       <c r="G30" s="22">
-        <v>6342734.1714803493</v>
+        <v>179073.80465116279</v>
       </c>
       <c r="H30" s="13">
         <v>0</v>
@@ -3444,13 +3444,13 @@
         <v>0</v>
       </c>
       <c r="J30" s="22">
-        <v>2.2072499999999999E-6</v>
+        <v>7.8180055576928815E-5</v>
       </c>
       <c r="K30" s="14">
         <v>0</v>
       </c>
       <c r="L30" s="14">
-        <v>5000</v>
+        <v>2148885.6558139534</v>
       </c>
       <c r="M30" s="13"/>
       <c r="N30" s="13"/>
@@ -3464,7 +3464,7 @@
         <v>0</v>
       </c>
       <c r="R30" s="22">
-        <v>2.5408518062501861E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S30" s="24">
         <v>0</v>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="X30" s="13">
         <f t="shared" si="0"/>
-        <v>7.8830357142857142E-4</v>
+        <v>12</v>
       </c>
       <c r="Y30" s="15"/>
       <c r="Z30" s="12"/>
@@ -3501,7 +3501,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="31" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A31" s="10"/>
       <c r="B31" s="19"/>
       <c r="C31" s="18" t="s">
@@ -3517,7 +3517,7 @@
         <v>1</v>
       </c>
       <c r="G31" s="22">
-        <v>407747.19673802244</v>
+        <v>2312.5519195166125</v>
       </c>
       <c r="H31" s="13">
         <v>0</v>
@@ -3526,13 +3526,13 @@
         <v>0</v>
       </c>
       <c r="J31" s="22">
-        <v>2.4524999999999998E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K31" s="14">
         <v>0</v>
       </c>
       <c r="L31" s="14">
-        <v>5000</v>
+        <v>27750.623034199351</v>
       </c>
       <c r="M31" s="13"/>
       <c r="N31" s="13"/>
@@ -3546,7 +3546,7 @@
         <v>0</v>
       </c>
       <c r="R31" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S31" s="24">
         <v>0</v>
@@ -3565,7 +3565,7 @@
       </c>
       <c r="X31" s="13">
         <f t="shared" si="0"/>
-        <v>1.2262499999999999E-2</v>
+        <v>12</v>
       </c>
       <c r="Y31" s="15"/>
       <c r="Z31" s="12"/>
@@ -3583,7 +3583,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="32" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A32" s="10"/>
       <c r="B32" s="19"/>
       <c r="C32" s="18" t="s">
@@ -3599,7 +3599,7 @@
         <v>1</v>
       </c>
       <c r="G32" s="22">
-        <v>768219.35617308575</v>
+        <v>204734.74925373134</v>
       </c>
       <c r="H32" s="13">
         <v>0</v>
@@ -3608,13 +3608,13 @@
         <v>0</v>
       </c>
       <c r="J32" s="22">
-        <v>1.6922249999999999E-5</v>
+        <v>6.3496793032866511E-5</v>
       </c>
       <c r="K32" s="14">
         <v>0</v>
       </c>
       <c r="L32" s="14">
-        <v>5000</v>
+        <v>2456816.991044776</v>
       </c>
       <c r="M32" s="13"/>
       <c r="N32" s="13"/>
@@ -3628,7 +3628,7 @@
         <v>0</v>
       </c>
       <c r="R32" s="22">
-        <v>2.0636457735681617E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S32" s="24">
         <v>0</v>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="X32" s="13">
         <f t="shared" si="0"/>
-        <v>6.508557692307692E-3</v>
+        <v>12</v>
       </c>
       <c r="Y32" s="15"/>
       <c r="Z32" s="12">
@@ -3667,7 +3667,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="33" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A33" s="10"/>
       <c r="B33" s="19"/>
       <c r="C33" s="18" t="s">
@@ -3683,7 +3683,7 @@
         <v>1</v>
       </c>
       <c r="G33" s="22">
-        <v>287821.55063860409</v>
+        <v>37022.94</v>
       </c>
       <c r="H33" s="13">
         <v>0</v>
@@ -3692,13 +3692,13 @@
         <v>0</v>
       </c>
       <c r="J33" s="22">
-        <v>2.0846250000000001E-5</v>
+        <v>1.6206168391813292E-4</v>
       </c>
       <c r="K33" s="14">
         <v>0</v>
       </c>
       <c r="L33" s="14">
-        <v>5000</v>
+        <v>444275.28</v>
       </c>
       <c r="M33" s="13"/>
       <c r="N33" s="13"/>
@@ -3712,7 +3712,7 @@
         <v>0</v>
       </c>
       <c r="R33" s="22">
-        <v>5.2670047273393192E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S33" s="24">
         <v>0</v>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="X33" s="13">
         <f t="shared" si="0"/>
-        <v>1.7371874999999998E-2</v>
+        <v>12</v>
       </c>
       <c r="Y33" s="15"/>
       <c r="Z33" s="12">
@@ -3751,7 +3751,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="34" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A34" s="10"/>
       <c r="B34" s="19"/>
       <c r="C34" s="18" t="s">
@@ -3767,7 +3767,7 @@
         <v>1</v>
       </c>
       <c r="G34" s="22">
-        <v>6523955.147808359</v>
+        <v>37000.830712265801</v>
       </c>
       <c r="H34" s="13">
         <v>0</v>
@@ -3776,13 +3776,13 @@
         <v>0</v>
       </c>
       <c r="J34" s="22">
-        <v>2.4524999999999998E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K34" s="14">
         <v>0</v>
       </c>
       <c r="L34" s="14">
-        <v>5000</v>
+        <v>444009.96854718961</v>
       </c>
       <c r="M34" s="13"/>
       <c r="N34" s="13"/>
@@ -3796,7 +3796,7 @@
         <v>0</v>
       </c>
       <c r="R34" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S34" s="24">
         <v>0</v>
@@ -3815,7 +3815,7 @@
       </c>
       <c r="X34" s="13">
         <f t="shared" si="0"/>
-        <v>7.6640624999999994E-4</v>
+        <v>12</v>
       </c>
       <c r="Y34" s="15"/>
       <c r="Z34" s="12"/>
@@ -3833,7 +3833,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="35" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A35" s="10"/>
       <c r="B35" s="19"/>
       <c r="C35" s="18" t="s">
@@ -3849,7 +3849,7 @@
         <v>1</v>
       </c>
       <c r="G35" s="22">
-        <v>4892966.3608562695</v>
+        <v>27750.623034199351</v>
       </c>
       <c r="H35" s="13">
         <v>0</v>
@@ -3858,13 +3858,13 @@
         <v>0</v>
       </c>
       <c r="J35" s="22">
-        <v>2.4524999999999998E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K35" s="14">
         <v>0</v>
       </c>
       <c r="L35" s="14">
-        <v>5000</v>
+        <v>333007.47641039221</v>
       </c>
       <c r="M35" s="13"/>
       <c r="N35" s="13"/>
@@ -3878,7 +3878,7 @@
         <v>0</v>
       </c>
       <c r="R35" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S35" s="24">
         <v>0</v>
@@ -3897,7 +3897,7 @@
       </c>
       <c r="X35" s="13">
         <f t="shared" si="0"/>
-        <v>1.021875E-3</v>
+        <v>12</v>
       </c>
       <c r="Y35" s="15"/>
       <c r="Z35" s="12"/>
@@ -3915,7 +3915,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="36" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A36" s="10"/>
       <c r="B36" s="19"/>
       <c r="C36" s="18" t="s">
@@ -3931,7 +3931,7 @@
         <v>1</v>
       </c>
       <c r="G36" s="22">
-        <v>407747.19673802244</v>
+        <v>2312.5519195166125</v>
       </c>
       <c r="H36" s="13">
         <v>0</v>
@@ -3940,13 +3940,13 @@
         <v>0</v>
       </c>
       <c r="J36" s="22">
-        <v>2.4524999999999998E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K36" s="14">
         <v>0</v>
       </c>
       <c r="L36" s="14">
-        <v>5000</v>
+        <v>27750.623034199351</v>
       </c>
       <c r="M36" s="13"/>
       <c r="N36" s="13"/>
@@ -3960,7 +3960,7 @@
         <v>0</v>
       </c>
       <c r="R36" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S36" s="24">
         <v>0</v>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="X36" s="13">
         <f t="shared" si="0"/>
-        <v>1.2262499999999999E-2</v>
+        <v>12</v>
       </c>
       <c r="Y36" s="15"/>
       <c r="Z36" s="12"/>
@@ -3997,7 +3997,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="37" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A37" s="10"/>
       <c r="B37" s="19"/>
       <c r="C37" s="18" t="s">
@@ -4013,7 +4013,7 @@
         <v>1</v>
       </c>
       <c r="G37" s="22">
-        <v>407747.19673802244</v>
+        <v>2312.5519195166125</v>
       </c>
       <c r="H37" s="13">
         <v>0</v>
@@ -4022,13 +4022,13 @@
         <v>0</v>
       </c>
       <c r="J37" s="22">
-        <v>2.4524999999999998E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K37" s="14">
         <v>0</v>
       </c>
       <c r="L37" s="14">
-        <v>5000</v>
+        <v>27750.623034199351</v>
       </c>
       <c r="M37" s="13"/>
       <c r="N37" s="13"/>
@@ -4042,7 +4042,7 @@
         <v>0</v>
       </c>
       <c r="R37" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S37" s="24">
         <v>0</v>
@@ -4061,7 +4061,7 @@
       </c>
       <c r="X37" s="13">
         <f t="shared" si="0"/>
-        <v>1.2262499999999999E-2</v>
+        <v>12</v>
       </c>
       <c r="Y37" s="15"/>
       <c r="Z37" s="12"/>
@@ -4079,7 +4079,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="38" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A38" s="10"/>
       <c r="B38" s="19"/>
       <c r="C38" s="18" t="s">
@@ -4095,7 +4095,7 @@
         <v>1</v>
       </c>
       <c r="G38" s="22">
-        <v>6301547.5859512556</v>
+        <v>39313.382631782413</v>
       </c>
       <c r="H38" s="13">
         <v>0</v>
@@ -4104,13 +4104,13 @@
         <v>0</v>
       </c>
       <c r="J38" s="22">
-        <v>2.6977499999999997E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K38" s="14">
         <v>0</v>
       </c>
       <c r="L38" s="14">
-        <v>5000</v>
+        <v>471760.59158138896</v>
       </c>
       <c r="M38" s="13"/>
       <c r="N38" s="13"/>
@@ -4124,7 +4124,7 @@
         <v>0</v>
       </c>
       <c r="R38" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S38" s="24">
         <v>0</v>
@@ -4143,7 +4143,7 @@
       </c>
       <c r="X38" s="13">
         <f t="shared" si="0"/>
-        <v>7.9345588235294113E-4</v>
+        <v>12</v>
       </c>
       <c r="Y38" s="15"/>
       <c r="Z38" s="12">
@@ -4163,7 +4163,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="39" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A39" s="10"/>
       <c r="B39" s="19"/>
       <c r="C39" s="18" t="s">
@@ -4179,7 +4179,7 @@
         <v>1</v>
       </c>
       <c r="G39" s="22">
-        <v>407747.19673802244</v>
+        <v>2312.5519195166125</v>
       </c>
       <c r="H39" s="13">
         <v>0</v>
@@ -4188,13 +4188,13 @@
         <v>0</v>
       </c>
       <c r="J39" s="22">
-        <v>2.4524999999999998E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K39" s="14">
         <v>0</v>
       </c>
       <c r="L39" s="14">
-        <v>5000</v>
+        <v>27750.623034199351</v>
       </c>
       <c r="M39" s="13"/>
       <c r="N39" s="13"/>
@@ -4208,7 +4208,7 @@
         <v>0</v>
       </c>
       <c r="R39" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S39" s="24">
         <v>0</v>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="X39" s="13">
         <f t="shared" si="0"/>
-        <v>1.2262499999999999E-2</v>
+        <v>12</v>
       </c>
       <c r="Y39" s="15"/>
       <c r="Z39" s="12"/>
@@ -4245,7 +4245,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="40" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A40" s="10"/>
       <c r="B40" s="19"/>
       <c r="C40" s="18" t="s">
@@ -4261,7 +4261,7 @@
         <v>1</v>
       </c>
       <c r="G40" s="22">
-        <v>1997961.26401631</v>
+        <v>11331.504405631402</v>
       </c>
       <c r="H40" s="13">
         <v>0</v>
@@ -4270,13 +4270,13 @@
         <v>0</v>
       </c>
       <c r="J40" s="22">
-        <v>2.4524999999999998E-6</v>
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K40" s="14">
         <v>0</v>
       </c>
       <c r="L40" s="14">
-        <v>5000</v>
+        <v>135978.05286757683</v>
       </c>
       <c r="M40" s="13"/>
       <c r="N40" s="13"/>
@@ -4290,7 +4290,7 @@
         <v>0</v>
       </c>
       <c r="R40" s="22">
-        <v>6.4282864637126621E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S40" s="24">
         <v>0</v>
@@ -4309,7 +4309,7 @@
       </c>
       <c r="X40" s="13">
         <f t="shared" si="0"/>
-        <v>2.502551020408163E-3</v>
+        <v>12</v>
       </c>
       <c r="Y40" s="15"/>
       <c r="Z40" s="12">
@@ -4329,7 +4329,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="41" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A41" s="10"/>
       <c r="B41" s="19"/>
       <c r="C41" s="18" t="s">
@@ -4345,7 +4345,7 @@
         <v>1</v>
       </c>
       <c r="G41" s="22">
-        <v>16059.361825050113</v>
+        <v>9898.1018181818181</v>
       </c>
       <c r="H41" s="13">
         <v>0</v>
@@ -4354,13 +4354,13 @@
         <v>0</v>
       </c>
       <c r="J41" s="22">
-        <v>6.2268974999999999E-4</v>
+        <v>1.010294719501774E-3</v>
       </c>
       <c r="K41" s="14">
         <v>0</v>
       </c>
       <c r="L41" s="14">
-        <v>5000</v>
+        <v>118777.22181818182</v>
       </c>
       <c r="M41" s="13"/>
       <c r="N41" s="13"/>
@@ -4374,7 +4374,7 @@
         <v>0</v>
       </c>
       <c r="R41" s="22">
-        <v>3.2834578383807655E-3</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S41" s="24">
         <v>0</v>
@@ -4393,7 +4393,7 @@
       </c>
       <c r="X41" s="13">
         <f t="shared" si="0"/>
-        <v>0.31134487500000002</v>
+        <v>12</v>
       </c>
       <c r="Y41" s="15"/>
       <c r="Z41" s="12">
@@ -4413,7 +4413,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="42" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A42" s="10"/>
       <c r="B42" s="19"/>
       <c r="C42" s="18" t="s">
@@ -4429,7 +4429,7 @@
         <v>1</v>
       </c>
       <c r="G42" s="22">
-        <v>49826.54135291517</v>
+        <v>355388.97599999997</v>
       </c>
       <c r="H42" s="13">
         <v>0</v>
@@ -4438,13 +4438,13 @@
         <v>0</v>
       </c>
       <c r="J42" s="22">
-        <v>6.0208875000000001E-4</v>
+        <v>8.4414548638109697E-5</v>
       </c>
       <c r="K42" s="14">
         <v>0</v>
       </c>
       <c r="L42" s="14">
-        <v>5000</v>
+        <v>4264667.7119999994</v>
       </c>
       <c r="M42" s="13"/>
       <c r="N42" s="13"/>
@@ -4458,7 +4458,7 @@
         <v>0</v>
       </c>
       <c r="R42" s="22">
-        <v>2.7434728307385649E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S42" s="24">
         <v>0</v>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="X42" s="13">
         <f t="shared" si="0"/>
-        <v>0.10034812499999998</v>
+        <v>12</v>
       </c>
       <c r="Y42" s="15"/>
       <c r="Z42" s="12">
@@ -4497,7 +4497,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="43" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A43" s="10"/>
       <c r="B43" s="19"/>
       <c r="C43" s="18" t="s">
@@ -4513,7 +4513,7 @@
         <v>1</v>
       </c>
       <c r="G43" s="22">
-        <v>949548.26637621643</v>
+        <v>180286.82497297297</v>
       </c>
       <c r="H43" s="13">
         <v>0</v>
@@ -4522,13 +4522,13 @@
         <v>0</v>
       </c>
       <c r="J43" s="22">
-        <v>1.7903250000000002E-5</v>
+        <v>9.4294189287256525E-5</v>
       </c>
       <c r="K43" s="14">
         <v>0</v>
       </c>
       <c r="L43" s="14">
-        <v>5000</v>
+        <v>2163441.8996756757</v>
       </c>
       <c r="M43" s="13"/>
       <c r="N43" s="13"/>
@@ -4542,7 +4542,7 @@
         <v>0</v>
       </c>
       <c r="R43" s="22">
-        <v>3.0645611518358368E-4</v>
+        <v>2.3328773748481666E-5</v>
       </c>
       <c r="S43" s="24">
         <v>0</v>
@@ -4561,7 +4561,7 @@
       </c>
       <c r="X43" s="13">
         <f t="shared" si="0"/>
-        <v>5.2656617647058833E-3</v>
+        <v>12</v>
       </c>
       <c r="Y43" s="15"/>
       <c r="Z43" s="12">

</xml_diff>

<commit_message>
Adjust Storage capacity, turbine factor, Omvar cost, inflow file
</commit_message>
<xml_diff>
--- a/data/hydroExample/Power_HydroAssets.xlsx
+++ b/data/hydroExample/Power_HydroAssets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth\Git\LEGO-Pyomo\data\hydroExample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D245B9AC-96A0-44A8-889F-6A4B203A8264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9749FC6-1F5D-4DBB-B7E0-B6D1C872347C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1632,7 +1632,7 @@
         <v>0</v>
       </c>
       <c r="R8" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S8" s="24">
         <v>0</v>
@@ -1716,7 +1716,7 @@
         <v>0</v>
       </c>
       <c r="R9" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S9" s="24">
         <v>0</v>
@@ -1798,10 +1798,10 @@
         <v>0</v>
       </c>
       <c r="R10" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S10" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="T10" s="12">
         <v>0</v>
@@ -1882,7 +1882,7 @@
         <v>0</v>
       </c>
       <c r="R11" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S11" s="24">
         <v>0</v>
@@ -1966,7 +1966,7 @@
         <v>0</v>
       </c>
       <c r="R12" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S12" s="24">
         <v>0</v>
@@ -2050,7 +2050,7 @@
         <v>0</v>
       </c>
       <c r="R13" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S13" s="24">
         <v>0</v>
@@ -2134,7 +2134,7 @@
         <v>0</v>
       </c>
       <c r="R14" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S14" s="24">
         <v>0</v>
@@ -2218,7 +2218,7 @@
         <v>0</v>
       </c>
       <c r="R15" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S15" s="24">
         <v>0</v>
@@ -2302,7 +2302,7 @@
         <v>0</v>
       </c>
       <c r="R16" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S16" s="24">
         <v>0</v>
@@ -2386,7 +2386,7 @@
         <v>0</v>
       </c>
       <c r="R17" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S17" s="24">
         <v>0</v>
@@ -2470,7 +2470,7 @@
         <v>0</v>
       </c>
       <c r="R18" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S18" s="24">
         <v>0</v>
@@ -2552,7 +2552,7 @@
         <v>0</v>
       </c>
       <c r="R19" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S19" s="24">
         <v>0</v>
@@ -2634,7 +2634,7 @@
         <v>1</v>
       </c>
       <c r="R20" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S20" s="24">
         <v>0</v>
@@ -2716,7 +2716,7 @@
         <v>0</v>
       </c>
       <c r="R21" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S21" s="24">
         <v>0</v>
@@ -2800,7 +2800,7 @@
         <v>0</v>
       </c>
       <c r="R22" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S22" s="24">
         <v>0</v>
@@ -2884,7 +2884,7 @@
         <v>0</v>
       </c>
       <c r="R23" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S23" s="24">
         <v>0</v>
@@ -2968,7 +2968,7 @@
         <v>0</v>
       </c>
       <c r="R24" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S24" s="24">
         <v>0</v>
@@ -3050,7 +3050,7 @@
         <v>0</v>
       </c>
       <c r="R25" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S25" s="24">
         <v>0</v>
@@ -3132,7 +3132,7 @@
         <v>1</v>
       </c>
       <c r="R26" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S26" s="24">
         <v>0</v>
@@ -3214,7 +3214,7 @@
         <v>0</v>
       </c>
       <c r="R27" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S27" s="24">
         <v>0</v>
@@ -3298,7 +3298,7 @@
         <v>0</v>
       </c>
       <c r="R28" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S28" s="24">
         <v>0</v>
@@ -3382,7 +3382,7 @@
         <v>0</v>
       </c>
       <c r="R29" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S29" s="24">
         <v>0</v>
@@ -3464,7 +3464,7 @@
         <v>0</v>
       </c>
       <c r="R30" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S30" s="24">
         <v>0</v>
@@ -3546,7 +3546,7 @@
         <v>0</v>
       </c>
       <c r="R31" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S31" s="24">
         <v>0</v>
@@ -3628,7 +3628,7 @@
         <v>0</v>
       </c>
       <c r="R32" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S32" s="24">
         <v>0</v>
@@ -3712,7 +3712,7 @@
         <v>0</v>
       </c>
       <c r="R33" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S33" s="24">
         <v>0</v>
@@ -3796,7 +3796,7 @@
         <v>0</v>
       </c>
       <c r="R34" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S34" s="24">
         <v>0</v>
@@ -3878,7 +3878,7 @@
         <v>0</v>
       </c>
       <c r="R35" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S35" s="24">
         <v>0</v>
@@ -3960,7 +3960,7 @@
         <v>0</v>
       </c>
       <c r="R36" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S36" s="24">
         <v>0</v>
@@ -4042,7 +4042,7 @@
         <v>0</v>
       </c>
       <c r="R37" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S37" s="24">
         <v>0</v>
@@ -4124,7 +4124,7 @@
         <v>0</v>
       </c>
       <c r="R38" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S38" s="24">
         <v>0</v>
@@ -4208,7 +4208,7 @@
         <v>0</v>
       </c>
       <c r="R39" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S39" s="24">
         <v>0</v>
@@ -4290,7 +4290,7 @@
         <v>0</v>
       </c>
       <c r="R40" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S40" s="24">
         <v>0</v>
@@ -4374,7 +4374,7 @@
         <v>0</v>
       </c>
       <c r="R41" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S41" s="24">
         <v>0</v>
@@ -4458,7 +4458,7 @@
         <v>0</v>
       </c>
       <c r="R42" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S42" s="24">
         <v>0</v>
@@ -4542,7 +4542,7 @@
         <v>0</v>
       </c>
       <c r="R43" s="22">
-        <v>2.3328773748481666E-5</v>
+        <v>4.6657547496963339E-4</v>
       </c>
       <c r="S43" s="24">
         <v>0</v>

</xml_diff>

<commit_message>
Adjust Hydro Asset file, Remove Energy2Power Ratio
Adjust MaxProd, Trubine factor, Storage capacity, Replace Energy2Power Ratio with Storage Capacity
</commit_message>
<xml_diff>
--- a/data/hydroExample/Power_HydroAssets.xlsx
+++ b/data/hydroExample/Power_HydroAssets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth\Git\LEGO-Pyomo\data\hydroExample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9749FC6-1F5D-4DBB-B7E0-B6D1C872347C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2FA42C0-992F-4D05-B7CB-0F86947FC28B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -556,11 +556,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -686,7 +685,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -734,12 +733,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1526,7 +1519,7 @@
       <c r="K7" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="L7" s="23" t="s">
+      <c r="L7" s="21" t="s">
         <v>90</v>
       </c>
       <c r="M7" s="9" t="s">
@@ -1602,8 +1595,8 @@
       <c r="F8" s="12">
         <v>1</v>
       </c>
-      <c r="G8" s="22">
-        <v>18795.432911392403</v>
+      <c r="G8" s="20">
+        <v>54909.846575342461</v>
       </c>
       <c r="H8" s="13">
         <v>0</v>
@@ -1611,14 +1604,14 @@
       <c r="I8" s="13">
         <v>0</v>
       </c>
-      <c r="J8" s="22">
-        <v>1.3833147724009441E-3</v>
+      <c r="J8" s="20">
+        <v>4.7350341735748772E-4</v>
       </c>
       <c r="K8" s="14">
         <v>0</v>
       </c>
       <c r="L8" s="14">
-        <v>225545.19493670884</v>
+        <v>658918.1589041095</v>
       </c>
       <c r="M8" s="13"/>
       <c r="N8" s="13"/>
@@ -1631,10 +1624,10 @@
       <c r="Q8" s="12">
         <v>0</v>
       </c>
-      <c r="R8" s="22">
+      <c r="R8" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S8" s="24">
+      <c r="S8" s="22">
         <v>0</v>
       </c>
       <c r="T8" s="12">
@@ -1686,8 +1679,8 @@
       <c r="F9" s="12">
         <v>1</v>
       </c>
-      <c r="G9" s="22">
-        <v>76314.213344048214</v>
+      <c r="G9" s="20">
+        <v>26170.257945205503</v>
       </c>
       <c r="H9" s="13">
         <v>0</v>
@@ -1695,14 +1688,14 @@
       <c r="I9" s="13">
         <v>0</v>
       </c>
-      <c r="J9" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J9" s="20">
+        <v>1.2609734328600966E-3</v>
       </c>
       <c r="K9" s="14">
         <v>0</v>
       </c>
       <c r="L9" s="14">
-        <v>915770.56012857857</v>
+        <v>314043.09534246603</v>
       </c>
       <c r="M9" s="13"/>
       <c r="N9" s="13"/>
@@ -1715,10 +1708,10 @@
       <c r="Q9" s="12">
         <v>0</v>
       </c>
-      <c r="R9" s="22">
+      <c r="R9" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S9" s="24">
+      <c r="S9" s="22">
         <v>0</v>
       </c>
       <c r="T9" s="12">
@@ -1768,23 +1761,23 @@
       <c r="F10" s="12">
         <v>1</v>
       </c>
-      <c r="G10" s="22">
-        <v>197455.68000000002</v>
+      <c r="G10" s="20">
+        <v>90723.6</v>
       </c>
       <c r="H10" s="13">
         <v>0</v>
       </c>
-      <c r="I10" s="21">
-        <v>123.1396524</v>
-      </c>
-      <c r="J10" s="22">
-        <v>1.7219053916301622E-4</v>
+      <c r="I10" s="20">
+        <v>11095.429726027354</v>
+      </c>
+      <c r="J10" s="20">
+        <v>3.7476466983232587E-4</v>
       </c>
       <c r="K10" s="20">
-        <v>1.6999999999999999E-3</v>
+        <v>3.7476466983232587E-4</v>
       </c>
       <c r="L10" s="14">
-        <v>2369468.16</v>
+        <v>1088683.2000000002</v>
       </c>
       <c r="M10" s="13"/>
       <c r="N10" s="13"/>
@@ -1797,10 +1790,10 @@
       <c r="Q10" s="12">
         <v>0</v>
       </c>
-      <c r="R10" s="22">
+      <c r="R10" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S10" s="22">
+      <c r="S10" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
       <c r="T10" s="12">
@@ -1817,7 +1810,7 @@
       </c>
       <c r="X10" s="13">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>12.000000000000002</v>
       </c>
       <c r="Y10" s="15"/>
       <c r="Z10" s="12">
@@ -1852,8 +1845,8 @@
       <c r="F11" s="12">
         <v>1</v>
       </c>
-      <c r="G11" s="22">
-        <v>117304.04284051221</v>
+      <c r="G11" s="20">
+        <v>303080.53109589039</v>
       </c>
       <c r="H11" s="13">
         <v>0</v>
@@ -1861,14 +1854,14 @@
       <c r="I11" s="13">
         <v>0</v>
       </c>
-      <c r="J11" s="22">
-        <v>1.3639768598388177E-4</v>
+      <c r="J11" s="20">
+        <v>5.2791249712235146E-5</v>
       </c>
       <c r="K11" s="14">
         <v>0</v>
       </c>
       <c r="L11" s="14">
-        <v>1407648.5140861464</v>
+        <v>3636966.3731506849</v>
       </c>
       <c r="M11" s="13"/>
       <c r="N11" s="13"/>
@@ -1881,10 +1874,10 @@
       <c r="Q11" s="12">
         <v>0</v>
       </c>
-      <c r="R11" s="22">
+      <c r="R11" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S11" s="24">
+      <c r="S11" s="22">
         <v>0</v>
       </c>
       <c r="T11" s="12">
@@ -1901,7 +1894,7 @@
       </c>
       <c r="X11" s="13">
         <f t="shared" si="0"/>
-        <v>11.999999999999998</v>
+        <v>12</v>
       </c>
       <c r="Y11" s="15"/>
       <c r="Z11" s="12">
@@ -1936,8 +1929,8 @@
       <c r="F12" s="12">
         <v>1</v>
       </c>
-      <c r="G12" s="22">
-        <v>50876.142229365476</v>
+      <c r="G12" s="20">
+        <v>38620.287567119769</v>
       </c>
       <c r="H12" s="13">
         <v>0</v>
@@ -1945,14 +1938,14 @@
       <c r="I12" s="13">
         <v>0</v>
       </c>
-      <c r="J12" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J12" s="20">
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K12" s="14">
         <v>0</v>
       </c>
       <c r="L12" s="14">
-        <v>610513.70675238571</v>
+        <v>463443.45080543723</v>
       </c>
       <c r="M12" s="13"/>
       <c r="N12" s="13"/>
@@ -1965,10 +1958,10 @@
       <c r="Q12" s="12">
         <v>0</v>
       </c>
-      <c r="R12" s="22">
+      <c r="R12" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S12" s="24">
+      <c r="S12" s="22">
         <v>0</v>
       </c>
       <c r="T12" s="12">
@@ -2020,8 +2013,8 @@
       <c r="F13" s="12">
         <v>1</v>
       </c>
-      <c r="G13" s="22">
-        <v>128145.67200000001</v>
+      <c r="G13" s="20">
+        <v>308190.13232876715</v>
       </c>
       <c r="H13" s="13">
         <v>0</v>
@@ -2029,14 +2022,14 @@
       <c r="I13" s="13">
         <v>0</v>
       </c>
-      <c r="J13" s="22">
-        <v>9.3643427926305622E-5</v>
+      <c r="J13" s="20">
+        <v>3.8937002652631305E-5</v>
       </c>
       <c r="K13" s="14">
         <v>0</v>
       </c>
       <c r="L13" s="14">
-        <v>1537748.064</v>
+        <v>3698281.5879452061</v>
       </c>
       <c r="M13" s="13"/>
       <c r="N13" s="13"/>
@@ -2049,10 +2042,10 @@
       <c r="Q13" s="12">
         <v>0</v>
       </c>
-      <c r="R13" s="22">
+      <c r="R13" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S13" s="24">
+      <c r="S13" s="22">
         <v>0</v>
       </c>
       <c r="T13" s="12">
@@ -2104,8 +2097,8 @@
       <c r="F14" s="12">
         <v>1</v>
       </c>
-      <c r="G14" s="22">
-        <v>192549.84</v>
+      <c r="G14" s="20">
+        <v>467759.68356164393</v>
       </c>
       <c r="H14" s="13">
         <v>0</v>
@@ -2113,14 +2106,14 @@
       <c r="I14" s="13">
         <v>0</v>
       </c>
-      <c r="J14" s="22">
-        <v>7.2708447849138697E-5</v>
+      <c r="J14" s="20">
+        <v>2.9929898817701346E-5</v>
       </c>
       <c r="K14" s="14">
         <v>0</v>
       </c>
       <c r="L14" s="14">
-        <v>2310598.08</v>
+        <v>5613116.2027397268</v>
       </c>
       <c r="M14" s="13"/>
       <c r="N14" s="13"/>
@@ -2133,10 +2126,10 @@
       <c r="Q14" s="12">
         <v>0</v>
       </c>
-      <c r="R14" s="22">
+      <c r="R14" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S14" s="24">
+      <c r="S14" s="22">
         <v>0</v>
       </c>
       <c r="T14" s="12">
@@ -2153,7 +2146,7 @@
       </c>
       <c r="X14" s="13">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>11.999999999999998</v>
       </c>
       <c r="Y14" s="15"/>
       <c r="Z14" s="12">
@@ -2188,8 +2181,8 @@
       <c r="F15" s="12">
         <v>1</v>
       </c>
-      <c r="G15" s="22">
-        <v>168293.23855530474</v>
+      <c r="G15" s="20">
+        <v>729653.91196388274</v>
       </c>
       <c r="H15" s="13">
         <v>0</v>
@@ -2197,14 +2190,14 @@
       <c r="I15" s="13">
         <v>0</v>
       </c>
-      <c r="J15" s="22">
-        <v>1.12898177984472E-4</v>
+      <c r="J15" s="20">
+        <v>2.6039742525139078E-5</v>
       </c>
       <c r="K15" s="14">
         <v>0</v>
       </c>
       <c r="L15" s="14">
-        <v>2019518.8626636569</v>
+        <v>8755846.9435665924</v>
       </c>
       <c r="M15" s="13"/>
       <c r="N15" s="13"/>
@@ -2217,10 +2210,10 @@
       <c r="Q15" s="12">
         <v>0</v>
       </c>
-      <c r="R15" s="22">
+      <c r="R15" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S15" s="24">
+      <c r="S15" s="22">
         <v>0</v>
       </c>
       <c r="T15" s="12">
@@ -2272,8 +2265,8 @@
       <c r="F16" s="12">
         <v>1</v>
       </c>
-      <c r="G16" s="22">
-        <v>735583.65842696629</v>
+      <c r="G16" s="20">
+        <v>467759.68356164393</v>
       </c>
       <c r="H16" s="13">
         <v>0</v>
@@ -2281,14 +2274,14 @@
       <c r="I16" s="13">
         <v>0</v>
       </c>
-      <c r="J16" s="22">
-        <v>1.9032505466392189E-5</v>
+      <c r="J16" s="20">
+        <v>2.9929898817701346E-5</v>
       </c>
       <c r="K16" s="14">
         <v>0</v>
       </c>
       <c r="L16" s="14">
-        <v>8827003.9011235945</v>
+        <v>5613116.2027397268</v>
       </c>
       <c r="M16" s="13"/>
       <c r="N16" s="13"/>
@@ -2301,10 +2294,10 @@
       <c r="Q16" s="12">
         <v>0</v>
       </c>
-      <c r="R16" s="22">
+      <c r="R16" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S16" s="24">
+      <c r="S16" s="22">
         <v>0</v>
       </c>
       <c r="T16" s="12">
@@ -2356,8 +2349,8 @@
       <c r="F17" s="12">
         <v>1</v>
       </c>
-      <c r="G17" s="22">
-        <v>184888.02933333334</v>
+      <c r="G17" s="20">
+        <v>413303.9589041096</v>
       </c>
       <c r="H17" s="13">
         <v>0</v>
@@ -2365,14 +2358,14 @@
       <c r="I17" s="13">
         <v>0</v>
       </c>
-      <c r="J17" s="22">
-        <v>5.9495468904415532E-5</v>
+      <c r="J17" s="20">
+        <v>2.6614794663876189E-5</v>
       </c>
       <c r="K17" s="14">
         <v>0</v>
       </c>
       <c r="L17" s="14">
-        <v>2218656.352</v>
+        <v>4959647.506849315</v>
       </c>
       <c r="M17" s="13"/>
       <c r="N17" s="13"/>
@@ -2385,10 +2378,10 @@
       <c r="Q17" s="12">
         <v>0</v>
       </c>
-      <c r="R17" s="22">
+      <c r="R17" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S17" s="24">
+      <c r="S17" s="22">
         <v>0</v>
       </c>
       <c r="T17" s="12">
@@ -2440,8 +2433,8 @@
       <c r="F18" s="12">
         <v>1</v>
       </c>
-      <c r="G18" s="22">
-        <v>169397.1903512195</v>
+      <c r="G18" s="20">
+        <v>388412.26027397258</v>
       </c>
       <c r="H18" s="13">
         <v>0</v>
@@ -2449,14 +2442,14 @@
       <c r="I18" s="13">
         <v>0</v>
       </c>
-      <c r="J18" s="22">
-        <v>1.0448815569668966E-4</v>
+      <c r="J18" s="20">
+        <v>4.5570137223565063E-5</v>
       </c>
       <c r="K18" s="14">
         <v>0</v>
       </c>
       <c r="L18" s="14">
-        <v>2032766.284214634</v>
+        <v>4660947.1232876712</v>
       </c>
       <c r="M18" s="13"/>
       <c r="N18" s="13"/>
@@ -2469,10 +2462,10 @@
       <c r="Q18" s="12">
         <v>0</v>
       </c>
-      <c r="R18" s="22">
+      <c r="R18" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S18" s="24">
+      <c r="S18" s="22">
         <v>0</v>
       </c>
       <c r="T18" s="12">
@@ -2522,8 +2515,8 @@
       <c r="F19" s="12">
         <v>1</v>
       </c>
-      <c r="G19" s="22">
-        <v>13875.311517099675</v>
+      <c r="G19" s="20">
+        <v>26170.2579452055</v>
       </c>
       <c r="H19" s="13">
         <v>0</v>
@@ -2531,14 +2524,14 @@
       <c r="I19" s="13">
         <v>0</v>
       </c>
-      <c r="J19" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J19" s="20">
+        <v>2.2926789688365392E-4</v>
       </c>
       <c r="K19" s="14">
         <v>0</v>
       </c>
       <c r="L19" s="14">
-        <v>166503.7382051961</v>
+        <v>314043.09534246603</v>
       </c>
       <c r="M19" s="13"/>
       <c r="N19" s="13"/>
@@ -2551,10 +2544,10 @@
       <c r="Q19" s="12">
         <v>0</v>
       </c>
-      <c r="R19" s="22">
+      <c r="R19" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S19" s="24">
+      <c r="S19" s="22">
         <v>0</v>
       </c>
       <c r="T19" s="12">
@@ -2571,7 +2564,7 @@
       </c>
       <c r="X19" s="13">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>12.000000000000002</v>
       </c>
       <c r="Y19" s="15"/>
       <c r="Z19" s="12"/>
@@ -2604,8 +2597,8 @@
       <c r="F20" s="12">
         <v>1</v>
       </c>
-      <c r="G20" s="22">
-        <v>21107.257600000001</v>
+      <c r="G20" s="20">
+        <v>11095.429726027354</v>
       </c>
       <c r="H20" s="13">
         <v>0</v>
@@ -2613,8 +2606,8 @@
       <c r="I20" s="13">
         <v>0</v>
       </c>
-      <c r="J20" s="22">
-        <v>4.9272151773994549E-3</v>
+      <c r="J20" s="20">
+        <v>9.3732286687409367E-3</v>
       </c>
       <c r="K20" s="14">
         <v>0</v>
@@ -2633,10 +2626,10 @@
       <c r="Q20" s="12">
         <v>1</v>
       </c>
-      <c r="R20" s="22">
+      <c r="R20" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S20" s="24">
+      <c r="S20" s="22">
         <v>0</v>
       </c>
       <c r="T20" s="12">
@@ -2653,7 +2646,7 @@
       </c>
       <c r="X20" s="13">
         <f t="shared" si="0"/>
-        <v>710.65603520184447</v>
+        <v>1351.9079810684045</v>
       </c>
       <c r="Y20" s="15"/>
       <c r="Z20" s="12"/>
@@ -2686,8 +2679,8 @@
       <c r="F21" s="12">
         <v>1</v>
       </c>
-      <c r="G21" s="22">
-        <v>183607.69530845954</v>
+      <c r="G21" s="20">
+        <v>388412.26027397258</v>
       </c>
       <c r="H21" s="13">
         <v>0</v>
@@ -2695,14 +2688,14 @@
       <c r="I21" s="13">
         <v>0</v>
       </c>
-      <c r="J21" s="22">
-        <v>1.0348150151375814E-4</v>
+      <c r="J21" s="20">
+        <v>4.8917096454674359E-5</v>
       </c>
       <c r="K21" s="14">
         <v>0</v>
       </c>
       <c r="L21" s="14">
-        <v>2203292.3437015144</v>
+        <v>4660947.1232876712</v>
       </c>
       <c r="M21" s="13"/>
       <c r="N21" s="13"/>
@@ -2715,10 +2708,10 @@
       <c r="Q21" s="12">
         <v>0</v>
       </c>
-      <c r="R21" s="22">
+      <c r="R21" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S21" s="24">
+      <c r="S21" s="22">
         <v>0</v>
       </c>
       <c r="T21" s="12">
@@ -2770,8 +2763,8 @@
       <c r="F22" s="12">
         <v>1</v>
       </c>
-      <c r="G22" s="22">
-        <v>122730.03966942149</v>
+      <c r="G22" s="20">
+        <v>391003.39726027398</v>
       </c>
       <c r="H22" s="13">
         <v>0</v>
@@ -2779,14 +2772,14 @@
       <c r="I22" s="13">
         <v>0</v>
       </c>
-      <c r="J22" s="22">
-        <v>1.4666336007454863E-4</v>
+      <c r="J22" s="20">
+        <v>4.6035405641292117E-5</v>
       </c>
       <c r="K22" s="14">
         <v>0</v>
       </c>
       <c r="L22" s="14">
-        <v>1472760.4760330578</v>
+        <v>4692040.7671232875</v>
       </c>
       <c r="M22" s="13"/>
       <c r="N22" s="13"/>
@@ -2799,10 +2792,10 @@
       <c r="Q22" s="12">
         <v>0</v>
       </c>
-      <c r="R22" s="22">
+      <c r="R22" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S22" s="24">
+      <c r="S22" s="22">
         <v>0</v>
       </c>
       <c r="T22" s="12">
@@ -2854,8 +2847,8 @@
       <c r="F23" s="12">
         <v>1</v>
       </c>
-      <c r="G23" s="22">
-        <v>111471.04648390942</v>
+      <c r="G23" s="20">
+        <v>467759.68356164382</v>
       </c>
       <c r="H23" s="13">
         <v>0</v>
@@ -2863,14 +2856,14 @@
       <c r="I23" s="13">
         <v>0</v>
       </c>
-      <c r="J23" s="22">
-        <v>8.9709393743275537E-5</v>
+      <c r="J23" s="20">
+        <v>2.1378499155500961E-5</v>
       </c>
       <c r="K23" s="14">
         <v>0</v>
       </c>
       <c r="L23" s="14">
-        <v>1337652.557806913</v>
+        <v>5613116.2027397258</v>
       </c>
       <c r="M23" s="13"/>
       <c r="N23" s="13"/>
@@ -2883,10 +2876,10 @@
       <c r="Q23" s="12">
         <v>0</v>
       </c>
-      <c r="R23" s="22">
+      <c r="R23" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S23" s="24">
+      <c r="S23" s="22">
         <v>0</v>
       </c>
       <c r="T23" s="12">
@@ -2938,8 +2931,8 @@
       <c r="F24" s="12">
         <v>1</v>
       </c>
-      <c r="G24" s="22">
-        <v>146262.2694969576</v>
+      <c r="G24" s="20">
+        <v>303080.53109589039</v>
       </c>
       <c r="H24" s="13">
         <v>0</v>
@@ -2947,14 +2940,14 @@
       <c r="I24" s="13">
         <v>0</v>
       </c>
-      <c r="J24" s="22">
-        <v>6.8370332515645875E-5</v>
+      <c r="J24" s="20">
+        <v>3.2994531070146968E-5</v>
       </c>
       <c r="K24" s="14">
         <v>0</v>
       </c>
       <c r="L24" s="14">
-        <v>1755147.2339634912</v>
+        <v>3636966.3731506849</v>
       </c>
       <c r="M24" s="13"/>
       <c r="N24" s="13"/>
@@ -2967,10 +2960,10 @@
       <c r="Q24" s="12">
         <v>0</v>
       </c>
-      <c r="R24" s="22">
+      <c r="R24" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S24" s="24">
+      <c r="S24" s="22">
         <v>0</v>
       </c>
       <c r="T24" s="12">
@@ -3020,8 +3013,8 @@
       <c r="F25" s="12">
         <v>1</v>
       </c>
-      <c r="G25" s="22">
-        <v>30063.174953715963</v>
+      <c r="G25" s="20">
+        <v>467759.68356164382</v>
       </c>
       <c r="H25" s="13">
         <v>0</v>
@@ -3029,14 +3022,14 @@
       <c r="I25" s="13">
         <v>0</v>
       </c>
-      <c r="J25" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J25" s="20">
+        <v>2.779204890215125E-5</v>
       </c>
       <c r="K25" s="14">
         <v>0</v>
       </c>
       <c r="L25" s="14">
-        <v>360758.09944459156</v>
+        <v>5613116.2027397258</v>
       </c>
       <c r="M25" s="13"/>
       <c r="N25" s="13"/>
@@ -3049,10 +3042,10 @@
       <c r="Q25" s="12">
         <v>0</v>
       </c>
-      <c r="R25" s="22">
+      <c r="R25" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S25" s="24">
+      <c r="S25" s="22">
         <v>0</v>
       </c>
       <c r="T25" s="12">
@@ -3102,8 +3095,8 @@
       <c r="F26" s="12">
         <v>1</v>
       </c>
-      <c r="G26" s="22">
-        <v>34688.278792749188</v>
+      <c r="G26" s="20">
+        <v>26170.2579452055</v>
       </c>
       <c r="H26" s="13">
         <v>0</v>
@@ -3111,14 +3104,14 @@
       <c r="I26" s="13">
         <v>0</v>
       </c>
-      <c r="J26" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J26" s="20">
+        <v>5.7316974220913486E-4</v>
       </c>
       <c r="K26" s="14">
         <v>0</v>
       </c>
       <c r="L26" s="14">
-        <v>416259.34551299026</v>
+        <v>314043.09534246603</v>
       </c>
       <c r="M26" s="13"/>
       <c r="N26" s="13"/>
@@ -3131,10 +3124,10 @@
       <c r="Q26" s="12">
         <v>1</v>
       </c>
-      <c r="R26" s="22">
+      <c r="R26" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S26" s="24">
+      <c r="S26" s="22">
         <v>0</v>
       </c>
       <c r="T26" s="12">
@@ -3151,7 +3144,7 @@
       </c>
       <c r="X26" s="13">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>12.000000000000002</v>
       </c>
       <c r="Y26" s="15"/>
       <c r="Z26" s="12"/>
@@ -3184,8 +3177,8 @@
       <c r="F27" s="12">
         <v>1</v>
       </c>
-      <c r="G27" s="22">
-        <v>131944.51443052923</v>
+      <c r="G27" s="20">
+        <v>391003.39726027398</v>
       </c>
       <c r="H27" s="13">
         <v>0</v>
@@ -3193,14 +3186,14 @@
       <c r="I27" s="13">
         <v>0</v>
       </c>
-      <c r="J27" s="22">
-        <v>9.8526263529088916E-5</v>
+      <c r="J27" s="20">
+        <v>3.324779296315542E-5</v>
       </c>
       <c r="K27" s="14">
         <v>0</v>
       </c>
       <c r="L27" s="14">
-        <v>1583334.1731663509</v>
+        <v>4692040.7671232875</v>
       </c>
       <c r="M27" s="13"/>
       <c r="N27" s="13"/>
@@ -3213,10 +3206,10 @@
       <c r="Q27" s="12">
         <v>0</v>
       </c>
-      <c r="R27" s="22">
+      <c r="R27" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S27" s="24">
+      <c r="S27" s="22">
         <v>0</v>
       </c>
       <c r="T27" s="12">
@@ -3268,8 +3261,8 @@
       <c r="F28" s="12">
         <v>1</v>
       </c>
-      <c r="G28" s="22">
-        <v>60126.349907431926</v>
+      <c r="G28" s="20">
+        <v>45642.158033868822</v>
       </c>
       <c r="H28" s="13">
         <v>0</v>
@@ -3277,14 +3270,14 @@
       <c r="I28" s="13">
         <v>0</v>
       </c>
-      <c r="J28" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J28" s="20">
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K28" s="14">
         <v>0</v>
       </c>
       <c r="L28" s="14">
-        <v>721516.19888918311</v>
+        <v>547705.89640642586</v>
       </c>
       <c r="M28" s="13"/>
       <c r="N28" s="13"/>
@@ -3297,10 +3290,10 @@
       <c r="Q28" s="12">
         <v>0</v>
       </c>
-      <c r="R28" s="22">
+      <c r="R28" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S28" s="24">
+      <c r="S28" s="22">
         <v>0</v>
       </c>
       <c r="T28" s="12">
@@ -3352,8 +3345,8 @@
       <c r="F29" s="12">
         <v>1</v>
       </c>
-      <c r="G29" s="22">
-        <v>4625.1038390332251</v>
+      <c r="G29" s="20">
+        <v>3510.9352333745246</v>
       </c>
       <c r="H29" s="13">
         <v>0</v>
@@ -3361,14 +3354,14 @@
       <c r="I29" s="13">
         <v>0</v>
       </c>
-      <c r="J29" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J29" s="20">
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K29" s="14">
         <v>0</v>
       </c>
       <c r="L29" s="14">
-        <v>55501.246068398701</v>
+        <v>42131.222800494295</v>
       </c>
       <c r="M29" s="13"/>
       <c r="N29" s="13"/>
@@ -3381,10 +3374,10 @@
       <c r="Q29" s="12">
         <v>0</v>
       </c>
-      <c r="R29" s="22">
+      <c r="R29" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S29" s="24">
+      <c r="S29" s="22">
         <v>0</v>
       </c>
       <c r="T29" s="12">
@@ -3434,8 +3427,8 @@
       <c r="F30" s="12">
         <v>1</v>
       </c>
-      <c r="G30" s="22">
-        <v>179073.80465116279</v>
+      <c r="G30" s="20">
+        <v>391003.39726027398</v>
       </c>
       <c r="H30" s="13">
         <v>0</v>
@@ -3443,14 +3436,14 @@
       <c r="I30" s="13">
         <v>0</v>
       </c>
-      <c r="J30" s="22">
-        <v>7.8180055576928815E-5</v>
+      <c r="J30" s="20">
+        <v>3.5805315498782759E-5</v>
       </c>
       <c r="K30" s="14">
         <v>0</v>
       </c>
       <c r="L30" s="14">
-        <v>2148885.6558139534</v>
+        <v>4692040.7671232875</v>
       </c>
       <c r="M30" s="13"/>
       <c r="N30" s="13"/>
@@ -3463,10 +3456,10 @@
       <c r="Q30" s="12">
         <v>0</v>
       </c>
-      <c r="R30" s="22">
+      <c r="R30" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S30" s="24">
+      <c r="S30" s="22">
         <v>0</v>
       </c>
       <c r="T30" s="12">
@@ -3516,8 +3509,8 @@
       <c r="F31" s="12">
         <v>1</v>
       </c>
-      <c r="G31" s="22">
-        <v>2312.5519195166125</v>
+      <c r="G31" s="20">
+        <v>1755.4676166872623</v>
       </c>
       <c r="H31" s="13">
         <v>0</v>
@@ -3525,14 +3518,14 @@
       <c r="I31" s="13">
         <v>0</v>
       </c>
-      <c r="J31" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J31" s="20">
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K31" s="14">
         <v>0</v>
       </c>
       <c r="L31" s="14">
-        <v>27750.623034199351</v>
+        <v>21065.611400247148</v>
       </c>
       <c r="M31" s="13"/>
       <c r="N31" s="13"/>
@@ -3545,10 +3538,10 @@
       <c r="Q31" s="12">
         <v>0</v>
       </c>
-      <c r="R31" s="22">
+      <c r="R31" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S31" s="24">
+      <c r="S31" s="22">
         <v>0</v>
       </c>
       <c r="T31" s="12">
@@ -3598,8 +3591,8 @@
       <c r="F32" s="12">
         <v>1</v>
       </c>
-      <c r="G32" s="22">
-        <v>204734.74925373134</v>
+      <c r="G32" s="20">
+        <v>558256.28219178075</v>
       </c>
       <c r="H32" s="13">
         <v>0</v>
@@ -3607,14 +3600,14 @@
       <c r="I32" s="13">
         <v>0</v>
       </c>
-      <c r="J32" s="22">
-        <v>6.3496793032866511E-5</v>
+      <c r="J32" s="20">
+        <v>2.3286795714972428E-5</v>
       </c>
       <c r="K32" s="14">
         <v>0</v>
       </c>
       <c r="L32" s="14">
-        <v>2456816.991044776</v>
+        <v>6699075.3863013685</v>
       </c>
       <c r="M32" s="13"/>
       <c r="N32" s="13"/>
@@ -3627,10 +3620,10 @@
       <c r="Q32" s="12">
         <v>0</v>
       </c>
-      <c r="R32" s="22">
+      <c r="R32" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S32" s="24">
+      <c r="S32" s="22">
         <v>0</v>
       </c>
       <c r="T32" s="12">
@@ -3682,8 +3675,8 @@
       <c r="F33" s="12">
         <v>1</v>
       </c>
-      <c r="G33" s="22">
-        <v>37022.94</v>
+      <c r="G33" s="20">
+        <v>90723.599999999991</v>
       </c>
       <c r="H33" s="13">
         <v>0</v>
@@ -3691,14 +3684,14 @@
       <c r="I33" s="13">
         <v>0</v>
       </c>
-      <c r="J33" s="22">
-        <v>1.6206168391813292E-4</v>
+      <c r="J33" s="20">
+        <v>6.6134941735116335E-5</v>
       </c>
       <c r="K33" s="14">
         <v>0</v>
       </c>
       <c r="L33" s="14">
-        <v>444275.28</v>
+        <v>1088683.2</v>
       </c>
       <c r="M33" s="13"/>
       <c r="N33" s="13"/>
@@ -3711,10 +3704,10 @@
       <c r="Q33" s="12">
         <v>0</v>
       </c>
-      <c r="R33" s="22">
+      <c r="R33" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S33" s="24">
+      <c r="S33" s="22">
         <v>0</v>
       </c>
       <c r="T33" s="12">
@@ -3766,8 +3759,8 @@
       <c r="F34" s="12">
         <v>1</v>
       </c>
-      <c r="G34" s="22">
-        <v>37000.830712265801</v>
+      <c r="G34" s="20">
+        <v>26170.257945205503</v>
       </c>
       <c r="H34" s="13">
         <v>0</v>
@@ -3775,14 +3768,14 @@
       <c r="I34" s="13">
         <v>0</v>
       </c>
-      <c r="J34" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J34" s="20">
+        <v>6.1138105835641045E-4</v>
       </c>
       <c r="K34" s="14">
         <v>0</v>
       </c>
       <c r="L34" s="14">
-        <v>444009.96854718961</v>
+        <v>314043.09534246603</v>
       </c>
       <c r="M34" s="13"/>
       <c r="N34" s="13"/>
@@ -3795,10 +3788,10 @@
       <c r="Q34" s="12">
         <v>0</v>
       </c>
-      <c r="R34" s="22">
+      <c r="R34" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S34" s="24">
+      <c r="S34" s="22">
         <v>0</v>
       </c>
       <c r="T34" s="12">
@@ -3848,8 +3841,8 @@
       <c r="F35" s="12">
         <v>1</v>
       </c>
-      <c r="G35" s="22">
-        <v>27750.623034199351</v>
+      <c r="G35" s="20">
+        <v>21065.611400247148</v>
       </c>
       <c r="H35" s="13">
         <v>0</v>
@@ -3857,14 +3850,14 @@
       <c r="I35" s="13">
         <v>0</v>
       </c>
-      <c r="J35" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J35" s="20">
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K35" s="14">
         <v>0</v>
       </c>
       <c r="L35" s="14">
-        <v>333007.47641039221</v>
+        <v>252787.33680296579</v>
       </c>
       <c r="M35" s="13"/>
       <c r="N35" s="13"/>
@@ -3877,10 +3870,10 @@
       <c r="Q35" s="12">
         <v>0</v>
       </c>
-      <c r="R35" s="22">
+      <c r="R35" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S35" s="24">
+      <c r="S35" s="22">
         <v>0</v>
       </c>
       <c r="T35" s="12">
@@ -3930,8 +3923,8 @@
       <c r="F36" s="12">
         <v>1</v>
       </c>
-      <c r="G36" s="22">
-        <v>2312.5519195166125</v>
+      <c r="G36" s="20">
+        <v>26170.257945205503</v>
       </c>
       <c r="H36" s="13">
         <v>0</v>
@@ -3939,14 +3932,14 @@
       <c r="I36" s="13">
         <v>0</v>
       </c>
-      <c r="J36" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J36" s="20">
+        <v>3.8211316147275653E-5</v>
       </c>
       <c r="K36" s="14">
         <v>0</v>
       </c>
       <c r="L36" s="14">
-        <v>27750.623034199351</v>
+        <v>314043.09534246603</v>
       </c>
       <c r="M36" s="13"/>
       <c r="N36" s="13"/>
@@ -3959,10 +3952,10 @@
       <c r="Q36" s="12">
         <v>0</v>
       </c>
-      <c r="R36" s="22">
+      <c r="R36" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S36" s="24">
+      <c r="S36" s="22">
         <v>0</v>
       </c>
       <c r="T36" s="12">
@@ -4012,8 +4005,8 @@
       <c r="F37" s="12">
         <v>1</v>
       </c>
-      <c r="G37" s="22">
-        <v>2312.5519195166125</v>
+      <c r="G37" s="20">
+        <v>1755.4676166872623</v>
       </c>
       <c r="H37" s="13">
         <v>0</v>
@@ -4021,14 +4014,14 @@
       <c r="I37" s="13">
         <v>0</v>
       </c>
-      <c r="J37" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J37" s="20">
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K37" s="14">
         <v>0</v>
       </c>
       <c r="L37" s="14">
-        <v>27750.623034199351</v>
+        <v>21065.611400247148</v>
       </c>
       <c r="M37" s="13"/>
       <c r="N37" s="13"/>
@@ -4041,10 +4034,10 @@
       <c r="Q37" s="12">
         <v>0</v>
       </c>
-      <c r="R37" s="22">
+      <c r="R37" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S37" s="24">
+      <c r="S37" s="22">
         <v>0</v>
       </c>
       <c r="T37" s="12">
@@ -4094,8 +4087,8 @@
       <c r="F38" s="12">
         <v>1</v>
       </c>
-      <c r="G38" s="22">
-        <v>39313.382631782413</v>
+      <c r="G38" s="20">
+        <v>29842.94948368346</v>
       </c>
       <c r="H38" s="13">
         <v>0</v>
@@ -4103,14 +4096,14 @@
       <c r="I38" s="13">
         <v>0</v>
       </c>
-      <c r="J38" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J38" s="20">
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K38" s="14">
         <v>0</v>
       </c>
       <c r="L38" s="14">
-        <v>471760.59158138896</v>
+        <v>358115.39380420151</v>
       </c>
       <c r="M38" s="13"/>
       <c r="N38" s="13"/>
@@ -4123,10 +4116,10 @@
       <c r="Q38" s="12">
         <v>0</v>
       </c>
-      <c r="R38" s="22">
+      <c r="R38" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S38" s="24">
+      <c r="S38" s="22">
         <v>0</v>
       </c>
       <c r="T38" s="12">
@@ -4178,8 +4171,8 @@
       <c r="F39" s="12">
         <v>1</v>
       </c>
-      <c r="G39" s="22">
-        <v>2312.5519195166125</v>
+      <c r="G39" s="20">
+        <v>1755.4676166872623</v>
       </c>
       <c r="H39" s="13">
         <v>0</v>
@@ -4187,14 +4180,14 @@
       <c r="I39" s="13">
         <v>0</v>
       </c>
-      <c r="J39" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J39" s="20">
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K39" s="14">
         <v>0</v>
       </c>
       <c r="L39" s="14">
-        <v>27750.623034199351</v>
+        <v>21065.611400247148</v>
       </c>
       <c r="M39" s="13"/>
       <c r="N39" s="13"/>
@@ -4207,10 +4200,10 @@
       <c r="Q39" s="12">
         <v>0</v>
       </c>
-      <c r="R39" s="22">
+      <c r="R39" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S39" s="24">
+      <c r="S39" s="22">
         <v>0</v>
       </c>
       <c r="T39" s="12">
@@ -4260,8 +4253,8 @@
       <c r="F40" s="12">
         <v>1</v>
       </c>
-      <c r="G40" s="22">
-        <v>11331.504405631402</v>
+      <c r="G40" s="20">
+        <v>8601.791321767585</v>
       </c>
       <c r="H40" s="13">
         <v>0</v>
@@ -4269,14 +4262,14 @@
       <c r="I40" s="13">
         <v>0</v>
       </c>
-      <c r="J40" s="22">
-        <v>4.3242272381457611E-4</v>
+      <c r="J40" s="20">
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K40" s="14">
         <v>0</v>
       </c>
       <c r="L40" s="14">
-        <v>135978.05286757683</v>
+        <v>103221.49586121102</v>
       </c>
       <c r="M40" s="13"/>
       <c r="N40" s="13"/>
@@ -4289,10 +4282,10 @@
       <c r="Q40" s="12">
         <v>0</v>
       </c>
-      <c r="R40" s="22">
+      <c r="R40" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S40" s="24">
+      <c r="S40" s="22">
         <v>0</v>
       </c>
       <c r="T40" s="12">
@@ -4344,8 +4337,8 @@
       <c r="F41" s="12">
         <v>1</v>
       </c>
-      <c r="G41" s="22">
-        <v>9898.1018181818181</v>
+      <c r="G41" s="20">
+        <v>14914.142876712329</v>
       </c>
       <c r="H41" s="13">
         <v>0</v>
@@ -4353,14 +4346,14 @@
       <c r="I41" s="13">
         <v>0</v>
       </c>
-      <c r="J41" s="22">
-        <v>1.010294719501774E-3</v>
+      <c r="J41" s="20">
+        <v>6.7050450586835192E-4</v>
       </c>
       <c r="K41" s="14">
         <v>0</v>
       </c>
       <c r="L41" s="14">
-        <v>118777.22181818182</v>
+        <v>178969.71452054795</v>
       </c>
       <c r="M41" s="13"/>
       <c r="N41" s="13"/>
@@ -4373,10 +4366,10 @@
       <c r="Q41" s="12">
         <v>0</v>
       </c>
-      <c r="R41" s="22">
+      <c r="R41" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S41" s="24">
+      <c r="S41" s="22">
         <v>0</v>
       </c>
       <c r="T41" s="12">
@@ -4428,8 +4421,8 @@
       <c r="F42" s="12">
         <v>1</v>
       </c>
-      <c r="G42" s="22">
-        <v>355388.97599999997</v>
+      <c r="G42" s="20">
+        <v>26170.2579452055</v>
       </c>
       <c r="H42" s="13">
         <v>0</v>
@@ -4437,14 +4430,14 @@
       <c r="I42" s="13">
         <v>0</v>
       </c>
-      <c r="J42" s="22">
-        <v>8.4414548638109697E-5</v>
+      <c r="J42" s="20">
+        <v>1.1463394844182697E-3</v>
       </c>
       <c r="K42" s="14">
         <v>0</v>
       </c>
       <c r="L42" s="14">
-        <v>4264667.7119999994</v>
+        <v>314043.09534246603</v>
       </c>
       <c r="M42" s="13"/>
       <c r="N42" s="13"/>
@@ -4457,10 +4450,10 @@
       <c r="Q42" s="12">
         <v>0</v>
       </c>
-      <c r="R42" s="22">
+      <c r="R42" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S42" s="24">
+      <c r="S42" s="22">
         <v>0</v>
       </c>
       <c r="T42" s="12">
@@ -4477,7 +4470,7 @@
       </c>
       <c r="X42" s="13">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>12.000000000000002</v>
       </c>
       <c r="Y42" s="15"/>
       <c r="Z42" s="12">
@@ -4512,8 +4505,8 @@
       <c r="F43" s="12">
         <v>1</v>
       </c>
-      <c r="G43" s="22">
-        <v>180286.82497297297</v>
+      <c r="G43" s="20">
+        <v>388412.26027397264</v>
       </c>
       <c r="H43" s="13">
         <v>0</v>
@@ -4521,14 +4514,14 @@
       <c r="I43" s="13">
         <v>0</v>
       </c>
-      <c r="J43" s="22">
-        <v>9.4294189287256525E-5</v>
+      <c r="J43" s="20">
+        <v>4.37679284068139E-5</v>
       </c>
       <c r="K43" s="14">
         <v>0</v>
       </c>
       <c r="L43" s="14">
-        <v>2163441.8996756757</v>
+        <v>4660947.1232876722</v>
       </c>
       <c r="M43" s="13"/>
       <c r="N43" s="13"/>
@@ -4541,10 +4534,10 @@
       <c r="Q43" s="12">
         <v>0</v>
       </c>
-      <c r="R43" s="22">
+      <c r="R43" s="20">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S43" s="24">
+      <c r="S43" s="22">
         <v>0</v>
       </c>
       <c r="T43" s="12">
@@ -4561,7 +4554,7 @@
       </c>
       <c r="X43" s="13">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>12.000000000000002</v>
       </c>
       <c r="Y43" s="15"/>
       <c r="Z43" s="12">

</xml_diff>

<commit_message>
Fix units in Power_HydroAssets and Power_Inflows_WaterAmount
Fix merge problems for hydro formulation
Switch to newest InOutModule
</commit_message>
<xml_diff>
--- a/data/hydroExample/Power_HydroAssets.xlsx
+++ b/data/hydroExample/Power_HydroAssets.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth\Git\LEGO-Pyomo\data\hydroExample\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\hydroExample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2FA42C0-992F-4D05-B7CB-0F86947FC28B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1938B92-3968-43BD-A84B-1C59D8C104BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34230" yWindow="-21705" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario_2016" sheetId="1" r:id="rId1"/>
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="138">
   <si>
     <t>Format:</t>
   </si>
@@ -183,9 +183,6 @@
     <t>InvestCostPerMWh</t>
   </si>
   <si>
-    <t>Energy to Power Ratio</t>
-  </si>
-  <si>
     <t>FirmCapCoef</t>
   </si>
   <si>
@@ -225,9 +222,6 @@
     <t>IniReserve</t>
   </si>
   <si>
-    <t>Ene2PowRatio</t>
-  </si>
-  <si>
     <t>YearCom</t>
   </si>
   <si>
@@ -300,9 +294,6 @@
     <t>Annualized investment cost per MWh of storage capacity</t>
   </si>
   <si>
-    <t>Energy to power ratio of the storage unit</t>
-  </si>
-  <si>
     <t>Firm capacity coefficient of the unit</t>
   </si>
   <si>
@@ -357,9 +348,6 @@
     <t>[€/MW]</t>
   </si>
   <si>
-    <t>[h]</t>
-  </si>
-  <si>
     <t>[Year]</t>
   </si>
   <si>
@@ -550,16 +538,20 @@
   </si>
   <si>
     <t>How much MWh are stored per m^3 of water?</t>
+  </si>
+  <si>
+    <t>[m^3/h]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -685,7 +677,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -734,6 +726,12 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment indent="1"/>
     </xf>
+    <xf numFmtId="166" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -743,7 +741,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1046,34 +1044,33 @@
   <sheetPr>
     <tabColor rgb="FF008080"/>
   </sheetPr>
-  <dimension ref="A1:AE43"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AD43"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.54296875" customWidth="1"/>
-    <col min="2" max="2" width="19.7265625" customWidth="1"/>
-    <col min="3" max="3" width="29.81640625" customWidth="1"/>
-    <col min="4" max="6" width="15.7265625" customWidth="1"/>
-    <col min="7" max="7" width="17.453125" customWidth="1"/>
-    <col min="8" max="9" width="15.7265625" customWidth="1"/>
-    <col min="10" max="12" width="21.7265625" customWidth="1"/>
-    <col min="13" max="16" width="15.7265625" customWidth="1"/>
-    <col min="17" max="17" width="20.7265625" customWidth="1"/>
-    <col min="18" max="18" width="20.453125" customWidth="1"/>
-    <col min="19" max="19" width="20.54296875" customWidth="1"/>
-    <col min="20" max="21" width="15.7265625" customWidth="1"/>
-    <col min="22" max="23" width="20.7265625" customWidth="1"/>
-    <col min="24" max="24" width="22.7265625" customWidth="1"/>
-    <col min="25" max="25" width="15.7265625" customWidth="1"/>
-    <col min="26" max="27" width="20.1796875" customWidth="1"/>
-    <col min="28" max="28" width="20.453125" customWidth="1"/>
-    <col min="29" max="29" width="19.453125" customWidth="1"/>
-    <col min="30" max="31" width="24.54296875" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="29.85546875" customWidth="1"/>
+    <col min="4" max="6" width="15.7109375" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" customWidth="1"/>
+    <col min="8" max="9" width="15.7109375" customWidth="1"/>
+    <col min="10" max="12" width="21.7109375" customWidth="1"/>
+    <col min="13" max="16" width="15.7109375" customWidth="1"/>
+    <col min="17" max="17" width="20.7109375" customWidth="1"/>
+    <col min="18" max="18" width="20.42578125" customWidth="1"/>
+    <col min="19" max="19" width="20.5703125" customWidth="1"/>
+    <col min="20" max="21" width="15.7109375" customWidth="1"/>
+    <col min="22" max="23" width="20.7109375" customWidth="1"/>
+    <col min="24" max="24" width="15.7109375" customWidth="1"/>
+    <col min="25" max="26" width="20.140625" customWidth="1"/>
+    <col min="27" max="27" width="20.42578125" customWidth="1"/>
+    <col min="28" max="28" width="19.42578125" customWidth="1"/>
+    <col min="29" max="30" width="24.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:30" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1103,17 +1100,16 @@
       <c r="AB1" s="1"/>
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
-      <c r="AE1" s="1"/>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
@@ -1139,16 +1135,16 @@
         <v>8</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="M3" s="5" t="s">
         <v>9</v>
@@ -1166,10 +1162,10 @@
         <v>13</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="T3" s="5" t="s">
         <v>14</v>
@@ -1204,46 +1200,43 @@
       <c r="AD3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="AE3" s="5" t="s">
+    </row>
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
+      <c r="B4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>30</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>6</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="M4" s="6" t="s">
         <v>9</v>
@@ -1255,16 +1248,16 @@
         <v>11</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Q4" s="6" t="s">
         <v>13</v>
       </c>
       <c r="R4" s="6" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="S4" s="6" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="T4" s="6" t="s">
         <v>14</v>
@@ -1279,324 +1272,312 @@
         <v>17</v>
       </c>
       <c r="X4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y4" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z4" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="Y4" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="Z4" s="6" t="s">
+      <c r="AA4" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="AA4" s="6" t="s">
+      <c r="AB4" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="AB4" s="6" t="s">
+      <c r="AC4" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="AC4" s="6" t="s">
+      <c r="AD4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="AD4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="AE4" s="6" t="s">
-        <v>38</v>
-      </c>
     </row>
-    <row r="5" spans="1:31" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:30" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="E5" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="J5" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="M5" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="N5" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="J5" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="M5" s="7" t="s">
+      <c r="O5" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="N5" s="7" t="s">
+      <c r="P5" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="Q5" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="R5" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="Q5" s="7" t="s">
+      <c r="S5" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="T5" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="R5" s="7" t="s">
+      <c r="U5" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="S5" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="T5" s="7" t="s">
+      <c r="V5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="U5" s="7" t="s">
+      <c r="W5" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="V5" s="7" t="s">
+      <c r="X5" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="W5" s="7" t="s">
+      <c r="Y5" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="X5" s="7" t="s">
+      <c r="Z5" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="Y5" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z5" s="7" t="s">
-        <v>59</v>
-      </c>
       <c r="AA5" s="7" t="s">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="AB5" s="7" t="s">
         <v>22</v>
       </c>
       <c r="AC5" s="7" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="AD5" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="AE5" s="7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:31" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:30" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="L6" s="8"/>
       <c r="M6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="N6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="O6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="P6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="Q6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="R6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="S6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="T6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="U6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="W6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="X6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="Y6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="Z6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="AA6" s="8" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="AB6" s="8" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="AC6" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="AD6" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="AE6" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="9"/>
       <c r="B7" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="F7" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="G7" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="L7" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="N7" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="O7" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="F7" s="9" t="s">
+      <c r="P7" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q7" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="G7" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="K7" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="L7" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="M7" s="9" t="s">
+      <c r="R7" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="S7" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="T7" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="U7" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="V7" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="N7" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="O7" s="9" t="s">
+      <c r="W7" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="P7" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q7" s="9" t="s">
+      <c r="X7" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y7" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="R7" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="S7" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="T7" s="9" t="s">
+      <c r="Z7" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="U7" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="V7" s="9" t="s">
+      <c r="AA7" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="AB7" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="AC7" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="W7" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="X7" s="9" t="s">
+      <c r="AD7" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="Y7" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="Z7" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="AA7" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="AB7" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="AC7" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="AD7" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="AE7" s="9" t="s">
-        <v>80</v>
-      </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="19"/>
       <c r="C8" s="18" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F8" s="12">
         <v>1</v>
       </c>
-      <c r="G8" s="20">
-        <v>54909.846575342461</v>
+      <c r="G8" s="22">
+        <v>18795.432911392403</v>
       </c>
       <c r="H8" s="13">
         <v>0</v>
@@ -1604,14 +1585,14 @@
       <c r="I8" s="13">
         <v>0</v>
       </c>
-      <c r="J8" s="20">
-        <v>4.7350341735748772E-4</v>
+      <c r="J8" s="22">
+        <v>1.3833147724009441E-3</v>
       </c>
       <c r="K8" s="14">
         <v>0</v>
       </c>
       <c r="L8" s="14">
-        <v>658918.1589041095</v>
+        <v>225545.19493670884</v>
       </c>
       <c r="M8" s="13"/>
       <c r="N8" s="13"/>
@@ -1624,10 +1605,10 @@
       <c r="Q8" s="12">
         <v>0</v>
       </c>
-      <c r="R8" s="20">
+      <c r="R8" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S8" s="22">
+      <c r="S8" s="24">
         <v>0</v>
       </c>
       <c r="T8" s="12">
@@ -1642,45 +1623,41 @@
       <c r="W8" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X8" s="13">
-        <f>L8/G8</f>
-        <v>12</v>
-      </c>
-      <c r="Y8" s="15"/>
-      <c r="Z8" s="12">
+      <c r="X8" s="15"/>
+      <c r="Y8" s="12">
         <v>1960</v>
       </c>
-      <c r="AA8" s="12"/>
+      <c r="Z8" s="12"/>
+      <c r="AA8" s="16">
+        <v>46.766666710000003</v>
+      </c>
       <c r="AB8" s="16">
-        <v>46.766666710000003</v>
-      </c>
-      <c r="AC8" s="16">
         <v>15.55000001</v>
       </c>
+      <c r="AC8" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD8" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE8" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" s="19"/>
       <c r="C9" s="18" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F9" s="12">
         <v>1</v>
       </c>
-      <c r="G9" s="20">
-        <v>26170.257945205503</v>
+      <c r="G9" s="22">
+        <v>76314.213344048214</v>
       </c>
       <c r="H9" s="13">
         <v>0</v>
@@ -1688,14 +1665,14 @@
       <c r="I9" s="13">
         <v>0</v>
       </c>
-      <c r="J9" s="20">
-        <v>1.2609734328600966E-3</v>
+      <c r="J9" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K9" s="14">
         <v>0</v>
       </c>
       <c r="L9" s="14">
-        <v>314043.09534246603</v>
+        <v>915770.56012857857</v>
       </c>
       <c r="M9" s="13"/>
       <c r="N9" s="13"/>
@@ -1708,10 +1685,10 @@
       <c r="Q9" s="12">
         <v>0</v>
       </c>
-      <c r="R9" s="20">
+      <c r="R9" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S9" s="22">
+      <c r="S9" s="24">
         <v>0</v>
       </c>
       <c r="T9" s="12">
@@ -1726,58 +1703,54 @@
       <c r="W9" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X9" s="13">
-        <f t="shared" ref="X9:X43" si="0">L9/G9</f>
-        <v>12</v>
-      </c>
-      <c r="Y9" s="15"/>
+      <c r="X9" s="15"/>
+      <c r="Y9" s="12"/>
       <c r="Z9" s="12"/>
-      <c r="AA9" s="12"/>
+      <c r="AA9" s="16">
+        <v>47.049999010000001</v>
+      </c>
       <c r="AB9" s="16">
-        <v>47.049999010000001</v>
-      </c>
-      <c r="AC9" s="16">
         <v>15.19400001</v>
       </c>
+      <c r="AC9" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD9" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE9" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="19"/>
       <c r="C10" s="18" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F10" s="12">
         <v>1</v>
       </c>
-      <c r="G10" s="20">
-        <v>90723.6</v>
+      <c r="G10" s="22">
+        <v>197455.68000000002</v>
       </c>
       <c r="H10" s="13">
         <v>0</v>
       </c>
-      <c r="I10" s="20">
-        <v>11095.429726027354</v>
-      </c>
-      <c r="J10" s="20">
-        <v>3.7476466983232587E-4</v>
+      <c r="I10" s="21">
+        <v>123.1396524</v>
+      </c>
+      <c r="J10" s="22">
+        <v>1.7219053916301622E-4</v>
       </c>
       <c r="K10" s="20">
-        <v>3.7476466983232587E-4</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="L10" s="14">
-        <v>1088683.2000000002</v>
+        <v>2369468.16</v>
       </c>
       <c r="M10" s="13"/>
       <c r="N10" s="13"/>
@@ -1790,10 +1763,10 @@
       <c r="Q10" s="12">
         <v>0</v>
       </c>
-      <c r="R10" s="20">
+      <c r="R10" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S10" s="20">
+      <c r="S10" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
       <c r="T10" s="12">
@@ -1808,45 +1781,41 @@
       <c r="W10" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X10" s="13">
-        <f t="shared" si="0"/>
-        <v>12.000000000000002</v>
-      </c>
-      <c r="Y10" s="15"/>
-      <c r="Z10" s="12">
+      <c r="X10" s="15"/>
+      <c r="Y10" s="12">
         <v>1982</v>
       </c>
-      <c r="AA10" s="12"/>
+      <c r="Z10" s="12"/>
+      <c r="AA10" s="16">
+        <v>47.107686170000001</v>
+      </c>
       <c r="AB10" s="16">
-        <v>47.107686170000001</v>
-      </c>
-      <c r="AC10" s="16">
         <v>14.065534960000001</v>
       </c>
+      <c r="AC10" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD10" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE10" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="B11" s="19"/>
       <c r="C11" s="18" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F11" s="12">
         <v>1</v>
       </c>
-      <c r="G11" s="20">
-        <v>303080.53109589039</v>
+      <c r="G11" s="22">
+        <v>117304.04284051221</v>
       </c>
       <c r="H11" s="13">
         <v>0</v>
@@ -1854,14 +1823,14 @@
       <c r="I11" s="13">
         <v>0</v>
       </c>
-      <c r="J11" s="20">
-        <v>5.2791249712235146E-5</v>
+      <c r="J11" s="22">
+        <v>1.3639768598388177E-4</v>
       </c>
       <c r="K11" s="14">
         <v>0</v>
       </c>
       <c r="L11" s="14">
-        <v>3636966.3731506849</v>
+        <v>1407648.5140861464</v>
       </c>
       <c r="M11" s="13"/>
       <c r="N11" s="13"/>
@@ -1874,10 +1843,10 @@
       <c r="Q11" s="12">
         <v>0</v>
       </c>
-      <c r="R11" s="20">
+      <c r="R11" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S11" s="22">
+      <c r="S11" s="24">
         <v>0</v>
       </c>
       <c r="T11" s="12">
@@ -1892,45 +1861,41 @@
       <c r="W11" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X11" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y11" s="15"/>
-      <c r="Z11" s="12">
+      <c r="X11" s="15"/>
+      <c r="Y11" s="12">
         <v>1949</v>
       </c>
-      <c r="AA11" s="12"/>
+      <c r="Z11" s="12"/>
+      <c r="AA11" s="16">
+        <v>47.410000009999997</v>
+      </c>
       <c r="AB11" s="16">
-        <v>47.410000009999997</v>
-      </c>
-      <c r="AC11" s="16">
         <v>15.214</v>
       </c>
+      <c r="AC11" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD11" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE11" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>
       <c r="B12" s="19"/>
       <c r="C12" s="18" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F12" s="12">
         <v>1</v>
       </c>
-      <c r="G12" s="20">
-        <v>38620.287567119769</v>
+      <c r="G12" s="22">
+        <v>50876.142229365476</v>
       </c>
       <c r="H12" s="13">
         <v>0</v>
@@ -1938,14 +1903,14 @@
       <c r="I12" s="13">
         <v>0</v>
       </c>
-      <c r="J12" s="20">
-        <v>5.6964878787516286E-4</v>
+      <c r="J12" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K12" s="14">
         <v>0</v>
       </c>
       <c r="L12" s="14">
-        <v>463443.45080543723</v>
+        <v>610513.70675238571</v>
       </c>
       <c r="M12" s="13"/>
       <c r="N12" s="13"/>
@@ -1958,10 +1923,10 @@
       <c r="Q12" s="12">
         <v>0</v>
       </c>
-      <c r="R12" s="20">
+      <c r="R12" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S12" s="22">
+      <c r="S12" s="24">
         <v>0</v>
       </c>
       <c r="T12" s="12">
@@ -1976,45 +1941,41 @@
       <c r="W12" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X12" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y12" s="15"/>
-      <c r="Z12" s="12">
+      <c r="X12" s="15"/>
+      <c r="Y12" s="12">
         <v>1994</v>
       </c>
-      <c r="AA12" s="12"/>
+      <c r="Z12" s="12"/>
+      <c r="AA12" s="16">
+        <v>47.174263209999999</v>
+      </c>
       <c r="AB12" s="16">
-        <v>47.174263209999999</v>
-      </c>
-      <c r="AC12" s="16">
         <v>14.722779259999999</v>
       </c>
+      <c r="AC12" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD12" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE12" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
       <c r="B13" s="19"/>
       <c r="C13" s="18" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F13" s="12">
         <v>1</v>
       </c>
-      <c r="G13" s="20">
-        <v>308190.13232876715</v>
+      <c r="G13" s="22">
+        <v>128145.67200000001</v>
       </c>
       <c r="H13" s="13">
         <v>0</v>
@@ -2022,14 +1983,14 @@
       <c r="I13" s="13">
         <v>0</v>
       </c>
-      <c r="J13" s="20">
-        <v>3.8937002652631305E-5</v>
+      <c r="J13" s="22">
+        <v>9.3643427926305622E-5</v>
       </c>
       <c r="K13" s="14">
         <v>0</v>
       </c>
       <c r="L13" s="14">
-        <v>3698281.5879452061</v>
+        <v>1537748.064</v>
       </c>
       <c r="M13" s="13"/>
       <c r="N13" s="13"/>
@@ -2042,10 +2003,10 @@
       <c r="Q13" s="12">
         <v>0</v>
       </c>
-      <c r="R13" s="20">
+      <c r="R13" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S13" s="22">
+      <c r="S13" s="24">
         <v>0</v>
       </c>
       <c r="T13" s="12">
@@ -2060,45 +2021,41 @@
       <c r="W13" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X13" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y13" s="15"/>
-      <c r="Z13" s="12">
+      <c r="X13" s="15"/>
+      <c r="Y13" s="12">
         <v>1998</v>
       </c>
-      <c r="AA13" s="12"/>
+      <c r="Z13" s="12"/>
+      <c r="AA13" s="16">
+        <v>47.186513009999999</v>
+      </c>
       <c r="AB13" s="16">
-        <v>47.186513009999999</v>
-      </c>
-      <c r="AC13" s="16">
         <v>15.33601401</v>
       </c>
+      <c r="AC13" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD13" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE13" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="10"/>
       <c r="B14" s="19"/>
       <c r="C14" s="18" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F14" s="12">
         <v>1</v>
       </c>
-      <c r="G14" s="20">
-        <v>467759.68356164393</v>
+      <c r="G14" s="22">
+        <v>192549.84</v>
       </c>
       <c r="H14" s="13">
         <v>0</v>
@@ -2106,14 +2063,14 @@
       <c r="I14" s="13">
         <v>0</v>
       </c>
-      <c r="J14" s="20">
-        <v>2.9929898817701346E-5</v>
+      <c r="J14" s="22">
+        <v>7.2708447849138697E-5</v>
       </c>
       <c r="K14" s="14">
         <v>0</v>
       </c>
       <c r="L14" s="14">
-        <v>5613116.2027397268</v>
+        <v>2310598.08</v>
       </c>
       <c r="M14" s="13"/>
       <c r="N14" s="13"/>
@@ -2126,10 +2083,10 @@
       <c r="Q14" s="12">
         <v>0</v>
       </c>
-      <c r="R14" s="20">
+      <c r="R14" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S14" s="22">
+      <c r="S14" s="24">
         <v>0</v>
       </c>
       <c r="T14" s="12">
@@ -2144,45 +2101,41 @@
       <c r="W14" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X14" s="13">
-        <f t="shared" si="0"/>
-        <v>11.999999999999998</v>
-      </c>
-      <c r="Y14" s="15"/>
-      <c r="Z14" s="12">
+      <c r="X14" s="15"/>
+      <c r="Y14" s="12">
         <v>1974</v>
       </c>
-      <c r="AA14" s="12"/>
+      <c r="Z14" s="12"/>
+      <c r="AA14" s="16">
+        <v>46.785117999999997</v>
+      </c>
       <c r="AB14" s="16">
-        <v>46.785117999999997</v>
-      </c>
-      <c r="AC14" s="16">
         <v>15.58555701</v>
       </c>
+      <c r="AC14" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD14" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE14" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
       <c r="B15" s="19"/>
       <c r="C15" s="18" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F15" s="12">
         <v>1</v>
       </c>
-      <c r="G15" s="20">
-        <v>729653.91196388274</v>
+      <c r="G15" s="22">
+        <v>168293.23855530474</v>
       </c>
       <c r="H15" s="13">
         <v>0</v>
@@ -2190,14 +2143,14 @@
       <c r="I15" s="13">
         <v>0</v>
       </c>
-      <c r="J15" s="20">
-        <v>2.6039742525139078E-5</v>
+      <c r="J15" s="22">
+        <v>1.12898177984472E-4</v>
       </c>
       <c r="K15" s="14">
         <v>0</v>
       </c>
       <c r="L15" s="14">
-        <v>8755846.9435665924</v>
+        <v>2019518.8626636569</v>
       </c>
       <c r="M15" s="13"/>
       <c r="N15" s="13"/>
@@ -2210,10 +2163,10 @@
       <c r="Q15" s="12">
         <v>0</v>
       </c>
-      <c r="R15" s="20">
+      <c r="R15" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S15" s="22">
+      <c r="S15" s="24">
         <v>0</v>
       </c>
       <c r="T15" s="12">
@@ -2228,45 +2181,41 @@
       <c r="W15" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X15" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y15" s="15"/>
-      <c r="Z15" s="12">
+      <c r="X15" s="15"/>
+      <c r="Y15" s="12">
         <v>2011</v>
       </c>
-      <c r="AA15" s="12"/>
+      <c r="Z15" s="12"/>
+      <c r="AA15" s="16">
+        <v>46.997841010000002</v>
+      </c>
       <c r="AB15" s="16">
-        <v>46.997841010000002</v>
-      </c>
-      <c r="AC15" s="16">
         <v>15.46751901</v>
       </c>
+      <c r="AC15" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD15" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE15" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="10"/>
       <c r="B16" s="19"/>
       <c r="C16" s="18" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F16" s="12">
         <v>1</v>
       </c>
-      <c r="G16" s="20">
-        <v>467759.68356164393</v>
+      <c r="G16" s="22">
+        <v>735583.65842696629</v>
       </c>
       <c r="H16" s="13">
         <v>0</v>
@@ -2274,14 +2223,14 @@
       <c r="I16" s="13">
         <v>0</v>
       </c>
-      <c r="J16" s="20">
-        <v>2.9929898817701346E-5</v>
+      <c r="J16" s="22">
+        <v>1.9032505466392189E-5</v>
       </c>
       <c r="K16" s="14">
         <v>0</v>
       </c>
       <c r="L16" s="14">
-        <v>5613116.2027397268</v>
+        <v>8827003.9011235945</v>
       </c>
       <c r="M16" s="13"/>
       <c r="N16" s="13"/>
@@ -2294,10 +2243,10 @@
       <c r="Q16" s="12">
         <v>0</v>
       </c>
-      <c r="R16" s="20">
+      <c r="R16" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S16" s="22">
+      <c r="S16" s="24">
         <v>0</v>
       </c>
       <c r="T16" s="12">
@@ -2312,45 +2261,41 @@
       <c r="W16" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X16" s="13">
-        <f t="shared" si="0"/>
-        <v>11.999999999999998</v>
-      </c>
-      <c r="Y16" s="15"/>
-      <c r="Z16" s="12">
+      <c r="X16" s="15"/>
+      <c r="Y16" s="12">
         <v>1964</v>
       </c>
-      <c r="AA16" s="12"/>
+      <c r="Z16" s="12"/>
+      <c r="AA16" s="16">
+        <v>46.828090680000003</v>
+      </c>
       <c r="AB16" s="16">
-        <v>46.828090680000003</v>
-      </c>
-      <c r="AC16" s="16">
         <v>15.566165529999999</v>
       </c>
+      <c r="AC16" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD16" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE16" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="19"/>
       <c r="C17" s="18" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F17" s="12">
         <v>1</v>
       </c>
-      <c r="G17" s="20">
-        <v>413303.9589041096</v>
+      <c r="G17" s="22">
+        <v>184888.02933333334</v>
       </c>
       <c r="H17" s="13">
         <v>0</v>
@@ -2358,14 +2303,14 @@
       <c r="I17" s="13">
         <v>0</v>
       </c>
-      <c r="J17" s="20">
-        <v>2.6614794663876189E-5</v>
+      <c r="J17" s="22">
+        <v>5.9495468904415532E-5</v>
       </c>
       <c r="K17" s="14">
         <v>0</v>
       </c>
       <c r="L17" s="14">
-        <v>4959647.506849315</v>
+        <v>2218656.352</v>
       </c>
       <c r="M17" s="13"/>
       <c r="N17" s="13"/>
@@ -2378,10 +2323,10 @@
       <c r="Q17" s="12">
         <v>0</v>
       </c>
-      <c r="R17" s="20">
+      <c r="R17" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S17" s="22">
+      <c r="S17" s="24">
         <v>0</v>
       </c>
       <c r="T17" s="12">
@@ -2396,45 +2341,41 @@
       <c r="W17" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X17" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y17" s="15"/>
-      <c r="Z17" s="12">
+      <c r="X17" s="15"/>
+      <c r="Y17" s="12">
         <v>2024</v>
       </c>
-      <c r="AA17" s="12"/>
+      <c r="Z17" s="12"/>
+      <c r="AA17" s="16">
+        <v>47.139091010000001</v>
+      </c>
       <c r="AB17" s="16">
-        <v>47.139091010000001</v>
-      </c>
-      <c r="AC17" s="16">
         <v>15.32804601</v>
       </c>
+      <c r="AC17" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD17" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE17" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="10"/>
       <c r="B18" s="19"/>
       <c r="C18" s="18" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F18" s="12">
         <v>1</v>
       </c>
-      <c r="G18" s="20">
-        <v>388412.26027397258</v>
+      <c r="G18" s="22">
+        <v>169397.1903512195</v>
       </c>
       <c r="H18" s="13">
         <v>0</v>
@@ -2442,14 +2383,14 @@
       <c r="I18" s="13">
         <v>0</v>
       </c>
-      <c r="J18" s="20">
-        <v>4.5570137223565063E-5</v>
+      <c r="J18" s="22">
+        <v>1.0448815569668966E-4</v>
       </c>
       <c r="K18" s="14">
         <v>0</v>
       </c>
       <c r="L18" s="14">
-        <v>4660947.1232876712</v>
+        <v>2032766.284214634</v>
       </c>
       <c r="M18" s="13"/>
       <c r="N18" s="13"/>
@@ -2462,10 +2403,10 @@
       <c r="Q18" s="12">
         <v>0</v>
       </c>
-      <c r="R18" s="20">
+      <c r="R18" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S18" s="22">
+      <c r="S18" s="24">
         <v>0</v>
       </c>
       <c r="T18" s="12">
@@ -2480,43 +2421,39 @@
       <c r="W18" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X18" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y18" s="15"/>
+      <c r="X18" s="15"/>
+      <c r="Y18" s="12"/>
       <c r="Z18" s="12"/>
-      <c r="AA18" s="12"/>
+      <c r="AA18" s="16">
+        <v>47.039863869999998</v>
+      </c>
       <c r="AB18" s="16">
-        <v>47.039863869999998</v>
-      </c>
-      <c r="AC18" s="16">
         <v>15.442751360000001</v>
       </c>
+      <c r="AC18" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD18" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE18" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="10"/>
       <c r="B19" s="19"/>
       <c r="C19" s="18" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F19" s="12">
         <v>1</v>
       </c>
-      <c r="G19" s="20">
-        <v>26170.2579452055</v>
+      <c r="G19" s="22">
+        <v>13875.311517099675</v>
       </c>
       <c r="H19" s="13">
         <v>0</v>
@@ -2524,14 +2461,14 @@
       <c r="I19" s="13">
         <v>0</v>
       </c>
-      <c r="J19" s="20">
-        <v>2.2926789688365392E-4</v>
+      <c r="J19" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K19" s="14">
         <v>0</v>
       </c>
       <c r="L19" s="14">
-        <v>314043.09534246603</v>
+        <v>166503.7382051961</v>
       </c>
       <c r="M19" s="13"/>
       <c r="N19" s="13"/>
@@ -2544,10 +2481,10 @@
       <c r="Q19" s="12">
         <v>0</v>
       </c>
-      <c r="R19" s="20">
+      <c r="R19" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S19" s="22">
+      <c r="S19" s="24">
         <v>0</v>
       </c>
       <c r="T19" s="12">
@@ -2562,43 +2499,39 @@
       <c r="W19" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X19" s="13">
-        <f t="shared" si="0"/>
-        <v>12.000000000000002</v>
-      </c>
-      <c r="Y19" s="15"/>
+      <c r="X19" s="15"/>
+      <c r="Y19" s="12"/>
       <c r="Z19" s="12"/>
-      <c r="AA19" s="12"/>
+      <c r="AA19" s="16">
+        <v>46.994091240000003</v>
+      </c>
       <c r="AB19" s="16">
-        <v>46.994091240000003</v>
-      </c>
-      <c r="AC19" s="16">
         <v>15.085024949999999</v>
       </c>
+      <c r="AC19" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD19" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE19" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="10"/>
       <c r="B20" s="19"/>
       <c r="C20" s="18" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F20" s="12">
         <v>1</v>
       </c>
-      <c r="G20" s="20">
-        <v>11095.429726027354</v>
+      <c r="G20" s="22">
+        <v>21107.257600000001</v>
       </c>
       <c r="H20" s="13">
         <v>0</v>
@@ -2606,8 +2539,8 @@
       <c r="I20" s="13">
         <v>0</v>
       </c>
-      <c r="J20" s="20">
-        <v>9.3732286687409367E-3</v>
+      <c r="J20" s="22">
+        <v>4.9272151773994549E-3</v>
       </c>
       <c r="K20" s="14">
         <v>0</v>
@@ -2626,10 +2559,10 @@
       <c r="Q20" s="12">
         <v>1</v>
       </c>
-      <c r="R20" s="20">
+      <c r="R20" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S20" s="22">
+      <c r="S20" s="24">
         <v>0</v>
       </c>
       <c r="T20" s="12">
@@ -2644,43 +2577,39 @@
       <c r="W20" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X20" s="13">
-        <f t="shared" si="0"/>
-        <v>1351.9079810684045</v>
-      </c>
-      <c r="Y20" s="15"/>
+      <c r="X20" s="15"/>
+      <c r="Y20" s="12"/>
       <c r="Z20" s="12"/>
-      <c r="AA20" s="12"/>
+      <c r="AA20" s="16">
+        <v>47.10370743</v>
+      </c>
       <c r="AB20" s="16">
-        <v>47.10370743</v>
-      </c>
-      <c r="AC20" s="16">
         <v>13.481122409999999</v>
       </c>
+      <c r="AC20" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD20" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE20" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="10"/>
       <c r="B21" s="19"/>
       <c r="C21" s="18" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F21" s="12">
         <v>1</v>
       </c>
-      <c r="G21" s="20">
-        <v>388412.26027397258</v>
+      <c r="G21" s="22">
+        <v>183607.69530845954</v>
       </c>
       <c r="H21" s="13">
         <v>0</v>
@@ -2688,14 +2617,14 @@
       <c r="I21" s="13">
         <v>0</v>
       </c>
-      <c r="J21" s="20">
-        <v>4.8917096454674359E-5</v>
+      <c r="J21" s="22">
+        <v>1.0348150151375814E-4</v>
       </c>
       <c r="K21" s="14">
         <v>0</v>
       </c>
       <c r="L21" s="14">
-        <v>4660947.1232876712</v>
+        <v>2203292.3437015144</v>
       </c>
       <c r="M21" s="13"/>
       <c r="N21" s="13"/>
@@ -2708,10 +2637,10 @@
       <c r="Q21" s="12">
         <v>0</v>
       </c>
-      <c r="R21" s="20">
+      <c r="R21" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S21" s="22">
+      <c r="S21" s="24">
         <v>0</v>
       </c>
       <c r="T21" s="12">
@@ -2726,45 +2655,41 @@
       <c r="W21" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X21" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y21" s="15"/>
-      <c r="Z21" s="12">
+      <c r="X21" s="15"/>
+      <c r="Y21" s="12">
         <v>2013</v>
       </c>
-      <c r="AA21" s="12"/>
+      <c r="Z21" s="12"/>
+      <c r="AA21" s="16">
+        <v>46.943604610000001</v>
+      </c>
       <c r="AB21" s="16">
-        <v>46.943604610000001</v>
-      </c>
-      <c r="AC21" s="16">
         <v>15.5040946</v>
       </c>
+      <c r="AC21" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD21" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE21" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="10"/>
       <c r="B22" s="19"/>
       <c r="C22" s="18" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F22" s="12">
         <v>1</v>
       </c>
-      <c r="G22" s="20">
-        <v>391003.39726027398</v>
+      <c r="G22" s="22">
+        <v>122730.03966942149</v>
       </c>
       <c r="H22" s="13">
         <v>0</v>
@@ -2772,14 +2697,14 @@
       <c r="I22" s="13">
         <v>0</v>
       </c>
-      <c r="J22" s="20">
-        <v>4.6035405641292117E-5</v>
+      <c r="J22" s="22">
+        <v>1.4666336007454863E-4</v>
       </c>
       <c r="K22" s="14">
         <v>0</v>
       </c>
       <c r="L22" s="14">
-        <v>4692040.7671232875</v>
+        <v>1472760.4760330578</v>
       </c>
       <c r="M22" s="13"/>
       <c r="N22" s="13"/>
@@ -2792,10 +2717,10 @@
       <c r="Q22" s="12">
         <v>0</v>
       </c>
-      <c r="R22" s="20">
+      <c r="R22" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S22" s="22">
+      <c r="S22" s="24">
         <v>0</v>
       </c>
       <c r="T22" s="12">
@@ -2810,45 +2735,41 @@
       <c r="W22" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X22" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y22" s="15"/>
-      <c r="Z22" s="12">
+      <c r="X22" s="15"/>
+      <c r="Y22" s="12">
         <v>2023</v>
       </c>
-      <c r="AA22" s="12"/>
+      <c r="Z22" s="12"/>
+      <c r="AA22" s="16">
+        <v>47.292000010000002</v>
+      </c>
       <c r="AB22" s="16">
-        <v>47.292000010000002</v>
-      </c>
-      <c r="AC22" s="16">
         <v>15.323</v>
       </c>
+      <c r="AC22" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD22" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE22" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="10"/>
       <c r="B23" s="19"/>
       <c r="C23" s="18" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F23" s="12">
         <v>1</v>
       </c>
-      <c r="G23" s="20">
-        <v>467759.68356164382</v>
+      <c r="G23" s="22">
+        <v>111471.04648390942</v>
       </c>
       <c r="H23" s="13">
         <v>0</v>
@@ -2856,14 +2777,14 @@
       <c r="I23" s="13">
         <v>0</v>
       </c>
-      <c r="J23" s="20">
-        <v>2.1378499155500961E-5</v>
+      <c r="J23" s="22">
+        <v>8.9709393743275537E-5</v>
       </c>
       <c r="K23" s="14">
         <v>0</v>
       </c>
       <c r="L23" s="14">
-        <v>5613116.2027397258</v>
+        <v>1337652.557806913</v>
       </c>
       <c r="M23" s="13"/>
       <c r="N23" s="13"/>
@@ -2876,10 +2797,10 @@
       <c r="Q23" s="12">
         <v>0</v>
       </c>
-      <c r="R23" s="20">
+      <c r="R23" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S23" s="22">
+      <c r="S23" s="24">
         <v>0</v>
       </c>
       <c r="T23" s="12">
@@ -2894,45 +2815,41 @@
       <c r="W23" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X23" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y23" s="15"/>
-      <c r="Z23" s="12">
+      <c r="X23" s="15"/>
+      <c r="Y23" s="12">
         <v>1988</v>
       </c>
-      <c r="AA23" s="12"/>
+      <c r="Z23" s="12"/>
+      <c r="AA23" s="16">
+        <v>46.857847</v>
+      </c>
       <c r="AB23" s="16">
-        <v>46.857847</v>
-      </c>
-      <c r="AC23" s="16">
         <v>15.537300009999999</v>
       </c>
+      <c r="AC23" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD23" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE23" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="10"/>
       <c r="B24" s="19"/>
       <c r="C24" s="18" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F24" s="12">
         <v>1</v>
       </c>
-      <c r="G24" s="20">
-        <v>303080.53109589039</v>
+      <c r="G24" s="22">
+        <v>146262.2694969576</v>
       </c>
       <c r="H24" s="13">
         <v>0</v>
@@ -2940,14 +2857,14 @@
       <c r="I24" s="13">
         <v>0</v>
       </c>
-      <c r="J24" s="20">
-        <v>3.2994531070146968E-5</v>
+      <c r="J24" s="22">
+        <v>6.8370332515645875E-5</v>
       </c>
       <c r="K24" s="14">
         <v>0</v>
       </c>
       <c r="L24" s="14">
-        <v>3636966.3731506849</v>
+        <v>1755147.2339634912</v>
       </c>
       <c r="M24" s="13"/>
       <c r="N24" s="13"/>
@@ -2960,10 +2877,10 @@
       <c r="Q24" s="12">
         <v>0</v>
       </c>
-      <c r="R24" s="20">
+      <c r="R24" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S24" s="22">
+      <c r="S24" s="24">
         <v>0</v>
       </c>
       <c r="T24" s="12">
@@ -2978,43 +2895,39 @@
       <c r="W24" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X24" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y24" s="15"/>
+      <c r="X24" s="15"/>
+      <c r="Y24" s="12"/>
       <c r="Z24" s="12"/>
-      <c r="AA24" s="12"/>
+      <c r="AA24" s="16">
+        <v>47.388476009999998</v>
+      </c>
       <c r="AB24" s="16">
-        <v>47.388476009999998</v>
-      </c>
-      <c r="AC24" s="16">
         <v>15.095160999999999</v>
       </c>
+      <c r="AC24" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD24" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE24" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="10"/>
       <c r="B25" s="19"/>
       <c r="C25" s="18" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F25" s="12">
         <v>1</v>
       </c>
-      <c r="G25" s="20">
-        <v>467759.68356164382</v>
+      <c r="G25" s="22">
+        <v>30063.174953715963</v>
       </c>
       <c r="H25" s="13">
         <v>0</v>
@@ -3022,14 +2935,14 @@
       <c r="I25" s="13">
         <v>0</v>
       </c>
-      <c r="J25" s="20">
-        <v>2.779204890215125E-5</v>
+      <c r="J25" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K25" s="14">
         <v>0</v>
       </c>
       <c r="L25" s="14">
-        <v>5613116.2027397258</v>
+        <v>360758.09944459156</v>
       </c>
       <c r="M25" s="13"/>
       <c r="N25" s="13"/>
@@ -3042,10 +2955,10 @@
       <c r="Q25" s="12">
         <v>0</v>
       </c>
-      <c r="R25" s="20">
+      <c r="R25" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S25" s="22">
+      <c r="S25" s="24">
         <v>0</v>
       </c>
       <c r="T25" s="12">
@@ -3060,43 +2973,39 @@
       <c r="W25" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X25" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y25" s="15"/>
+      <c r="X25" s="15"/>
+      <c r="Y25" s="12"/>
       <c r="Z25" s="12"/>
-      <c r="AA25" s="12"/>
+      <c r="AA25" s="16">
+        <v>46.745757689999998</v>
+      </c>
       <c r="AB25" s="16">
-        <v>46.745757689999998</v>
-      </c>
-      <c r="AC25" s="16">
         <v>15.57182718</v>
       </c>
+      <c r="AC25" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD25" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE25" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="10"/>
       <c r="B26" s="19"/>
       <c r="C26" s="18" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F26" s="12">
         <v>1</v>
       </c>
-      <c r="G26" s="20">
-        <v>26170.2579452055</v>
+      <c r="G26" s="22">
+        <v>34688.278792749188</v>
       </c>
       <c r="H26" s="13">
         <v>0</v>
@@ -3104,14 +3013,14 @@
       <c r="I26" s="13">
         <v>0</v>
       </c>
-      <c r="J26" s="20">
-        <v>5.7316974220913486E-4</v>
+      <c r="J26" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K26" s="14">
         <v>0</v>
       </c>
       <c r="L26" s="14">
-        <v>314043.09534246603</v>
+        <v>416259.34551299026</v>
       </c>
       <c r="M26" s="13"/>
       <c r="N26" s="13"/>
@@ -3124,10 +3033,10 @@
       <c r="Q26" s="12">
         <v>1</v>
       </c>
-      <c r="R26" s="20">
+      <c r="R26" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S26" s="22">
+      <c r="S26" s="24">
         <v>0</v>
       </c>
       <c r="T26" s="12">
@@ -3142,43 +3051,39 @@
       <c r="W26" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X26" s="13">
-        <f t="shared" si="0"/>
-        <v>12.000000000000002</v>
-      </c>
-      <c r="Y26" s="15"/>
+      <c r="X26" s="15"/>
+      <c r="Y26" s="12"/>
       <c r="Z26" s="12"/>
-      <c r="AA26" s="12"/>
+      <c r="AA26" s="16">
+        <v>46.978785770000002</v>
+      </c>
       <c r="AB26" s="16">
-        <v>46.978785770000002</v>
-      </c>
-      <c r="AC26" s="16">
         <v>15.023196179999999</v>
       </c>
+      <c r="AC26" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD26" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE26" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="10"/>
       <c r="B27" s="19"/>
       <c r="C27" s="18" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F27" s="12">
         <v>1</v>
       </c>
-      <c r="G27" s="20">
-        <v>391003.39726027398</v>
+      <c r="G27" s="22">
+        <v>131944.51443052923</v>
       </c>
       <c r="H27" s="13">
         <v>0</v>
@@ -3186,14 +3091,14 @@
       <c r="I27" s="13">
         <v>0</v>
       </c>
-      <c r="J27" s="20">
-        <v>3.324779296315542E-5</v>
+      <c r="J27" s="22">
+        <v>9.8526263529088916E-5</v>
       </c>
       <c r="K27" s="14">
         <v>0</v>
       </c>
       <c r="L27" s="14">
-        <v>4692040.7671232875</v>
+        <v>1583334.1731663509</v>
       </c>
       <c r="M27" s="13"/>
       <c r="N27" s="13"/>
@@ -3206,10 +3111,10 @@
       <c r="Q27" s="12">
         <v>0</v>
       </c>
-      <c r="R27" s="20">
+      <c r="R27" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S27" s="22">
+      <c r="S27" s="24">
         <v>0</v>
       </c>
       <c r="T27" s="12">
@@ -3224,45 +3129,41 @@
       <c r="W27" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X27" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y27" s="15"/>
-      <c r="Z27" s="12">
+      <c r="X27" s="15"/>
+      <c r="Y27" s="12">
         <v>2009</v>
       </c>
-      <c r="AA27" s="12"/>
+      <c r="Z27" s="12"/>
+      <c r="AA27" s="16">
+        <v>47.209260010000001</v>
+      </c>
       <c r="AB27" s="16">
-        <v>47.209260010000001</v>
-      </c>
-      <c r="AC27" s="16">
         <v>15.335656</v>
       </c>
+      <c r="AC27" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD27" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE27" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
       <c r="B28" s="19"/>
       <c r="C28" s="18" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F28" s="12">
         <v>1</v>
       </c>
-      <c r="G28" s="20">
-        <v>45642.158033868822</v>
+      <c r="G28" s="22">
+        <v>60126.349907431926</v>
       </c>
       <c r="H28" s="13">
         <v>0</v>
@@ -3270,14 +3171,14 @@
       <c r="I28" s="13">
         <v>0</v>
       </c>
-      <c r="J28" s="20">
-        <v>5.6964878787516286E-4</v>
+      <c r="J28" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K28" s="14">
         <v>0</v>
       </c>
       <c r="L28" s="14">
-        <v>547705.89640642586</v>
+        <v>721516.19888918311</v>
       </c>
       <c r="M28" s="13"/>
       <c r="N28" s="13"/>
@@ -3290,10 +3191,10 @@
       <c r="Q28" s="12">
         <v>0</v>
       </c>
-      <c r="R28" s="20">
+      <c r="R28" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S28" s="22">
+      <c r="S28" s="24">
         <v>0</v>
       </c>
       <c r="T28" s="12">
@@ -3308,45 +3209,41 @@
       <c r="W28" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X28" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y28" s="15"/>
-      <c r="Z28" s="12">
+      <c r="X28" s="15"/>
+      <c r="Y28" s="12">
         <v>2013</v>
       </c>
-      <c r="AA28" s="12"/>
+      <c r="Z28" s="12"/>
+      <c r="AA28" s="16">
+        <v>47.365200010000002</v>
+      </c>
       <c r="AB28" s="16">
-        <v>47.365200010000002</v>
-      </c>
-      <c r="AC28" s="16">
         <v>15.33440001</v>
       </c>
+      <c r="AC28" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD28" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE28" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="10"/>
       <c r="B29" s="19"/>
       <c r="C29" s="18" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F29" s="12">
         <v>1</v>
       </c>
-      <c r="G29" s="20">
-        <v>3510.9352333745246</v>
+      <c r="G29" s="22">
+        <v>4625.1038390332251</v>
       </c>
       <c r="H29" s="13">
         <v>0</v>
@@ -3354,14 +3251,14 @@
       <c r="I29" s="13">
         <v>0</v>
       </c>
-      <c r="J29" s="20">
-        <v>5.6964878787516286E-4</v>
+      <c r="J29" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K29" s="14">
         <v>0</v>
       </c>
       <c r="L29" s="14">
-        <v>42131.222800494295</v>
+        <v>55501.246068398701</v>
       </c>
       <c r="M29" s="13"/>
       <c r="N29" s="13"/>
@@ -3374,10 +3271,10 @@
       <c r="Q29" s="12">
         <v>0</v>
       </c>
-      <c r="R29" s="20">
+      <c r="R29" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S29" s="22">
+      <c r="S29" s="24">
         <v>0</v>
       </c>
       <c r="T29" s="12">
@@ -3392,43 +3289,39 @@
       <c r="W29" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X29" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y29" s="15"/>
+      <c r="X29" s="15"/>
+      <c r="Y29" s="12"/>
       <c r="Z29" s="12"/>
-      <c r="AA29" s="12"/>
+      <c r="AA29" s="16">
+        <v>47.217744009999997</v>
+      </c>
       <c r="AB29" s="16">
-        <v>47.217744009999997</v>
-      </c>
-      <c r="AC29" s="16">
         <v>14.599074999999999</v>
       </c>
+      <c r="AC29" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD29" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE29" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="10"/>
       <c r="B30" s="19"/>
       <c r="C30" s="18" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F30" s="12">
         <v>1</v>
       </c>
-      <c r="G30" s="20">
-        <v>391003.39726027398</v>
+      <c r="G30" s="22">
+        <v>179073.80465116279</v>
       </c>
       <c r="H30" s="13">
         <v>0</v>
@@ -3436,14 +3329,14 @@
       <c r="I30" s="13">
         <v>0</v>
       </c>
-      <c r="J30" s="20">
-        <v>3.5805315498782759E-5</v>
+      <c r="J30" s="22">
+        <v>7.8180055576928815E-5</v>
       </c>
       <c r="K30" s="14">
         <v>0</v>
       </c>
       <c r="L30" s="14">
-        <v>4692040.7671232875</v>
+        <v>2148885.6558139534</v>
       </c>
       <c r="M30" s="13"/>
       <c r="N30" s="13"/>
@@ -3456,10 +3349,10 @@
       <c r="Q30" s="12">
         <v>0</v>
       </c>
-      <c r="R30" s="20">
+      <c r="R30" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S30" s="22">
+      <c r="S30" s="24">
         <v>0</v>
       </c>
       <c r="T30" s="12">
@@ -3474,43 +3367,39 @@
       <c r="W30" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X30" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y30" s="15"/>
+      <c r="X30" s="15"/>
+      <c r="Y30" s="12"/>
       <c r="Z30" s="12"/>
-      <c r="AA30" s="12"/>
+      <c r="AA30" s="16">
+        <v>47.250870140000004</v>
+      </c>
       <c r="AB30" s="16">
-        <v>47.250870140000004</v>
-      </c>
-      <c r="AC30" s="16">
         <v>15.310090219999999</v>
       </c>
+      <c r="AC30" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD30" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE30" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="31" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
       <c r="B31" s="19"/>
       <c r="C31" s="18" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F31" s="12">
         <v>1</v>
       </c>
-      <c r="G31" s="20">
-        <v>1755.4676166872623</v>
+      <c r="G31" s="22">
+        <v>2312.5519195166125</v>
       </c>
       <c r="H31" s="13">
         <v>0</v>
@@ -3518,14 +3407,14 @@
       <c r="I31" s="13">
         <v>0</v>
       </c>
-      <c r="J31" s="20">
-        <v>5.6964878787516286E-4</v>
+      <c r="J31" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K31" s="14">
         <v>0</v>
       </c>
       <c r="L31" s="14">
-        <v>21065.611400247148</v>
+        <v>27750.623034199351</v>
       </c>
       <c r="M31" s="13"/>
       <c r="N31" s="13"/>
@@ -3538,10 +3427,10 @@
       <c r="Q31" s="12">
         <v>0</v>
       </c>
-      <c r="R31" s="20">
+      <c r="R31" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S31" s="22">
+      <c r="S31" s="24">
         <v>0</v>
       </c>
       <c r="T31" s="12">
@@ -3556,43 +3445,39 @@
       <c r="W31" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X31" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y31" s="15"/>
+      <c r="X31" s="15"/>
+      <c r="Y31" s="12"/>
       <c r="Z31" s="12"/>
-      <c r="AA31" s="12"/>
+      <c r="AA31" s="16">
+        <v>46.74433801</v>
+      </c>
       <c r="AB31" s="16">
-        <v>46.74433801</v>
-      </c>
-      <c r="AC31" s="16">
         <v>15.57045501</v>
       </c>
+      <c r="AC31" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD31" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE31" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="32" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="10"/>
       <c r="B32" s="19"/>
       <c r="C32" s="18" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F32" s="12">
         <v>1</v>
       </c>
-      <c r="G32" s="20">
-        <v>558256.28219178075</v>
+      <c r="G32" s="22">
+        <v>204734.74925373134</v>
       </c>
       <c r="H32" s="13">
         <v>0</v>
@@ -3600,14 +3485,14 @@
       <c r="I32" s="13">
         <v>0</v>
       </c>
-      <c r="J32" s="20">
-        <v>2.3286795714972428E-5</v>
+      <c r="J32" s="22">
+        <v>6.3496793032866511E-5</v>
       </c>
       <c r="K32" s="14">
         <v>0</v>
       </c>
       <c r="L32" s="14">
-        <v>6699075.3863013685</v>
+        <v>2456816.991044776</v>
       </c>
       <c r="M32" s="13"/>
       <c r="N32" s="13"/>
@@ -3620,10 +3505,10 @@
       <c r="Q32" s="12">
         <v>0</v>
       </c>
-      <c r="R32" s="20">
+      <c r="R32" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S32" s="22">
+      <c r="S32" s="24">
         <v>0</v>
       </c>
       <c r="T32" s="12">
@@ -3638,45 +3523,41 @@
       <c r="W32" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X32" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y32" s="15"/>
-      <c r="Z32" s="12">
+      <c r="X32" s="15"/>
+      <c r="Y32" s="12">
         <v>1982</v>
       </c>
-      <c r="AA32" s="12"/>
+      <c r="Z32" s="12"/>
+      <c r="AA32" s="16">
+        <v>46.716855860000003</v>
+      </c>
       <c r="AB32" s="16">
-        <v>46.716855860000003</v>
-      </c>
-      <c r="AC32" s="16">
         <v>15.621529779999999</v>
       </c>
+      <c r="AC32" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD32" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE32" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="33" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="10"/>
       <c r="B33" s="19"/>
       <c r="C33" s="18" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F33" s="12">
         <v>1</v>
       </c>
-      <c r="G33" s="20">
-        <v>90723.599999999991</v>
+      <c r="G33" s="22">
+        <v>37022.94</v>
       </c>
       <c r="H33" s="13">
         <v>0</v>
@@ -3684,14 +3565,14 @@
       <c r="I33" s="13">
         <v>0</v>
       </c>
-      <c r="J33" s="20">
-        <v>6.6134941735116335E-5</v>
+      <c r="J33" s="22">
+        <v>1.6206168391813292E-4</v>
       </c>
       <c r="K33" s="14">
         <v>0</v>
       </c>
       <c r="L33" s="14">
-        <v>1088683.2</v>
+        <v>444275.28</v>
       </c>
       <c r="M33" s="13"/>
       <c r="N33" s="13"/>
@@ -3704,10 +3585,10 @@
       <c r="Q33" s="12">
         <v>0</v>
       </c>
-      <c r="R33" s="20">
+      <c r="R33" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S33" s="22">
+      <c r="S33" s="24">
         <v>0</v>
       </c>
       <c r="T33" s="12">
@@ -3722,45 +3603,41 @@
       <c r="W33" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X33" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y33" s="15"/>
-      <c r="Z33" s="12">
+      <c r="X33" s="15"/>
+      <c r="Y33" s="12">
         <v>1985</v>
       </c>
-      <c r="AA33" s="12"/>
+      <c r="Z33" s="12"/>
+      <c r="AA33" s="16">
+        <v>47.104410209999998</v>
+      </c>
       <c r="AB33" s="16">
-        <v>47.104410209999998</v>
-      </c>
-      <c r="AC33" s="16">
         <v>14.08673125</v>
       </c>
+      <c r="AC33" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD33" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE33" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="34" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="10"/>
       <c r="B34" s="19"/>
       <c r="C34" s="18" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F34" s="12">
         <v>1</v>
       </c>
-      <c r="G34" s="20">
-        <v>26170.257945205503</v>
+      <c r="G34" s="22">
+        <v>37000.830712265801</v>
       </c>
       <c r="H34" s="13">
         <v>0</v>
@@ -3768,14 +3645,14 @@
       <c r="I34" s="13">
         <v>0</v>
       </c>
-      <c r="J34" s="20">
-        <v>6.1138105835641045E-4</v>
+      <c r="J34" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K34" s="14">
         <v>0</v>
       </c>
       <c r="L34" s="14">
-        <v>314043.09534246603</v>
+        <v>444009.96854718961</v>
       </c>
       <c r="M34" s="13"/>
       <c r="N34" s="13"/>
@@ -3788,10 +3665,10 @@
       <c r="Q34" s="12">
         <v>0</v>
       </c>
-      <c r="R34" s="20">
+      <c r="R34" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S34" s="22">
+      <c r="S34" s="24">
         <v>0</v>
       </c>
       <c r="T34" s="12">
@@ -3806,43 +3683,39 @@
       <c r="W34" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X34" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y34" s="15"/>
+      <c r="X34" s="15"/>
+      <c r="Y34" s="12"/>
       <c r="Z34" s="12"/>
-      <c r="AA34" s="12"/>
+      <c r="AA34" s="16">
+        <v>46.987347919999998</v>
+      </c>
       <c r="AB34" s="16">
-        <v>46.987347919999998</v>
-      </c>
-      <c r="AC34" s="16">
         <v>15.091276199999999</v>
       </c>
+      <c r="AC34" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD34" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE34" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="35" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="10"/>
       <c r="B35" s="19"/>
       <c r="C35" s="18" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F35" s="12">
         <v>1</v>
       </c>
-      <c r="G35" s="20">
-        <v>21065.611400247148</v>
+      <c r="G35" s="22">
+        <v>27750.623034199351</v>
       </c>
       <c r="H35" s="13">
         <v>0</v>
@@ -3850,14 +3723,14 @@
       <c r="I35" s="13">
         <v>0</v>
       </c>
-      <c r="J35" s="20">
-        <v>5.6964878787516286E-4</v>
+      <c r="J35" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K35" s="14">
         <v>0</v>
       </c>
       <c r="L35" s="14">
-        <v>252787.33680296579</v>
+        <v>333007.47641039221</v>
       </c>
       <c r="M35" s="13"/>
       <c r="N35" s="13"/>
@@ -3870,10 +3743,10 @@
       <c r="Q35" s="12">
         <v>0</v>
       </c>
-      <c r="R35" s="20">
+      <c r="R35" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S35" s="22">
+      <c r="S35" s="24">
         <v>0</v>
       </c>
       <c r="T35" s="12">
@@ -3888,43 +3761,39 @@
       <c r="W35" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X35" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y35" s="15"/>
+      <c r="X35" s="15"/>
+      <c r="Y35" s="12"/>
       <c r="Z35" s="12"/>
-      <c r="AA35" s="12"/>
+      <c r="AA35" s="16">
+        <v>47.175225009999998</v>
+      </c>
       <c r="AB35" s="16">
-        <v>47.175225009999998</v>
-      </c>
-      <c r="AC35" s="16">
         <v>15.320385010000001</v>
       </c>
+      <c r="AC35" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD35" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE35" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="36" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="10"/>
       <c r="B36" s="19"/>
       <c r="C36" s="18" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F36" s="12">
         <v>1</v>
       </c>
-      <c r="G36" s="20">
-        <v>26170.257945205503</v>
+      <c r="G36" s="22">
+        <v>2312.5519195166125</v>
       </c>
       <c r="H36" s="13">
         <v>0</v>
@@ -3932,14 +3801,14 @@
       <c r="I36" s="13">
         <v>0</v>
       </c>
-      <c r="J36" s="20">
-        <v>3.8211316147275653E-5</v>
+      <c r="J36" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K36" s="14">
         <v>0</v>
       </c>
       <c r="L36" s="14">
-        <v>314043.09534246603</v>
+        <v>27750.623034199351</v>
       </c>
       <c r="M36" s="13"/>
       <c r="N36" s="13"/>
@@ -3952,10 +3821,10 @@
       <c r="Q36" s="12">
         <v>0</v>
       </c>
-      <c r="R36" s="20">
+      <c r="R36" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S36" s="22">
+      <c r="S36" s="24">
         <v>0</v>
       </c>
       <c r="T36" s="12">
@@ -3970,43 +3839,39 @@
       <c r="W36" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X36" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y36" s="15"/>
+      <c r="X36" s="15"/>
+      <c r="Y36" s="12"/>
       <c r="Z36" s="12"/>
-      <c r="AA36" s="12"/>
+      <c r="AA36" s="16">
+        <v>47.02151301</v>
+      </c>
       <c r="AB36" s="16">
-        <v>47.02151301</v>
-      </c>
-      <c r="AC36" s="16">
         <v>15.166537010000001</v>
       </c>
+      <c r="AC36" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD36" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE36" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="37" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="10"/>
       <c r="B37" s="19"/>
       <c r="C37" s="18" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F37" s="12">
         <v>1</v>
       </c>
-      <c r="G37" s="20">
-        <v>1755.4676166872623</v>
+      <c r="G37" s="22">
+        <v>2312.5519195166125</v>
       </c>
       <c r="H37" s="13">
         <v>0</v>
@@ -4014,14 +3879,14 @@
       <c r="I37" s="13">
         <v>0</v>
       </c>
-      <c r="J37" s="20">
-        <v>5.6964878787516286E-4</v>
+      <c r="J37" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K37" s="14">
         <v>0</v>
       </c>
       <c r="L37" s="14">
-        <v>21065.611400247148</v>
+        <v>27750.623034199351</v>
       </c>
       <c r="M37" s="13"/>
       <c r="N37" s="13"/>
@@ -4034,10 +3899,10 @@
       <c r="Q37" s="12">
         <v>0</v>
       </c>
-      <c r="R37" s="20">
+      <c r="R37" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S37" s="22">
+      <c r="S37" s="24">
         <v>0</v>
       </c>
       <c r="T37" s="12">
@@ -4052,43 +3917,39 @@
       <c r="W37" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X37" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y37" s="15"/>
+      <c r="X37" s="15"/>
+      <c r="Y37" s="12"/>
       <c r="Z37" s="12"/>
-      <c r="AA37" s="12"/>
+      <c r="AA37" s="16">
+        <v>47.495437010000003</v>
+      </c>
       <c r="AB37" s="16">
-        <v>47.495437010000003</v>
-      </c>
-      <c r="AC37" s="16">
         <v>14.99248</v>
       </c>
+      <c r="AC37" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD37" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE37" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="38" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="10"/>
       <c r="B38" s="19"/>
       <c r="C38" s="18" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F38" s="12">
         <v>1</v>
       </c>
-      <c r="G38" s="20">
-        <v>29842.94948368346</v>
+      <c r="G38" s="22">
+        <v>39313.382631782413</v>
       </c>
       <c r="H38" s="13">
         <v>0</v>
@@ -4096,14 +3957,14 @@
       <c r="I38" s="13">
         <v>0</v>
       </c>
-      <c r="J38" s="20">
-        <v>5.6964878787516286E-4</v>
+      <c r="J38" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K38" s="14">
         <v>0</v>
       </c>
       <c r="L38" s="14">
-        <v>358115.39380420151</v>
+        <v>471760.59158138896</v>
       </c>
       <c r="M38" s="13"/>
       <c r="N38" s="13"/>
@@ -4116,10 +3977,10 @@
       <c r="Q38" s="12">
         <v>0</v>
       </c>
-      <c r="R38" s="20">
+      <c r="R38" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S38" s="22">
+      <c r="S38" s="24">
         <v>0</v>
       </c>
       <c r="T38" s="12">
@@ -4134,45 +3995,41 @@
       <c r="W38" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X38" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y38" s="15"/>
-      <c r="Z38" s="12">
+      <c r="X38" s="15"/>
+      <c r="Y38" s="12">
         <v>1982</v>
       </c>
-      <c r="AA38" s="12"/>
+      <c r="Z38" s="12"/>
+      <c r="AA38" s="16">
+        <v>47.10900101</v>
+      </c>
       <c r="AB38" s="16">
-        <v>47.10900101</v>
-      </c>
-      <c r="AC38" s="16">
         <v>15.39200001</v>
       </c>
+      <c r="AC38" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD38" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE38" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="39" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="10"/>
       <c r="B39" s="19"/>
       <c r="C39" s="18" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F39" s="12">
         <v>1</v>
       </c>
-      <c r="G39" s="20">
-        <v>1755.4676166872623</v>
+      <c r="G39" s="22">
+        <v>2312.5519195166125</v>
       </c>
       <c r="H39" s="13">
         <v>0</v>
@@ -4180,14 +4037,14 @@
       <c r="I39" s="13">
         <v>0</v>
       </c>
-      <c r="J39" s="20">
-        <v>5.6964878787516286E-4</v>
+      <c r="J39" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K39" s="14">
         <v>0</v>
       </c>
       <c r="L39" s="14">
-        <v>21065.611400247148</v>
+        <v>27750.623034199351</v>
       </c>
       <c r="M39" s="13"/>
       <c r="N39" s="13"/>
@@ -4200,10 +4057,10 @@
       <c r="Q39" s="12">
         <v>0</v>
       </c>
-      <c r="R39" s="20">
+      <c r="R39" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S39" s="22">
+      <c r="S39" s="24">
         <v>0</v>
       </c>
       <c r="T39" s="12">
@@ -4218,43 +4075,39 @@
       <c r="W39" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X39" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y39" s="15"/>
+      <c r="X39" s="15"/>
+      <c r="Y39" s="12"/>
       <c r="Z39" s="12"/>
-      <c r="AA39" s="12"/>
+      <c r="AA39" s="16">
+        <v>46.912548010000002</v>
+      </c>
       <c r="AB39" s="16">
-        <v>46.912548010000002</v>
-      </c>
-      <c r="AC39" s="16">
         <v>15.48666401</v>
       </c>
+      <c r="AC39" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD39" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE39" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="40" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="10"/>
       <c r="B40" s="19"/>
       <c r="C40" s="18" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F40" s="12">
         <v>1</v>
       </c>
-      <c r="G40" s="20">
-        <v>8601.791321767585</v>
+      <c r="G40" s="22">
+        <v>11331.504405631402</v>
       </c>
       <c r="H40" s="13">
         <v>0</v>
@@ -4262,14 +4115,14 @@
       <c r="I40" s="13">
         <v>0</v>
       </c>
-      <c r="J40" s="20">
-        <v>5.6964878787516286E-4</v>
+      <c r="J40" s="22">
+        <v>4.3242272381457611E-4</v>
       </c>
       <c r="K40" s="14">
         <v>0</v>
       </c>
       <c r="L40" s="14">
-        <v>103221.49586121102</v>
+        <v>135978.05286757683</v>
       </c>
       <c r="M40" s="13"/>
       <c r="N40" s="13"/>
@@ -4282,10 +4135,10 @@
       <c r="Q40" s="12">
         <v>0</v>
       </c>
-      <c r="R40" s="20">
+      <c r="R40" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S40" s="22">
+      <c r="S40" s="24">
         <v>0</v>
       </c>
       <c r="T40" s="12">
@@ -4300,45 +4153,41 @@
       <c r="W40" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X40" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y40" s="15"/>
-      <c r="Z40" s="12">
+      <c r="X40" s="15"/>
+      <c r="Y40" s="12">
         <v>1988</v>
       </c>
-      <c r="AA40" s="12"/>
+      <c r="Z40" s="12"/>
+      <c r="AA40" s="16">
+        <v>47.20008473</v>
+      </c>
       <c r="AB40" s="16">
-        <v>47.20008473</v>
-      </c>
-      <c r="AC40" s="16">
         <v>14.442535319999999</v>
       </c>
+      <c r="AC40" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD40" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE40" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="41" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="10"/>
       <c r="B41" s="19"/>
       <c r="C41" s="18" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F41" s="12">
         <v>1</v>
       </c>
-      <c r="G41" s="20">
-        <v>14914.142876712329</v>
+      <c r="G41" s="22">
+        <v>9898.1018181818181</v>
       </c>
       <c r="H41" s="13">
         <v>0</v>
@@ -4346,14 +4195,14 @@
       <c r="I41" s="13">
         <v>0</v>
       </c>
-      <c r="J41" s="20">
-        <v>6.7050450586835192E-4</v>
+      <c r="J41" s="22">
+        <v>1.010294719501774E-3</v>
       </c>
       <c r="K41" s="14">
         <v>0</v>
       </c>
       <c r="L41" s="14">
-        <v>178969.71452054795</v>
+        <v>118777.22181818182</v>
       </c>
       <c r="M41" s="13"/>
       <c r="N41" s="13"/>
@@ -4366,10 +4215,10 @@
       <c r="Q41" s="12">
         <v>0</v>
       </c>
-      <c r="R41" s="20">
+      <c r="R41" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S41" s="22">
+      <c r="S41" s="24">
         <v>0</v>
       </c>
       <c r="T41" s="12">
@@ -4384,45 +4233,41 @@
       <c r="W41" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X41" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="Y41" s="15"/>
-      <c r="Z41" s="12">
+      <c r="X41" s="15"/>
+      <c r="Y41" s="12">
         <v>1984</v>
       </c>
-      <c r="AA41" s="12"/>
+      <c r="Z41" s="12"/>
+      <c r="AA41" s="16">
+        <v>47.164754000000002</v>
+      </c>
       <c r="AB41" s="16">
-        <v>47.164754000000002</v>
-      </c>
-      <c r="AC41" s="16">
         <v>13.47057096</v>
       </c>
+      <c r="AC41" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD41" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE41" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="42" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="10"/>
       <c r="B42" s="19"/>
       <c r="C42" s="18" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F42" s="12">
         <v>1</v>
       </c>
-      <c r="G42" s="20">
-        <v>26170.2579452055</v>
+      <c r="G42" s="22">
+        <v>355388.97599999997</v>
       </c>
       <c r="H42" s="13">
         <v>0</v>
@@ -4430,14 +4275,14 @@
       <c r="I42" s="13">
         <v>0</v>
       </c>
-      <c r="J42" s="20">
-        <v>1.1463394844182697E-3</v>
+      <c r="J42" s="22">
+        <v>8.4414548638109697E-5</v>
       </c>
       <c r="K42" s="14">
         <v>0</v>
       </c>
       <c r="L42" s="14">
-        <v>314043.09534246603</v>
+        <v>4264667.7119999994</v>
       </c>
       <c r="M42" s="13"/>
       <c r="N42" s="13"/>
@@ -4450,10 +4295,10 @@
       <c r="Q42" s="12">
         <v>0</v>
       </c>
-      <c r="R42" s="20">
+      <c r="R42" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S42" s="22">
+      <c r="S42" s="24">
         <v>0</v>
       </c>
       <c r="T42" s="12">
@@ -4468,45 +4313,41 @@
       <c r="W42" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X42" s="13">
-        <f t="shared" si="0"/>
-        <v>12.000000000000002</v>
-      </c>
-      <c r="Y42" s="15"/>
-      <c r="Z42" s="12">
+      <c r="X42" s="15"/>
+      <c r="Y42" s="12">
         <v>1925</v>
       </c>
-      <c r="AA42" s="12"/>
+      <c r="Z42" s="12"/>
+      <c r="AA42" s="16">
+        <v>47.018382189999997</v>
+      </c>
       <c r="AB42" s="16">
-        <v>47.018382189999997</v>
-      </c>
-      <c r="AC42" s="16">
         <v>15.15986506</v>
       </c>
+      <c r="AC42" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD42" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE42" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
-    <row r="43" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="10"/>
       <c r="B43" s="19"/>
       <c r="C43" s="18" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F43" s="12">
         <v>1</v>
       </c>
-      <c r="G43" s="20">
-        <v>388412.26027397264</v>
+      <c r="G43" s="22">
+        <v>180286.82497297297</v>
       </c>
       <c r="H43" s="13">
         <v>0</v>
@@ -4514,14 +4355,14 @@
       <c r="I43" s="13">
         <v>0</v>
       </c>
-      <c r="J43" s="20">
-        <v>4.37679284068139E-5</v>
+      <c r="J43" s="22">
+        <v>9.4294189287256525E-5</v>
       </c>
       <c r="K43" s="14">
         <v>0</v>
       </c>
       <c r="L43" s="14">
-        <v>4660947.1232876722</v>
+        <v>2163441.8996756757</v>
       </c>
       <c r="M43" s="13"/>
       <c r="N43" s="13"/>
@@ -4534,10 +4375,10 @@
       <c r="Q43" s="12">
         <v>0</v>
       </c>
-      <c r="R43" s="20">
+      <c r="R43" s="22">
         <v>4.6657547496963339E-4</v>
       </c>
-      <c r="S43" s="22">
+      <c r="S43" s="24">
         <v>0</v>
       </c>
       <c r="T43" s="12">
@@ -4552,26 +4393,22 @@
       <c r="W43" s="14">
         <v>99999999999</v>
       </c>
-      <c r="X43" s="13">
-        <f t="shared" si="0"/>
-        <v>12.000000000000002</v>
-      </c>
-      <c r="Y43" s="15"/>
-      <c r="Z43" s="12">
+      <c r="X43" s="15"/>
+      <c r="Y43" s="12">
         <v>1985</v>
       </c>
-      <c r="AA43" s="12"/>
+      <c r="Z43" s="12"/>
+      <c r="AA43" s="16">
+        <v>46.910999009999998</v>
+      </c>
       <c r="AB43" s="16">
-        <v>46.910999009999998</v>
-      </c>
-      <c r="AC43" s="16">
         <v>15.48600001</v>
       </c>
+      <c r="AC43" s="17" t="s">
+        <v>132</v>
+      </c>
       <c r="AD43" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE43" s="17" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Hydro Assets file
Maxprod, power factor, OMvar Costs
</commit_message>
<xml_diff>
--- a/data/hydroExample/Power_HydroAssets.xlsx
+++ b/data/hydroExample/Power_HydroAssets.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\hydroExample\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth\Documents\LEGO_Pyomo\LEGO-Pyomo\data\hydroExample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1938B92-3968-43BD-A84B-1C59D8C104BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85A4F1E3-7A0C-4455-A57B-9E7D11794327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34230" yWindow="-21705" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario_2016" sheetId="1" r:id="rId1"/>
@@ -741,7 +741,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1045,7 +1045,7 @@
     <tabColor rgb="FF008080"/>
   </sheetPr>
   <dimension ref="A1:AD43"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" customWidth="1"/>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
@@ -1577,7 +1577,7 @@
         <v>1</v>
       </c>
       <c r="G8" s="22">
-        <v>18795.432911392403</v>
+        <v>54909.846575342461</v>
       </c>
       <c r="H8" s="13">
         <v>0</v>
@@ -1586,13 +1586,13 @@
         <v>0</v>
       </c>
       <c r="J8" s="22">
-        <v>1.3833147724009441E-3</v>
+        <v>4.7350341735748772E-4</v>
       </c>
       <c r="K8" s="14">
         <v>0</v>
       </c>
       <c r="L8" s="14">
-        <v>225545.19493670884</v>
+        <v>658918.1589041095</v>
       </c>
       <c r="M8" s="13"/>
       <c r="N8" s="13"/>
@@ -1606,7 +1606,7 @@
         <v>0</v>
       </c>
       <c r="R8" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S8" s="24">
         <v>0</v>
@@ -1657,7 +1657,7 @@
         <v>1</v>
       </c>
       <c r="G9" s="22">
-        <v>76314.213344048214</v>
+        <v>26170.257945205503</v>
       </c>
       <c r="H9" s="13">
         <v>0</v>
@@ -1666,13 +1666,13 @@
         <v>0</v>
       </c>
       <c r="J9" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>1.2609734328600966E-3</v>
       </c>
       <c r="K9" s="14">
         <v>0</v>
       </c>
       <c r="L9" s="14">
-        <v>915770.56012857857</v>
+        <v>314043.09534246603</v>
       </c>
       <c r="M9" s="13"/>
       <c r="N9" s="13"/>
@@ -1686,7 +1686,7 @@
         <v>0</v>
       </c>
       <c r="R9" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S9" s="24">
         <v>0</v>
@@ -1735,7 +1735,7 @@
         <v>1</v>
       </c>
       <c r="G10" s="22">
-        <v>197455.68000000002</v>
+        <v>90723.6</v>
       </c>
       <c r="H10" s="13">
         <v>0</v>
@@ -1744,13 +1744,13 @@
         <v>123.1396524</v>
       </c>
       <c r="J10" s="22">
-        <v>1.7219053916301622E-4</v>
+        <v>3.7476466983232587E-4</v>
       </c>
       <c r="K10" s="20">
         <v>1.6999999999999999E-3</v>
       </c>
       <c r="L10" s="14">
-        <v>2369468.16</v>
+        <v>1088683.2000000002</v>
       </c>
       <c r="M10" s="13"/>
       <c r="N10" s="13"/>
@@ -1764,10 +1764,10 @@
         <v>0</v>
       </c>
       <c r="R10" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S10" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="T10" s="12">
         <v>0</v>
@@ -1815,7 +1815,7 @@
         <v>1</v>
       </c>
       <c r="G11" s="22">
-        <v>117304.04284051221</v>
+        <v>303080.53109589039</v>
       </c>
       <c r="H11" s="13">
         <v>0</v>
@@ -1824,13 +1824,13 @@
         <v>0</v>
       </c>
       <c r="J11" s="22">
-        <v>1.3639768598388177E-4</v>
+        <v>5.2791249712235146E-5</v>
       </c>
       <c r="K11" s="14">
         <v>0</v>
       </c>
       <c r="L11" s="14">
-        <v>1407648.5140861464</v>
+        <v>3636966.3731506849</v>
       </c>
       <c r="M11" s="13"/>
       <c r="N11" s="13"/>
@@ -1844,7 +1844,7 @@
         <v>0</v>
       </c>
       <c r="R11" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S11" s="24">
         <v>0</v>
@@ -1895,7 +1895,7 @@
         <v>1</v>
       </c>
       <c r="G12" s="22">
-        <v>50876.142229365476</v>
+        <v>38620.287567119769</v>
       </c>
       <c r="H12" s="13">
         <v>0</v>
@@ -1904,13 +1904,13 @@
         <v>0</v>
       </c>
       <c r="J12" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K12" s="14">
         <v>0</v>
       </c>
       <c r="L12" s="14">
-        <v>610513.70675238571</v>
+        <v>463443.45080543723</v>
       </c>
       <c r="M12" s="13"/>
       <c r="N12" s="13"/>
@@ -1924,7 +1924,7 @@
         <v>0</v>
       </c>
       <c r="R12" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S12" s="24">
         <v>0</v>
@@ -1975,7 +1975,7 @@
         <v>1</v>
       </c>
       <c r="G13" s="22">
-        <v>128145.67200000001</v>
+        <v>308190.13232876715</v>
       </c>
       <c r="H13" s="13">
         <v>0</v>
@@ -1984,13 +1984,13 @@
         <v>0</v>
       </c>
       <c r="J13" s="22">
-        <v>9.3643427926305622E-5</v>
+        <v>3.8937002652631305E-5</v>
       </c>
       <c r="K13" s="14">
         <v>0</v>
       </c>
       <c r="L13" s="14">
-        <v>1537748.064</v>
+        <v>3698281.5879452061</v>
       </c>
       <c r="M13" s="13"/>
       <c r="N13" s="13"/>
@@ -2004,7 +2004,7 @@
         <v>0</v>
       </c>
       <c r="R13" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S13" s="24">
         <v>0</v>
@@ -2055,7 +2055,7 @@
         <v>1</v>
       </c>
       <c r="G14" s="22">
-        <v>192549.84</v>
+        <v>467759.68356164393</v>
       </c>
       <c r="H14" s="13">
         <v>0</v>
@@ -2064,13 +2064,13 @@
         <v>0</v>
       </c>
       <c r="J14" s="22">
-        <v>7.2708447849138697E-5</v>
+        <v>2.9929898817701346E-5</v>
       </c>
       <c r="K14" s="14">
         <v>0</v>
       </c>
       <c r="L14" s="14">
-        <v>2310598.08</v>
+        <v>5613116.2027397268</v>
       </c>
       <c r="M14" s="13"/>
       <c r="N14" s="13"/>
@@ -2084,7 +2084,7 @@
         <v>0</v>
       </c>
       <c r="R14" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S14" s="24">
         <v>0</v>
@@ -2135,7 +2135,7 @@
         <v>1</v>
       </c>
       <c r="G15" s="22">
-        <v>168293.23855530474</v>
+        <v>729653.91196388274</v>
       </c>
       <c r="H15" s="13">
         <v>0</v>
@@ -2144,13 +2144,13 @@
         <v>0</v>
       </c>
       <c r="J15" s="22">
-        <v>1.12898177984472E-4</v>
+        <v>2.6039742525139078E-5</v>
       </c>
       <c r="K15" s="14">
         <v>0</v>
       </c>
       <c r="L15" s="14">
-        <v>2019518.8626636569</v>
+        <v>8755846.9435665924</v>
       </c>
       <c r="M15" s="13"/>
       <c r="N15" s="13"/>
@@ -2164,7 +2164,7 @@
         <v>0</v>
       </c>
       <c r="R15" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S15" s="24">
         <v>0</v>
@@ -2215,7 +2215,7 @@
         <v>1</v>
       </c>
       <c r="G16" s="22">
-        <v>735583.65842696629</v>
+        <v>467759.68356164393</v>
       </c>
       <c r="H16" s="13">
         <v>0</v>
@@ -2224,13 +2224,13 @@
         <v>0</v>
       </c>
       <c r="J16" s="22">
-        <v>1.9032505466392189E-5</v>
+        <v>2.9929898817701346E-5</v>
       </c>
       <c r="K16" s="14">
         <v>0</v>
       </c>
       <c r="L16" s="14">
-        <v>8827003.9011235945</v>
+        <v>5613116.2027397268</v>
       </c>
       <c r="M16" s="13"/>
       <c r="N16" s="13"/>
@@ -2244,7 +2244,7 @@
         <v>0</v>
       </c>
       <c r="R16" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S16" s="24">
         <v>0</v>
@@ -2295,7 +2295,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="22">
-        <v>184888.02933333334</v>
+        <v>413303.9589041096</v>
       </c>
       <c r="H17" s="13">
         <v>0</v>
@@ -2304,13 +2304,13 @@
         <v>0</v>
       </c>
       <c r="J17" s="22">
-        <v>5.9495468904415532E-5</v>
+        <v>2.6614794663876189E-5</v>
       </c>
       <c r="K17" s="14">
         <v>0</v>
       </c>
       <c r="L17" s="14">
-        <v>2218656.352</v>
+        <v>4959647.506849315</v>
       </c>
       <c r="M17" s="13"/>
       <c r="N17" s="13"/>
@@ -2324,7 +2324,7 @@
         <v>0</v>
       </c>
       <c r="R17" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S17" s="24">
         <v>0</v>
@@ -2375,7 +2375,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="22">
-        <v>169397.1903512195</v>
+        <v>388412.26027397258</v>
       </c>
       <c r="H18" s="13">
         <v>0</v>
@@ -2384,13 +2384,13 @@
         <v>0</v>
       </c>
       <c r="J18" s="22">
-        <v>1.0448815569668966E-4</v>
+        <v>4.5570137223565063E-5</v>
       </c>
       <c r="K18" s="14">
         <v>0</v>
       </c>
       <c r="L18" s="14">
-        <v>2032766.284214634</v>
+        <v>4660947.1232876712</v>
       </c>
       <c r="M18" s="13"/>
       <c r="N18" s="13"/>
@@ -2404,7 +2404,7 @@
         <v>0</v>
       </c>
       <c r="R18" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S18" s="24">
         <v>0</v>
@@ -2453,7 +2453,7 @@
         <v>1</v>
       </c>
       <c r="G19" s="22">
-        <v>13875.311517099675</v>
+        <v>26170.2579452055</v>
       </c>
       <c r="H19" s="13">
         <v>0</v>
@@ -2462,13 +2462,13 @@
         <v>0</v>
       </c>
       <c r="J19" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>2.2926789688365392E-4</v>
       </c>
       <c r="K19" s="14">
         <v>0</v>
       </c>
       <c r="L19" s="14">
-        <v>166503.7382051961</v>
+        <v>314043.09534246603</v>
       </c>
       <c r="M19" s="13"/>
       <c r="N19" s="13"/>
@@ -2482,7 +2482,7 @@
         <v>0</v>
       </c>
       <c r="R19" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S19" s="24">
         <v>0</v>
@@ -2531,7 +2531,7 @@
         <v>1</v>
       </c>
       <c r="G20" s="22">
-        <v>21107.257600000001</v>
+        <v>11095.429726027354</v>
       </c>
       <c r="H20" s="13">
         <v>0</v>
@@ -2540,13 +2540,13 @@
         <v>0</v>
       </c>
       <c r="J20" s="22">
-        <v>4.9272151773994549E-3</v>
+        <v>9.3732286687409367E-3</v>
       </c>
       <c r="K20" s="14">
         <v>0</v>
       </c>
       <c r="L20" s="14">
-        <v>15000000</v>
+        <v>1500000</v>
       </c>
       <c r="M20" s="13"/>
       <c r="N20" s="13"/>
@@ -2560,7 +2560,7 @@
         <v>1</v>
       </c>
       <c r="R20" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S20" s="24">
         <v>0</v>
@@ -2609,7 +2609,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="22">
-        <v>183607.69530845954</v>
+        <v>388412.26027397258</v>
       </c>
       <c r="H21" s="13">
         <v>0</v>
@@ -2618,13 +2618,13 @@
         <v>0</v>
       </c>
       <c r="J21" s="22">
-        <v>1.0348150151375814E-4</v>
+        <v>4.8917096454674359E-5</v>
       </c>
       <c r="K21" s="14">
         <v>0</v>
       </c>
       <c r="L21" s="14">
-        <v>2203292.3437015144</v>
+        <v>4660947.1232876712</v>
       </c>
       <c r="M21" s="13"/>
       <c r="N21" s="13"/>
@@ -2638,7 +2638,7 @@
         <v>0</v>
       </c>
       <c r="R21" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S21" s="24">
         <v>0</v>
@@ -2689,7 +2689,7 @@
         <v>1</v>
       </c>
       <c r="G22" s="22">
-        <v>122730.03966942149</v>
+        <v>391003.39726027398</v>
       </c>
       <c r="H22" s="13">
         <v>0</v>
@@ -2698,13 +2698,13 @@
         <v>0</v>
       </c>
       <c r="J22" s="22">
-        <v>1.4666336007454863E-4</v>
+        <v>4.6035405641292117E-5</v>
       </c>
       <c r="K22" s="14">
         <v>0</v>
       </c>
       <c r="L22" s="14">
-        <v>1472760.4760330578</v>
+        <v>4692040.7671232875</v>
       </c>
       <c r="M22" s="13"/>
       <c r="N22" s="13"/>
@@ -2718,7 +2718,7 @@
         <v>0</v>
       </c>
       <c r="R22" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S22" s="24">
         <v>0</v>
@@ -2769,7 +2769,7 @@
         <v>1</v>
       </c>
       <c r="G23" s="22">
-        <v>111471.04648390942</v>
+        <v>467759.68356164382</v>
       </c>
       <c r="H23" s="13">
         <v>0</v>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="J23" s="22">
-        <v>8.9709393743275537E-5</v>
+        <v>2.1378499155500961E-5</v>
       </c>
       <c r="K23" s="14">
         <v>0</v>
       </c>
       <c r="L23" s="14">
-        <v>1337652.557806913</v>
+        <v>5613116.2027397258</v>
       </c>
       <c r="M23" s="13"/>
       <c r="N23" s="13"/>
@@ -2798,7 +2798,7 @@
         <v>0</v>
       </c>
       <c r="R23" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S23" s="24">
         <v>0</v>
@@ -2849,7 +2849,7 @@
         <v>1</v>
       </c>
       <c r="G24" s="22">
-        <v>146262.2694969576</v>
+        <v>303080.53109589039</v>
       </c>
       <c r="H24" s="13">
         <v>0</v>
@@ -2858,13 +2858,13 @@
         <v>0</v>
       </c>
       <c r="J24" s="22">
-        <v>6.8370332515645875E-5</v>
+        <v>3.2994531070146968E-5</v>
       </c>
       <c r="K24" s="14">
         <v>0</v>
       </c>
       <c r="L24" s="14">
-        <v>1755147.2339634912</v>
+        <v>3636966.3731506849</v>
       </c>
       <c r="M24" s="13"/>
       <c r="N24" s="13"/>
@@ -2878,7 +2878,7 @@
         <v>0</v>
       </c>
       <c r="R24" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S24" s="24">
         <v>0</v>
@@ -2927,7 +2927,7 @@
         <v>1</v>
       </c>
       <c r="G25" s="22">
-        <v>30063.174953715963</v>
+        <v>467759.68356164382</v>
       </c>
       <c r="H25" s="13">
         <v>0</v>
@@ -2936,13 +2936,13 @@
         <v>0</v>
       </c>
       <c r="J25" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>2.779204890215125E-5</v>
       </c>
       <c r="K25" s="14">
         <v>0</v>
       </c>
       <c r="L25" s="14">
-        <v>360758.09944459156</v>
+        <v>5613116.2027397258</v>
       </c>
       <c r="M25" s="13"/>
       <c r="N25" s="13"/>
@@ -2956,7 +2956,7 @@
         <v>0</v>
       </c>
       <c r="R25" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S25" s="24">
         <v>0</v>
@@ -3005,7 +3005,7 @@
         <v>1</v>
       </c>
       <c r="G26" s="22">
-        <v>34688.278792749188</v>
+        <v>26170.2579452055</v>
       </c>
       <c r="H26" s="13">
         <v>0</v>
@@ -3014,13 +3014,13 @@
         <v>0</v>
       </c>
       <c r="J26" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>5.7316974220913486E-4</v>
       </c>
       <c r="K26" s="14">
         <v>0</v>
       </c>
       <c r="L26" s="14">
-        <v>416259.34551299026</v>
+        <v>314043.09534246603</v>
       </c>
       <c r="M26" s="13"/>
       <c r="N26" s="13"/>
@@ -3034,7 +3034,7 @@
         <v>1</v>
       </c>
       <c r="R26" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S26" s="24">
         <v>0</v>
@@ -3083,7 +3083,7 @@
         <v>1</v>
       </c>
       <c r="G27" s="22">
-        <v>131944.51443052923</v>
+        <v>391003.39726027398</v>
       </c>
       <c r="H27" s="13">
         <v>0</v>
@@ -3092,13 +3092,13 @@
         <v>0</v>
       </c>
       <c r="J27" s="22">
-        <v>9.8526263529088916E-5</v>
+        <v>3.324779296315542E-5</v>
       </c>
       <c r="K27" s="14">
         <v>0</v>
       </c>
       <c r="L27" s="14">
-        <v>1583334.1731663509</v>
+        <v>4692040.7671232875</v>
       </c>
       <c r="M27" s="13"/>
       <c r="N27" s="13"/>
@@ -3112,7 +3112,7 @@
         <v>0</v>
       </c>
       <c r="R27" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S27" s="24">
         <v>0</v>
@@ -3163,7 +3163,7 @@
         <v>1</v>
       </c>
       <c r="G28" s="22">
-        <v>60126.349907431926</v>
+        <v>45642.158033868822</v>
       </c>
       <c r="H28" s="13">
         <v>0</v>
@@ -3172,13 +3172,13 @@
         <v>0</v>
       </c>
       <c r="J28" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K28" s="14">
         <v>0</v>
       </c>
       <c r="L28" s="14">
-        <v>721516.19888918311</v>
+        <v>547705.89640642586</v>
       </c>
       <c r="M28" s="13"/>
       <c r="N28" s="13"/>
@@ -3192,7 +3192,7 @@
         <v>0</v>
       </c>
       <c r="R28" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S28" s="24">
         <v>0</v>
@@ -3243,7 +3243,7 @@
         <v>1</v>
       </c>
       <c r="G29" s="22">
-        <v>4625.1038390332251</v>
+        <v>3510.9352333745246</v>
       </c>
       <c r="H29" s="13">
         <v>0</v>
@@ -3252,13 +3252,13 @@
         <v>0</v>
       </c>
       <c r="J29" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K29" s="14">
         <v>0</v>
       </c>
       <c r="L29" s="14">
-        <v>55501.246068398701</v>
+        <v>42131.222800494295</v>
       </c>
       <c r="M29" s="13"/>
       <c r="N29" s="13"/>
@@ -3272,7 +3272,7 @@
         <v>0</v>
       </c>
       <c r="R29" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S29" s="24">
         <v>0</v>
@@ -3321,7 +3321,7 @@
         <v>1</v>
       </c>
       <c r="G30" s="22">
-        <v>179073.80465116279</v>
+        <v>391003.39726027398</v>
       </c>
       <c r="H30" s="13">
         <v>0</v>
@@ -3330,13 +3330,13 @@
         <v>0</v>
       </c>
       <c r="J30" s="22">
-        <v>7.8180055576928815E-5</v>
+        <v>3.5805315498782759E-5</v>
       </c>
       <c r="K30" s="14">
         <v>0</v>
       </c>
       <c r="L30" s="14">
-        <v>2148885.6558139534</v>
+        <v>4692040.7671232875</v>
       </c>
       <c r="M30" s="13"/>
       <c r="N30" s="13"/>
@@ -3350,7 +3350,7 @@
         <v>0</v>
       </c>
       <c r="R30" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S30" s="24">
         <v>0</v>
@@ -3399,7 +3399,7 @@
         <v>1</v>
       </c>
       <c r="G31" s="22">
-        <v>2312.5519195166125</v>
+        <v>1755.4676166872623</v>
       </c>
       <c r="H31" s="13">
         <v>0</v>
@@ -3408,13 +3408,13 @@
         <v>0</v>
       </c>
       <c r="J31" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K31" s="14">
         <v>0</v>
       </c>
       <c r="L31" s="14">
-        <v>27750.623034199351</v>
+        <v>21065.611400247148</v>
       </c>
       <c r="M31" s="13"/>
       <c r="N31" s="13"/>
@@ -3428,7 +3428,7 @@
         <v>0</v>
       </c>
       <c r="R31" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S31" s="24">
         <v>0</v>
@@ -3477,7 +3477,7 @@
         <v>1</v>
       </c>
       <c r="G32" s="22">
-        <v>204734.74925373134</v>
+        <v>558256.28219178075</v>
       </c>
       <c r="H32" s="13">
         <v>0</v>
@@ -3486,13 +3486,13 @@
         <v>0</v>
       </c>
       <c r="J32" s="22">
-        <v>6.3496793032866511E-5</v>
+        <v>2.3286795714972428E-5</v>
       </c>
       <c r="K32" s="14">
         <v>0</v>
       </c>
       <c r="L32" s="14">
-        <v>2456816.991044776</v>
+        <v>6699075.3863013685</v>
       </c>
       <c r="M32" s="13"/>
       <c r="N32" s="13"/>
@@ -3506,7 +3506,7 @@
         <v>0</v>
       </c>
       <c r="R32" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S32" s="24">
         <v>0</v>
@@ -3557,7 +3557,7 @@
         <v>1</v>
       </c>
       <c r="G33" s="22">
-        <v>37022.94</v>
+        <v>90723.599999999991</v>
       </c>
       <c r="H33" s="13">
         <v>0</v>
@@ -3566,13 +3566,13 @@
         <v>0</v>
       </c>
       <c r="J33" s="22">
-        <v>1.6206168391813292E-4</v>
+        <v>6.6134941735116335E-5</v>
       </c>
       <c r="K33" s="14">
         <v>0</v>
       </c>
       <c r="L33" s="14">
-        <v>444275.28</v>
+        <v>1088683.2</v>
       </c>
       <c r="M33" s="13"/>
       <c r="N33" s="13"/>
@@ -3586,7 +3586,7 @@
         <v>0</v>
       </c>
       <c r="R33" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S33" s="24">
         <v>0</v>
@@ -3637,7 +3637,7 @@
         <v>1</v>
       </c>
       <c r="G34" s="22">
-        <v>37000.830712265801</v>
+        <v>26170.257945205503</v>
       </c>
       <c r="H34" s="13">
         <v>0</v>
@@ -3646,13 +3646,13 @@
         <v>0</v>
       </c>
       <c r="J34" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>6.1138105835641045E-4</v>
       </c>
       <c r="K34" s="14">
         <v>0</v>
       </c>
       <c r="L34" s="14">
-        <v>444009.96854718961</v>
+        <v>314043.09534246603</v>
       </c>
       <c r="M34" s="13"/>
       <c r="N34" s="13"/>
@@ -3666,7 +3666,7 @@
         <v>0</v>
       </c>
       <c r="R34" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S34" s="24">
         <v>0</v>
@@ -3715,7 +3715,7 @@
         <v>1</v>
       </c>
       <c r="G35" s="22">
-        <v>27750.623034199351</v>
+        <v>21065.611400247148</v>
       </c>
       <c r="H35" s="13">
         <v>0</v>
@@ -3724,13 +3724,13 @@
         <v>0</v>
       </c>
       <c r="J35" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K35" s="14">
         <v>0</v>
       </c>
       <c r="L35" s="14">
-        <v>333007.47641039221</v>
+        <v>252787.33680296579</v>
       </c>
       <c r="M35" s="13"/>
       <c r="N35" s="13"/>
@@ -3744,7 +3744,7 @@
         <v>0</v>
       </c>
       <c r="R35" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S35" s="24">
         <v>0</v>
@@ -3793,7 +3793,7 @@
         <v>1</v>
       </c>
       <c r="G36" s="22">
-        <v>2312.5519195166125</v>
+        <v>26170.257945205503</v>
       </c>
       <c r="H36" s="13">
         <v>0</v>
@@ -3802,13 +3802,13 @@
         <v>0</v>
       </c>
       <c r="J36" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>3.8211316147275653E-5</v>
       </c>
       <c r="K36" s="14">
         <v>0</v>
       </c>
       <c r="L36" s="14">
-        <v>27750.623034199351</v>
+        <v>314043.09534246603</v>
       </c>
       <c r="M36" s="13"/>
       <c r="N36" s="13"/>
@@ -3822,7 +3822,7 @@
         <v>0</v>
       </c>
       <c r="R36" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S36" s="24">
         <v>0</v>
@@ -3871,7 +3871,7 @@
         <v>1</v>
       </c>
       <c r="G37" s="22">
-        <v>2312.5519195166125</v>
+        <v>1755.4676166872623</v>
       </c>
       <c r="H37" s="13">
         <v>0</v>
@@ -3880,13 +3880,13 @@
         <v>0</v>
       </c>
       <c r="J37" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K37" s="14">
         <v>0</v>
       </c>
       <c r="L37" s="14">
-        <v>27750.623034199351</v>
+        <v>21065.611400247148</v>
       </c>
       <c r="M37" s="13"/>
       <c r="N37" s="13"/>
@@ -3900,7 +3900,7 @@
         <v>0</v>
       </c>
       <c r="R37" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S37" s="24">
         <v>0</v>
@@ -3949,7 +3949,7 @@
         <v>1</v>
       </c>
       <c r="G38" s="22">
-        <v>39313.382631782413</v>
+        <v>29842.94948368346</v>
       </c>
       <c r="H38" s="13">
         <v>0</v>
@@ -3958,13 +3958,13 @@
         <v>0</v>
       </c>
       <c r="J38" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K38" s="14">
         <v>0</v>
       </c>
       <c r="L38" s="14">
-        <v>471760.59158138896</v>
+        <v>358115.39380420151</v>
       </c>
       <c r="M38" s="13"/>
       <c r="N38" s="13"/>
@@ -3978,7 +3978,7 @@
         <v>0</v>
       </c>
       <c r="R38" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S38" s="24">
         <v>0</v>
@@ -4029,7 +4029,7 @@
         <v>1</v>
       </c>
       <c r="G39" s="22">
-        <v>2312.5519195166125</v>
+        <v>1755.4676166872623</v>
       </c>
       <c r="H39" s="13">
         <v>0</v>
@@ -4038,13 +4038,13 @@
         <v>0</v>
       </c>
       <c r="J39" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K39" s="14">
         <v>0</v>
       </c>
       <c r="L39" s="14">
-        <v>27750.623034199351</v>
+        <v>21065.611400247148</v>
       </c>
       <c r="M39" s="13"/>
       <c r="N39" s="13"/>
@@ -4058,7 +4058,7 @@
         <v>0</v>
       </c>
       <c r="R39" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S39" s="24">
         <v>0</v>
@@ -4107,7 +4107,7 @@
         <v>1</v>
       </c>
       <c r="G40" s="22">
-        <v>11331.504405631402</v>
+        <v>8601.791321767585</v>
       </c>
       <c r="H40" s="13">
         <v>0</v>
@@ -4116,13 +4116,13 @@
         <v>0</v>
       </c>
       <c r="J40" s="22">
-        <v>4.3242272381457611E-4</v>
+        <v>5.6964878787516286E-4</v>
       </c>
       <c r="K40" s="14">
         <v>0</v>
       </c>
       <c r="L40" s="14">
-        <v>135978.05286757683</v>
+        <v>103221.49586121102</v>
       </c>
       <c r="M40" s="13"/>
       <c r="N40" s="13"/>
@@ -4136,7 +4136,7 @@
         <v>0</v>
       </c>
       <c r="R40" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S40" s="24">
         <v>0</v>
@@ -4187,7 +4187,7 @@
         <v>1</v>
       </c>
       <c r="G41" s="22">
-        <v>9898.1018181818181</v>
+        <v>14914.142876712329</v>
       </c>
       <c r="H41" s="13">
         <v>0</v>
@@ -4196,13 +4196,13 @@
         <v>0</v>
       </c>
       <c r="J41" s="22">
-        <v>1.010294719501774E-3</v>
+        <v>6.7050450586835192E-4</v>
       </c>
       <c r="K41" s="14">
         <v>0</v>
       </c>
       <c r="L41" s="14">
-        <v>118777.22181818182</v>
+        <v>178969.71452054795</v>
       </c>
       <c r="M41" s="13"/>
       <c r="N41" s="13"/>
@@ -4216,7 +4216,7 @@
         <v>0</v>
       </c>
       <c r="R41" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S41" s="24">
         <v>0</v>
@@ -4267,7 +4267,7 @@
         <v>1</v>
       </c>
       <c r="G42" s="22">
-        <v>355388.97599999997</v>
+        <v>26170.2579452055</v>
       </c>
       <c r="H42" s="13">
         <v>0</v>
@@ -4276,13 +4276,13 @@
         <v>0</v>
       </c>
       <c r="J42" s="22">
-        <v>8.4414548638109697E-5</v>
+        <v>1.1463394844182697E-3</v>
       </c>
       <c r="K42" s="14">
         <v>0</v>
       </c>
       <c r="L42" s="14">
-        <v>4264667.7119999994</v>
+        <v>314043.09534246603</v>
       </c>
       <c r="M42" s="13"/>
       <c r="N42" s="13"/>
@@ -4296,7 +4296,7 @@
         <v>0</v>
       </c>
       <c r="R42" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S42" s="24">
         <v>0</v>
@@ -4347,7 +4347,7 @@
         <v>1</v>
       </c>
       <c r="G43" s="22">
-        <v>180286.82497297297</v>
+        <v>388412.26027397264</v>
       </c>
       <c r="H43" s="13">
         <v>0</v>
@@ -4356,13 +4356,13 @@
         <v>0</v>
       </c>
       <c r="J43" s="22">
-        <v>9.4294189287256525E-5</v>
+        <v>4.37679284068139E-5</v>
       </c>
       <c r="K43" s="14">
         <v>0</v>
       </c>
       <c r="L43" s="14">
-        <v>2163441.8996756757</v>
+        <v>4660947.1232876722</v>
       </c>
       <c r="M43" s="13"/>
       <c r="N43" s="13"/>
@@ -4376,7 +4376,7 @@
         <v>0</v>
       </c>
       <c r="R43" s="22">
-        <v>4.6657547496963339E-4</v>
+        <v>3.1109458176473712E-4</v>
       </c>
       <c r="S43" s="24">
         <v>0</v>

</xml_diff>